<commit_message>
Add Google Sheets data layer (DATA_BACKEND=sheets) with append-only writes; sales total moved to last column; remove unused helper
</commit_message>
<xml_diff>
--- a/data/Ayyappa_Pooja_Store_Data.xlsx
+++ b/data/Ayyappa_Pooja_Store_Data.xlsx
@@ -12549,9 +12549,9 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12597,3028 +12597,3028 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Customer_Name</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Customer_Phone</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="I2">
+      <c r="L2">
         <f>IF(A2="","",F2*G2)</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="I3">
+      <c r="L3">
         <f>IF(A3="","",F3*G3)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="I4">
+      <c r="L4">
         <f>IF(A4="","",F4*G4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="I5">
+      <c r="L5">
         <f>IF(A5="","",F5*G5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="I6">
+      <c r="L6">
         <f>IF(A6="","",F6*G6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="I7">
+      <c r="L7">
         <f>IF(A7="","",F7*G7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="I8">
+      <c r="L8">
         <f>IF(A8="","",F8*G8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="I9">
+      <c r="L9">
         <f>IF(A9="","",F9*G9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="I10">
+      <c r="L10">
         <f>IF(A10="","",F10*G10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="I11">
+      <c r="L11">
         <f>IF(A11="","",F11*G11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="I12">
+      <c r="L12">
         <f>IF(A12="","",F12*G12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="I13">
+      <c r="L13">
         <f>IF(A13="","",F13*G13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="I14">
+      <c r="L14">
         <f>IF(A14="","",F14*G14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="I15">
+      <c r="L15">
         <f>IF(A15="","",F15*G15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="I16">
+      <c r="L16">
         <f>IF(A16="","",F16*G16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="I17">
+      <c r="L17">
         <f>IF(A17="","",F17*G17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="I18">
+      <c r="L18">
         <f>IF(A18="","",F18*G18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="I19">
+      <c r="L19">
         <f>IF(A19="","",F19*G19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="I20">
+      <c r="L20">
         <f>IF(A20="","",F20*G20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="I21">
+      <c r="L21">
         <f>IF(A21="","",F21*G21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="I22">
+      <c r="L22">
         <f>IF(A22="","",F22*G22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="I23">
+      <c r="L23">
         <f>IF(A23="","",F23*G23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="I24">
+      <c r="L24">
         <f>IF(A24="","",F24*G24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="I25">
+      <c r="L25">
         <f>IF(A25="","",F25*G25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="I26">
+      <c r="L26">
         <f>IF(A26="","",F26*G26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="I27">
+      <c r="L27">
         <f>IF(A27="","",F27*G27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="I28">
+      <c r="L28">
         <f>IF(A28="","",F28*G28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="I29">
+      <c r="L29">
         <f>IF(A29="","",F29*G29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="I30">
+      <c r="L30">
         <f>IF(A30="","",F30*G30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="I31">
+      <c r="L31">
         <f>IF(A31="","",F31*G31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="I32">
+      <c r="L32">
         <f>IF(A32="","",F32*G32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="I33">
+      <c r="L33">
         <f>IF(A33="","",F33*G33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="I34">
+      <c r="L34">
         <f>IF(A34="","",F34*G34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="I35">
+      <c r="L35">
         <f>IF(A35="","",F35*G35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="I36">
+      <c r="L36">
         <f>IF(A36="","",F36*G36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="I37">
+      <c r="L37">
         <f>IF(A37="","",F37*G37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="I38">
+      <c r="L38">
         <f>IF(A38="","",F38*G38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="I39">
+      <c r="L39">
         <f>IF(A39="","",F39*G39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="I40">
+      <c r="L40">
         <f>IF(A40="","",F40*G40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="I41">
+      <c r="L41">
         <f>IF(A41="","",F41*G41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="I42">
+      <c r="L42">
         <f>IF(A42="","",F42*G42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="I43">
+      <c r="L43">
         <f>IF(A43="","",F43*G43)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="I44">
+      <c r="L44">
         <f>IF(A44="","",F44*G44)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="I45">
+      <c r="L45">
         <f>IF(A45="","",F45*G45)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="I46">
+      <c r="L46">
         <f>IF(A46="","",F46*G46)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="I47">
+      <c r="L47">
         <f>IF(A47="","",F47*G47)</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="I48">
+      <c r="L48">
         <f>IF(A48="","",F48*G48)</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="I49">
+      <c r="L49">
         <f>IF(A49="","",F49*G49)</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="I50">
+      <c r="L50">
         <f>IF(A50="","",F50*G50)</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="I51">
+      <c r="L51">
         <f>IF(A51="","",F51*G51)</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="I52">
+      <c r="L52">
         <f>IF(A52="","",F52*G52)</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="I53">
+      <c r="L53">
         <f>IF(A53="","",F53*G53)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="I54">
+      <c r="L54">
         <f>IF(A54="","",F54*G54)</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="I55">
+      <c r="L55">
         <f>IF(A55="","",F55*G55)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="I56">
+      <c r="L56">
         <f>IF(A56="","",F56*G56)</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="I57">
+      <c r="L57">
         <f>IF(A57="","",F57*G57)</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="I58">
+      <c r="L58">
         <f>IF(A58="","",F58*G58)</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="I59">
+      <c r="L59">
         <f>IF(A59="","",F59*G59)</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="I60">
+      <c r="L60">
         <f>IF(A60="","",F60*G60)</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="I61">
+      <c r="L61">
         <f>IF(A61="","",F61*G61)</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="I62">
+      <c r="L62">
         <f>IF(A62="","",F62*G62)</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="I63">
+      <c r="L63">
         <f>IF(A63="","",F63*G63)</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="I64">
+      <c r="L64">
         <f>IF(A64="","",F64*G64)</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="I65">
+      <c r="L65">
         <f>IF(A65="","",F65*G65)</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="I66">
+      <c r="L66">
         <f>IF(A66="","",F66*G66)</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="I67">
+      <c r="L67">
         <f>IF(A67="","",F67*G67)</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="I68">
+      <c r="L68">
         <f>IF(A68="","",F68*G68)</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="I69">
+      <c r="L69">
         <f>IF(A69="","",F69*G69)</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="I70">
+      <c r="L70">
         <f>IF(A70="","",F70*G70)</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="I71">
+      <c r="L71">
         <f>IF(A71="","",F71*G71)</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="I72">
+      <c r="L72">
         <f>IF(A72="","",F72*G72)</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="I73">
+      <c r="L73">
         <f>IF(A73="","",F73*G73)</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="I74">
+      <c r="L74">
         <f>IF(A74="","",F74*G74)</f>
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="I75">
+      <c r="L75">
         <f>IF(A75="","",F75*G75)</f>
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="I76">
+      <c r="L76">
         <f>IF(A76="","",F76*G76)</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="I77">
+      <c r="L77">
         <f>IF(A77="","",F77*G77)</f>
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="I78">
+      <c r="L78">
         <f>IF(A78="","",F78*G78)</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="I79">
+      <c r="L79">
         <f>IF(A79="","",F79*G79)</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="I80">
+      <c r="L80">
         <f>IF(A80="","",F80*G80)</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="I81">
+      <c r="L81">
         <f>IF(A81="","",F81*G81)</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="I82">
+      <c r="L82">
         <f>IF(A82="","",F82*G82)</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="I83">
+      <c r="L83">
         <f>IF(A83="","",F83*G83)</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="I84">
+      <c r="L84">
         <f>IF(A84="","",F84*G84)</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="I85">
+      <c r="L85">
         <f>IF(A85="","",F85*G85)</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="I86">
+      <c r="L86">
         <f>IF(A86="","",F86*G86)</f>
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="I87">
+      <c r="L87">
         <f>IF(A87="","",F87*G87)</f>
         <v/>
       </c>
     </row>
     <row r="88">
-      <c r="I88">
+      <c r="L88">
         <f>IF(A88="","",F88*G88)</f>
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="I89">
+      <c r="L89">
         <f>IF(A89="","",F89*G89)</f>
         <v/>
       </c>
     </row>
     <row r="90">
-      <c r="I90">
+      <c r="L90">
         <f>IF(A90="","",F90*G90)</f>
         <v/>
       </c>
     </row>
     <row r="91">
-      <c r="I91">
+      <c r="L91">
         <f>IF(A91="","",F91*G91)</f>
         <v/>
       </c>
     </row>
     <row r="92">
-      <c r="I92">
+      <c r="L92">
         <f>IF(A92="","",F92*G92)</f>
         <v/>
       </c>
     </row>
     <row r="93">
-      <c r="I93">
+      <c r="L93">
         <f>IF(A93="","",F93*G93)</f>
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="I94">
+      <c r="L94">
         <f>IF(A94="","",F94*G94)</f>
         <v/>
       </c>
     </row>
     <row r="95">
-      <c r="I95">
+      <c r="L95">
         <f>IF(A95="","",F95*G95)</f>
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="I96">
+      <c r="L96">
         <f>IF(A96="","",F96*G96)</f>
         <v/>
       </c>
     </row>
     <row r="97">
-      <c r="I97">
+      <c r="L97">
         <f>IF(A97="","",F97*G97)</f>
         <v/>
       </c>
     </row>
     <row r="98">
-      <c r="I98">
+      <c r="L98">
         <f>IF(A98="","",F98*G98)</f>
         <v/>
       </c>
     </row>
     <row r="99">
-      <c r="I99">
+      <c r="L99">
         <f>IF(A99="","",F99*G99)</f>
         <v/>
       </c>
     </row>
     <row r="100">
-      <c r="I100">
+      <c r="L100">
         <f>IF(A100="","",F100*G100)</f>
         <v/>
       </c>
     </row>
     <row r="101">
-      <c r="I101">
+      <c r="L101">
         <f>IF(A101="","",F101*G101)</f>
         <v/>
       </c>
     </row>
     <row r="102">
-      <c r="I102">
+      <c r="L102">
         <f>IF(A102="","",F102*G102)</f>
         <v/>
       </c>
     </row>
     <row r="103">
-      <c r="I103">
+      <c r="L103">
         <f>IF(A103="","",F103*G103)</f>
         <v/>
       </c>
     </row>
     <row r="104">
-      <c r="I104">
+      <c r="L104">
         <f>IF(A104="","",F104*G104)</f>
         <v/>
       </c>
     </row>
     <row r="105">
-      <c r="I105">
+      <c r="L105">
         <f>IF(A105="","",F105*G105)</f>
         <v/>
       </c>
     </row>
     <row r="106">
-      <c r="I106">
+      <c r="L106">
         <f>IF(A106="","",F106*G106)</f>
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="I107">
+      <c r="L107">
         <f>IF(A107="","",F107*G107)</f>
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="I108">
+      <c r="L108">
         <f>IF(A108="","",F108*G108)</f>
         <v/>
       </c>
     </row>
     <row r="109">
-      <c r="I109">
+      <c r="L109">
         <f>IF(A109="","",F109*G109)</f>
         <v/>
       </c>
     </row>
     <row r="110">
-      <c r="I110">
+      <c r="L110">
         <f>IF(A110="","",F110*G110)</f>
         <v/>
       </c>
     </row>
     <row r="111">
-      <c r="I111">
+      <c r="L111">
         <f>IF(A111="","",F111*G111)</f>
         <v/>
       </c>
     </row>
     <row r="112">
-      <c r="I112">
+      <c r="L112">
         <f>IF(A112="","",F112*G112)</f>
         <v/>
       </c>
     </row>
     <row r="113">
-      <c r="I113">
+      <c r="L113">
         <f>IF(A113="","",F113*G113)</f>
         <v/>
       </c>
     </row>
     <row r="114">
-      <c r="I114">
+      <c r="L114">
         <f>IF(A114="","",F114*G114)</f>
         <v/>
       </c>
     </row>
     <row r="115">
-      <c r="I115">
+      <c r="L115">
         <f>IF(A115="","",F115*G115)</f>
         <v/>
       </c>
     </row>
     <row r="116">
-      <c r="I116">
+      <c r="L116">
         <f>IF(A116="","",F116*G116)</f>
         <v/>
       </c>
     </row>
     <row r="117">
-      <c r="I117">
+      <c r="L117">
         <f>IF(A117="","",F117*G117)</f>
         <v/>
       </c>
     </row>
     <row r="118">
-      <c r="I118">
+      <c r="L118">
         <f>IF(A118="","",F118*G118)</f>
         <v/>
       </c>
     </row>
     <row r="119">
-      <c r="I119">
+      <c r="L119">
         <f>IF(A119="","",F119*G119)</f>
         <v/>
       </c>
     </row>
     <row r="120">
-      <c r="I120">
+      <c r="L120">
         <f>IF(A120="","",F120*G120)</f>
         <v/>
       </c>
     </row>
     <row r="121">
-      <c r="I121">
+      <c r="L121">
         <f>IF(A121="","",F121*G121)</f>
         <v/>
       </c>
     </row>
     <row r="122">
-      <c r="I122">
+      <c r="L122">
         <f>IF(A122="","",F122*G122)</f>
         <v/>
       </c>
     </row>
     <row r="123">
-      <c r="I123">
+      <c r="L123">
         <f>IF(A123="","",F123*G123)</f>
         <v/>
       </c>
     </row>
     <row r="124">
-      <c r="I124">
+      <c r="L124">
         <f>IF(A124="","",F124*G124)</f>
         <v/>
       </c>
     </row>
     <row r="125">
-      <c r="I125">
+      <c r="L125">
         <f>IF(A125="","",F125*G125)</f>
         <v/>
       </c>
     </row>
     <row r="126">
-      <c r="I126">
+      <c r="L126">
         <f>IF(A126="","",F126*G126)</f>
         <v/>
       </c>
     </row>
     <row r="127">
-      <c r="I127">
+      <c r="L127">
         <f>IF(A127="","",F127*G127)</f>
         <v/>
       </c>
     </row>
     <row r="128">
-      <c r="I128">
+      <c r="L128">
         <f>IF(A128="","",F128*G128)</f>
         <v/>
       </c>
     </row>
     <row r="129">
-      <c r="I129">
+      <c r="L129">
         <f>IF(A129="","",F129*G129)</f>
         <v/>
       </c>
     </row>
     <row r="130">
-      <c r="I130">
+      <c r="L130">
         <f>IF(A130="","",F130*G130)</f>
         <v/>
       </c>
     </row>
     <row r="131">
-      <c r="I131">
+      <c r="L131">
         <f>IF(A131="","",F131*G131)</f>
         <v/>
       </c>
     </row>
     <row r="132">
-      <c r="I132">
+      <c r="L132">
         <f>IF(A132="","",F132*G132)</f>
         <v/>
       </c>
     </row>
     <row r="133">
-      <c r="I133">
+      <c r="L133">
         <f>IF(A133="","",F133*G133)</f>
         <v/>
       </c>
     </row>
     <row r="134">
-      <c r="I134">
+      <c r="L134">
         <f>IF(A134="","",F134*G134)</f>
         <v/>
       </c>
     </row>
     <row r="135">
-      <c r="I135">
+      <c r="L135">
         <f>IF(A135="","",F135*G135)</f>
         <v/>
       </c>
     </row>
     <row r="136">
-      <c r="I136">
+      <c r="L136">
         <f>IF(A136="","",F136*G136)</f>
         <v/>
       </c>
     </row>
     <row r="137">
-      <c r="I137">
+      <c r="L137">
         <f>IF(A137="","",F137*G137)</f>
         <v/>
       </c>
     </row>
     <row r="138">
-      <c r="I138">
+      <c r="L138">
         <f>IF(A138="","",F138*G138)</f>
         <v/>
       </c>
     </row>
     <row r="139">
-      <c r="I139">
+      <c r="L139">
         <f>IF(A139="","",F139*G139)</f>
         <v/>
       </c>
     </row>
     <row r="140">
-      <c r="I140">
+      <c r="L140">
         <f>IF(A140="","",F140*G140)</f>
         <v/>
       </c>
     </row>
     <row r="141">
-      <c r="I141">
+      <c r="L141">
         <f>IF(A141="","",F141*G141)</f>
         <v/>
       </c>
     </row>
     <row r="142">
-      <c r="I142">
+      <c r="L142">
         <f>IF(A142="","",F142*G142)</f>
         <v/>
       </c>
     </row>
     <row r="143">
-      <c r="I143">
+      <c r="L143">
         <f>IF(A143="","",F143*G143)</f>
         <v/>
       </c>
     </row>
     <row r="144">
-      <c r="I144">
+      <c r="L144">
         <f>IF(A144="","",F144*G144)</f>
         <v/>
       </c>
     </row>
     <row r="145">
-      <c r="I145">
+      <c r="L145">
         <f>IF(A145="","",F145*G145)</f>
         <v/>
       </c>
     </row>
     <row r="146">
-      <c r="I146">
+      <c r="L146">
         <f>IF(A146="","",F146*G146)</f>
         <v/>
       </c>
     </row>
     <row r="147">
-      <c r="I147">
+      <c r="L147">
         <f>IF(A147="","",F147*G147)</f>
         <v/>
       </c>
     </row>
     <row r="148">
-      <c r="I148">
+      <c r="L148">
         <f>IF(A148="","",F148*G148)</f>
         <v/>
       </c>
     </row>
     <row r="149">
-      <c r="I149">
+      <c r="L149">
         <f>IF(A149="","",F149*G149)</f>
         <v/>
       </c>
     </row>
     <row r="150">
-      <c r="I150">
+      <c r="L150">
         <f>IF(A150="","",F150*G150)</f>
         <v/>
       </c>
     </row>
     <row r="151">
-      <c r="I151">
+      <c r="L151">
         <f>IF(A151="","",F151*G151)</f>
         <v/>
       </c>
     </row>
     <row r="152">
-      <c r="I152">
+      <c r="L152">
         <f>IF(A152="","",F152*G152)</f>
         <v/>
       </c>
     </row>
     <row r="153">
-      <c r="I153">
+      <c r="L153">
         <f>IF(A153="","",F153*G153)</f>
         <v/>
       </c>
     </row>
     <row r="154">
-      <c r="I154">
+      <c r="L154">
         <f>IF(A154="","",F154*G154)</f>
         <v/>
       </c>
     </row>
     <row r="155">
-      <c r="I155">
+      <c r="L155">
         <f>IF(A155="","",F155*G155)</f>
         <v/>
       </c>
     </row>
     <row r="156">
-      <c r="I156">
+      <c r="L156">
         <f>IF(A156="","",F156*G156)</f>
         <v/>
       </c>
     </row>
     <row r="157">
-      <c r="I157">
+      <c r="L157">
         <f>IF(A157="","",F157*G157)</f>
         <v/>
       </c>
     </row>
     <row r="158">
-      <c r="I158">
+      <c r="L158">
         <f>IF(A158="","",F158*G158)</f>
         <v/>
       </c>
     </row>
     <row r="159">
-      <c r="I159">
+      <c r="L159">
         <f>IF(A159="","",F159*G159)</f>
         <v/>
       </c>
     </row>
     <row r="160">
-      <c r="I160">
+      <c r="L160">
         <f>IF(A160="","",F160*G160)</f>
         <v/>
       </c>
     </row>
     <row r="161">
-      <c r="I161">
+      <c r="L161">
         <f>IF(A161="","",F161*G161)</f>
         <v/>
       </c>
     </row>
     <row r="162">
-      <c r="I162">
+      <c r="L162">
         <f>IF(A162="","",F162*G162)</f>
         <v/>
       </c>
     </row>
     <row r="163">
-      <c r="I163">
+      <c r="L163">
         <f>IF(A163="","",F163*G163)</f>
         <v/>
       </c>
     </row>
     <row r="164">
-      <c r="I164">
+      <c r="L164">
         <f>IF(A164="","",F164*G164)</f>
         <v/>
       </c>
     </row>
     <row r="165">
-      <c r="I165">
+      <c r="L165">
         <f>IF(A165="","",F165*G165)</f>
         <v/>
       </c>
     </row>
     <row r="166">
-      <c r="I166">
+      <c r="L166">
         <f>IF(A166="","",F166*G166)</f>
         <v/>
       </c>
     </row>
     <row r="167">
-      <c r="I167">
+      <c r="L167">
         <f>IF(A167="","",F167*G167)</f>
         <v/>
       </c>
     </row>
     <row r="168">
-      <c r="I168">
+      <c r="L168">
         <f>IF(A168="","",F168*G168)</f>
         <v/>
       </c>
     </row>
     <row r="169">
-      <c r="I169">
+      <c r="L169">
         <f>IF(A169="","",F169*G169)</f>
         <v/>
       </c>
     </row>
     <row r="170">
-      <c r="I170">
+      <c r="L170">
         <f>IF(A170="","",F170*G170)</f>
         <v/>
       </c>
     </row>
     <row r="171">
-      <c r="I171">
+      <c r="L171">
         <f>IF(A171="","",F171*G171)</f>
         <v/>
       </c>
     </row>
     <row r="172">
-      <c r="I172">
+      <c r="L172">
         <f>IF(A172="","",F172*G172)</f>
         <v/>
       </c>
     </row>
     <row r="173">
-      <c r="I173">
+      <c r="L173">
         <f>IF(A173="","",F173*G173)</f>
         <v/>
       </c>
     </row>
     <row r="174">
-      <c r="I174">
+      <c r="L174">
         <f>IF(A174="","",F174*G174)</f>
         <v/>
       </c>
     </row>
     <row r="175">
-      <c r="I175">
+      <c r="L175">
         <f>IF(A175="","",F175*G175)</f>
         <v/>
       </c>
     </row>
     <row r="176">
-      <c r="I176">
+      <c r="L176">
         <f>IF(A176="","",F176*G176)</f>
         <v/>
       </c>
     </row>
     <row r="177">
-      <c r="I177">
+      <c r="L177">
         <f>IF(A177="","",F177*G177)</f>
         <v/>
       </c>
     </row>
     <row r="178">
-      <c r="I178">
+      <c r="L178">
         <f>IF(A178="","",F178*G178)</f>
         <v/>
       </c>
     </row>
     <row r="179">
-      <c r="I179">
+      <c r="L179">
         <f>IF(A179="","",F179*G179)</f>
         <v/>
       </c>
     </row>
     <row r="180">
-      <c r="I180">
+      <c r="L180">
         <f>IF(A180="","",F180*G180)</f>
         <v/>
       </c>
     </row>
     <row r="181">
-      <c r="I181">
+      <c r="L181">
         <f>IF(A181="","",F181*G181)</f>
         <v/>
       </c>
     </row>
     <row r="182">
-      <c r="I182">
+      <c r="L182">
         <f>IF(A182="","",F182*G182)</f>
         <v/>
       </c>
     </row>
     <row r="183">
-      <c r="I183">
+      <c r="L183">
         <f>IF(A183="","",F183*G183)</f>
         <v/>
       </c>
     </row>
     <row r="184">
-      <c r="I184">
+      <c r="L184">
         <f>IF(A184="","",F184*G184)</f>
         <v/>
       </c>
     </row>
     <row r="185">
-      <c r="I185">
+      <c r="L185">
         <f>IF(A185="","",F185*G185)</f>
         <v/>
       </c>
     </row>
     <row r="186">
-      <c r="I186">
+      <c r="L186">
         <f>IF(A186="","",F186*G186)</f>
         <v/>
       </c>
     </row>
     <row r="187">
-      <c r="I187">
+      <c r="L187">
         <f>IF(A187="","",F187*G187)</f>
         <v/>
       </c>
     </row>
     <row r="188">
-      <c r="I188">
+      <c r="L188">
         <f>IF(A188="","",F188*G188)</f>
         <v/>
       </c>
     </row>
     <row r="189">
-      <c r="I189">
+      <c r="L189">
         <f>IF(A189="","",F189*G189)</f>
         <v/>
       </c>
     </row>
     <row r="190">
-      <c r="I190">
+      <c r="L190">
         <f>IF(A190="","",F190*G190)</f>
         <v/>
       </c>
     </row>
     <row r="191">
-      <c r="I191">
+      <c r="L191">
         <f>IF(A191="","",F191*G191)</f>
         <v/>
       </c>
     </row>
     <row r="192">
-      <c r="I192">
+      <c r="L192">
         <f>IF(A192="","",F192*G192)</f>
         <v/>
       </c>
     </row>
     <row r="193">
-      <c r="I193">
+      <c r="L193">
         <f>IF(A193="","",F193*G193)</f>
         <v/>
       </c>
     </row>
     <row r="194">
-      <c r="I194">
+      <c r="L194">
         <f>IF(A194="","",F194*G194)</f>
         <v/>
       </c>
     </row>
     <row r="195">
-      <c r="I195">
+      <c r="L195">
         <f>IF(A195="","",F195*G195)</f>
         <v/>
       </c>
     </row>
     <row r="196">
-      <c r="I196">
+      <c r="L196">
         <f>IF(A196="","",F196*G196)</f>
         <v/>
       </c>
     </row>
     <row r="197">
-      <c r="I197">
+      <c r="L197">
         <f>IF(A197="","",F197*G197)</f>
         <v/>
       </c>
     </row>
     <row r="198">
-      <c r="I198">
+      <c r="L198">
         <f>IF(A198="","",F198*G198)</f>
         <v/>
       </c>
     </row>
     <row r="199">
-      <c r="I199">
+      <c r="L199">
         <f>IF(A199="","",F199*G199)</f>
         <v/>
       </c>
     </row>
     <row r="200">
-      <c r="I200">
+      <c r="L200">
         <f>IF(A200="","",F200*G200)</f>
         <v/>
       </c>
     </row>
     <row r="201">
-      <c r="I201">
+      <c r="L201">
         <f>IF(A201="","",F201*G201)</f>
         <v/>
       </c>
     </row>
     <row r="202">
-      <c r="I202">
+      <c r="L202">
         <f>IF(A202="","",F202*G202)</f>
         <v/>
       </c>
     </row>
     <row r="203">
-      <c r="I203">
+      <c r="L203">
         <f>IF(A203="","",F203*G203)</f>
         <v/>
       </c>
     </row>
     <row r="204">
-      <c r="I204">
+      <c r="L204">
         <f>IF(A204="","",F204*G204)</f>
         <v/>
       </c>
     </row>
     <row r="205">
-      <c r="I205">
+      <c r="L205">
         <f>IF(A205="","",F205*G205)</f>
         <v/>
       </c>
     </row>
     <row r="206">
-      <c r="I206">
+      <c r="L206">
         <f>IF(A206="","",F206*G206)</f>
         <v/>
       </c>
     </row>
     <row r="207">
-      <c r="I207">
+      <c r="L207">
         <f>IF(A207="","",F207*G207)</f>
         <v/>
       </c>
     </row>
     <row r="208">
-      <c r="I208">
+      <c r="L208">
         <f>IF(A208="","",F208*G208)</f>
         <v/>
       </c>
     </row>
     <row r="209">
-      <c r="I209">
+      <c r="L209">
         <f>IF(A209="","",F209*G209)</f>
         <v/>
       </c>
     </row>
     <row r="210">
-      <c r="I210">
+      <c r="L210">
         <f>IF(A210="","",F210*G210)</f>
         <v/>
       </c>
     </row>
     <row r="211">
-      <c r="I211">
+      <c r="L211">
         <f>IF(A211="","",F211*G211)</f>
         <v/>
       </c>
     </row>
     <row r="212">
-      <c r="I212">
+      <c r="L212">
         <f>IF(A212="","",F212*G212)</f>
         <v/>
       </c>
     </row>
     <row r="213">
-      <c r="I213">
+      <c r="L213">
         <f>IF(A213="","",F213*G213)</f>
         <v/>
       </c>
     </row>
     <row r="214">
-      <c r="I214">
+      <c r="L214">
         <f>IF(A214="","",F214*G214)</f>
         <v/>
       </c>
     </row>
     <row r="215">
-      <c r="I215">
+      <c r="L215">
         <f>IF(A215="","",F215*G215)</f>
         <v/>
       </c>
     </row>
     <row r="216">
-      <c r="I216">
+      <c r="L216">
         <f>IF(A216="","",F216*G216)</f>
         <v/>
       </c>
     </row>
     <row r="217">
-      <c r="I217">
+      <c r="L217">
         <f>IF(A217="","",F217*G217)</f>
         <v/>
       </c>
     </row>
     <row r="218">
-      <c r="I218">
+      <c r="L218">
         <f>IF(A218="","",F218*G218)</f>
         <v/>
       </c>
     </row>
     <row r="219">
-      <c r="I219">
+      <c r="L219">
         <f>IF(A219="","",F219*G219)</f>
         <v/>
       </c>
     </row>
     <row r="220">
-      <c r="I220">
+      <c r="L220">
         <f>IF(A220="","",F220*G220)</f>
         <v/>
       </c>
     </row>
     <row r="221">
-      <c r="I221">
+      <c r="L221">
         <f>IF(A221="","",F221*G221)</f>
         <v/>
       </c>
     </row>
     <row r="222">
-      <c r="I222">
+      <c r="L222">
         <f>IF(A222="","",F222*G222)</f>
         <v/>
       </c>
     </row>
     <row r="223">
-      <c r="I223">
+      <c r="L223">
         <f>IF(A223="","",F223*G223)</f>
         <v/>
       </c>
     </row>
     <row r="224">
-      <c r="I224">
+      <c r="L224">
         <f>IF(A224="","",F224*G224)</f>
         <v/>
       </c>
     </row>
     <row r="225">
-      <c r="I225">
+      <c r="L225">
         <f>IF(A225="","",F225*G225)</f>
         <v/>
       </c>
     </row>
     <row r="226">
-      <c r="I226">
+      <c r="L226">
         <f>IF(A226="","",F226*G226)</f>
         <v/>
       </c>
     </row>
     <row r="227">
-      <c r="I227">
+      <c r="L227">
         <f>IF(A227="","",F227*G227)</f>
         <v/>
       </c>
     </row>
     <row r="228">
-      <c r="I228">
+      <c r="L228">
         <f>IF(A228="","",F228*G228)</f>
         <v/>
       </c>
     </row>
     <row r="229">
-      <c r="I229">
+      <c r="L229">
         <f>IF(A229="","",F229*G229)</f>
         <v/>
       </c>
     </row>
     <row r="230">
-      <c r="I230">
+      <c r="L230">
         <f>IF(A230="","",F230*G230)</f>
         <v/>
       </c>
     </row>
     <row r="231">
-      <c r="I231">
+      <c r="L231">
         <f>IF(A231="","",F231*G231)</f>
         <v/>
       </c>
     </row>
     <row r="232">
-      <c r="I232">
+      <c r="L232">
         <f>IF(A232="","",F232*G232)</f>
         <v/>
       </c>
     </row>
     <row r="233">
-      <c r="I233">
+      <c r="L233">
         <f>IF(A233="","",F233*G233)</f>
         <v/>
       </c>
     </row>
     <row r="234">
-      <c r="I234">
+      <c r="L234">
         <f>IF(A234="","",F234*G234)</f>
         <v/>
       </c>
     </row>
     <row r="235">
-      <c r="I235">
+      <c r="L235">
         <f>IF(A235="","",F235*G235)</f>
         <v/>
       </c>
     </row>
     <row r="236">
-      <c r="I236">
+      <c r="L236">
         <f>IF(A236="","",F236*G236)</f>
         <v/>
       </c>
     </row>
     <row r="237">
-      <c r="I237">
+      <c r="L237">
         <f>IF(A237="","",F237*G237)</f>
         <v/>
       </c>
     </row>
     <row r="238">
-      <c r="I238">
+      <c r="L238">
         <f>IF(A238="","",F238*G238)</f>
         <v/>
       </c>
     </row>
     <row r="239">
-      <c r="I239">
+      <c r="L239">
         <f>IF(A239="","",F239*G239)</f>
         <v/>
       </c>
     </row>
     <row r="240">
-      <c r="I240">
+      <c r="L240">
         <f>IF(A240="","",F240*G240)</f>
         <v/>
       </c>
     </row>
     <row r="241">
-      <c r="I241">
+      <c r="L241">
         <f>IF(A241="","",F241*G241)</f>
         <v/>
       </c>
     </row>
     <row r="242">
-      <c r="I242">
+      <c r="L242">
         <f>IF(A242="","",F242*G242)</f>
         <v/>
       </c>
     </row>
     <row r="243">
-      <c r="I243">
+      <c r="L243">
         <f>IF(A243="","",F243*G243)</f>
         <v/>
       </c>
     </row>
     <row r="244">
-      <c r="I244">
+      <c r="L244">
         <f>IF(A244="","",F244*G244)</f>
         <v/>
       </c>
     </row>
     <row r="245">
-      <c r="I245">
+      <c r="L245">
         <f>IF(A245="","",F245*G245)</f>
         <v/>
       </c>
     </row>
     <row r="246">
-      <c r="I246">
+      <c r="L246">
         <f>IF(A246="","",F246*G246)</f>
         <v/>
       </c>
     </row>
     <row r="247">
-      <c r="I247">
+      <c r="L247">
         <f>IF(A247="","",F247*G247)</f>
         <v/>
       </c>
     </row>
     <row r="248">
-      <c r="I248">
+      <c r="L248">
         <f>IF(A248="","",F248*G248)</f>
         <v/>
       </c>
     </row>
     <row r="249">
-      <c r="I249">
+      <c r="L249">
         <f>IF(A249="","",F249*G249)</f>
         <v/>
       </c>
     </row>
     <row r="250">
-      <c r="I250">
+      <c r="L250">
         <f>IF(A250="","",F250*G250)</f>
         <v/>
       </c>
     </row>
     <row r="251">
-      <c r="I251">
+      <c r="L251">
         <f>IF(A251="","",F251*G251)</f>
         <v/>
       </c>
     </row>
     <row r="252">
-      <c r="I252">
+      <c r="L252">
         <f>IF(A252="","",F252*G252)</f>
         <v/>
       </c>
     </row>
     <row r="253">
-      <c r="I253">
+      <c r="L253">
         <f>IF(A253="","",F253*G253)</f>
         <v/>
       </c>
     </row>
     <row r="254">
-      <c r="I254">
+      <c r="L254">
         <f>IF(A254="","",F254*G254)</f>
         <v/>
       </c>
     </row>
     <row r="255">
-      <c r="I255">
+      <c r="L255">
         <f>IF(A255="","",F255*G255)</f>
         <v/>
       </c>
     </row>
     <row r="256">
-      <c r="I256">
+      <c r="L256">
         <f>IF(A256="","",F256*G256)</f>
         <v/>
       </c>
     </row>
     <row r="257">
-      <c r="I257">
+      <c r="L257">
         <f>IF(A257="","",F257*G257)</f>
         <v/>
       </c>
     </row>
     <row r="258">
-      <c r="I258">
+      <c r="L258">
         <f>IF(A258="","",F258*G258)</f>
         <v/>
       </c>
     </row>
     <row r="259">
-      <c r="I259">
+      <c r="L259">
         <f>IF(A259="","",F259*G259)</f>
         <v/>
       </c>
     </row>
     <row r="260">
-      <c r="I260">
+      <c r="L260">
         <f>IF(A260="","",F260*G260)</f>
         <v/>
       </c>
     </row>
     <row r="261">
-      <c r="I261">
+      <c r="L261">
         <f>IF(A261="","",F261*G261)</f>
         <v/>
       </c>
     </row>
     <row r="262">
-      <c r="I262">
+      <c r="L262">
         <f>IF(A262="","",F262*G262)</f>
         <v/>
       </c>
     </row>
     <row r="263">
-      <c r="I263">
+      <c r="L263">
         <f>IF(A263="","",F263*G263)</f>
         <v/>
       </c>
     </row>
     <row r="264">
-      <c r="I264">
+      <c r="L264">
         <f>IF(A264="","",F264*G264)</f>
         <v/>
       </c>
     </row>
     <row r="265">
-      <c r="I265">
+      <c r="L265">
         <f>IF(A265="","",F265*G265)</f>
         <v/>
       </c>
     </row>
     <row r="266">
-      <c r="I266">
+      <c r="L266">
         <f>IF(A266="","",F266*G266)</f>
         <v/>
       </c>
     </row>
     <row r="267">
-      <c r="I267">
+      <c r="L267">
         <f>IF(A267="","",F267*G267)</f>
         <v/>
       </c>
     </row>
     <row r="268">
-      <c r="I268">
+      <c r="L268">
         <f>IF(A268="","",F268*G268)</f>
         <v/>
       </c>
     </row>
     <row r="269">
-      <c r="I269">
+      <c r="L269">
         <f>IF(A269="","",F269*G269)</f>
         <v/>
       </c>
     </row>
     <row r="270">
-      <c r="I270">
+      <c r="L270">
         <f>IF(A270="","",F270*G270)</f>
         <v/>
       </c>
     </row>
     <row r="271">
-      <c r="I271">
+      <c r="L271">
         <f>IF(A271="","",F271*G271)</f>
         <v/>
       </c>
     </row>
     <row r="272">
-      <c r="I272">
+      <c r="L272">
         <f>IF(A272="","",F272*G272)</f>
         <v/>
       </c>
     </row>
     <row r="273">
-      <c r="I273">
+      <c r="L273">
         <f>IF(A273="","",F273*G273)</f>
         <v/>
       </c>
     </row>
     <row r="274">
-      <c r="I274">
+      <c r="L274">
         <f>IF(A274="","",F274*G274)</f>
         <v/>
       </c>
     </row>
     <row r="275">
-      <c r="I275">
+      <c r="L275">
         <f>IF(A275="","",F275*G275)</f>
         <v/>
       </c>
     </row>
     <row r="276">
-      <c r="I276">
+      <c r="L276">
         <f>IF(A276="","",F276*G276)</f>
         <v/>
       </c>
     </row>
     <row r="277">
-      <c r="I277">
+      <c r="L277">
         <f>IF(A277="","",F277*G277)</f>
         <v/>
       </c>
     </row>
     <row r="278">
-      <c r="I278">
+      <c r="L278">
         <f>IF(A278="","",F278*G278)</f>
         <v/>
       </c>
     </row>
     <row r="279">
-      <c r="I279">
+      <c r="L279">
         <f>IF(A279="","",F279*G279)</f>
         <v/>
       </c>
     </row>
     <row r="280">
-      <c r="I280">
+      <c r="L280">
         <f>IF(A280="","",F280*G280)</f>
         <v/>
       </c>
     </row>
     <row r="281">
-      <c r="I281">
+      <c r="L281">
         <f>IF(A281="","",F281*G281)</f>
         <v/>
       </c>
     </row>
     <row r="282">
-      <c r="I282">
+      <c r="L282">
         <f>IF(A282="","",F282*G282)</f>
         <v/>
       </c>
     </row>
     <row r="283">
-      <c r="I283">
+      <c r="L283">
         <f>IF(A283="","",F283*G283)</f>
         <v/>
       </c>
     </row>
     <row r="284">
-      <c r="I284">
+      <c r="L284">
         <f>IF(A284="","",F284*G284)</f>
         <v/>
       </c>
     </row>
     <row r="285">
-      <c r="I285">
+      <c r="L285">
         <f>IF(A285="","",F285*G285)</f>
         <v/>
       </c>
     </row>
     <row r="286">
-      <c r="I286">
+      <c r="L286">
         <f>IF(A286="","",F286*G286)</f>
         <v/>
       </c>
     </row>
     <row r="287">
-      <c r="I287">
+      <c r="L287">
         <f>IF(A287="","",F287*G287)</f>
         <v/>
       </c>
     </row>
     <row r="288">
-      <c r="I288">
+      <c r="L288">
         <f>IF(A288="","",F288*G288)</f>
         <v/>
       </c>
     </row>
     <row r="289">
-      <c r="I289">
+      <c r="L289">
         <f>IF(A289="","",F289*G289)</f>
         <v/>
       </c>
     </row>
     <row r="290">
-      <c r="I290">
+      <c r="L290">
         <f>IF(A290="","",F290*G290)</f>
         <v/>
       </c>
     </row>
     <row r="291">
-      <c r="I291">
+      <c r="L291">
         <f>IF(A291="","",F291*G291)</f>
         <v/>
       </c>
     </row>
     <row r="292">
-      <c r="I292">
+      <c r="L292">
         <f>IF(A292="","",F292*G292)</f>
         <v/>
       </c>
     </row>
     <row r="293">
-      <c r="I293">
+      <c r="L293">
         <f>IF(A293="","",F293*G293)</f>
         <v/>
       </c>
     </row>
     <row r="294">
-      <c r="I294">
+      <c r="L294">
         <f>IF(A294="","",F294*G294)</f>
         <v/>
       </c>
     </row>
     <row r="295">
-      <c r="I295">
+      <c r="L295">
         <f>IF(A295="","",F295*G295)</f>
         <v/>
       </c>
     </row>
     <row r="296">
-      <c r="I296">
+      <c r="L296">
         <f>IF(A296="","",F296*G296)</f>
         <v/>
       </c>
     </row>
     <row r="297">
-      <c r="I297">
+      <c r="L297">
         <f>IF(A297="","",F297*G297)</f>
         <v/>
       </c>
     </row>
     <row r="298">
-      <c r="I298">
+      <c r="L298">
         <f>IF(A298="","",F298*G298)</f>
         <v/>
       </c>
     </row>
     <row r="299">
-      <c r="I299">
+      <c r="L299">
         <f>IF(A299="","",F299*G299)</f>
         <v/>
       </c>
     </row>
     <row r="300">
-      <c r="I300">
+      <c r="L300">
         <f>IF(A300="","",F300*G300)</f>
         <v/>
       </c>
     </row>
     <row r="301">
-      <c r="I301">
+      <c r="L301">
         <f>IF(A301="","",F301*G301)</f>
         <v/>
       </c>
     </row>
     <row r="302">
-      <c r="I302">
+      <c r="L302">
         <f>IF(A302="","",F302*G302)</f>
         <v/>
       </c>
     </row>
     <row r="303">
-      <c r="I303">
+      <c r="L303">
         <f>IF(A303="","",F303*G303)</f>
         <v/>
       </c>
     </row>
     <row r="304">
-      <c r="I304">
+      <c r="L304">
         <f>IF(A304="","",F304*G304)</f>
         <v/>
       </c>
     </row>
     <row r="305">
-      <c r="I305">
+      <c r="L305">
         <f>IF(A305="","",F305*G305)</f>
         <v/>
       </c>
     </row>
     <row r="306">
-      <c r="I306">
+      <c r="L306">
         <f>IF(A306="","",F306*G306)</f>
         <v/>
       </c>
     </row>
     <row r="307">
-      <c r="I307">
+      <c r="L307">
         <f>IF(A307="","",F307*G307)</f>
         <v/>
       </c>
     </row>
     <row r="308">
-      <c r="I308">
+      <c r="L308">
         <f>IF(A308="","",F308*G308)</f>
         <v/>
       </c>
     </row>
     <row r="309">
-      <c r="I309">
+      <c r="L309">
         <f>IF(A309="","",F309*G309)</f>
         <v/>
       </c>
     </row>
     <row r="310">
-      <c r="I310">
+      <c r="L310">
         <f>IF(A310="","",F310*G310)</f>
         <v/>
       </c>
     </row>
     <row r="311">
-      <c r="I311">
+      <c r="L311">
         <f>IF(A311="","",F311*G311)</f>
         <v/>
       </c>
     </row>
     <row r="312">
-      <c r="I312">
+      <c r="L312">
         <f>IF(A312="","",F312*G312)</f>
         <v/>
       </c>
     </row>
     <row r="313">
-      <c r="I313">
+      <c r="L313">
         <f>IF(A313="","",F313*G313)</f>
         <v/>
       </c>
     </row>
     <row r="314">
-      <c r="I314">
+      <c r="L314">
         <f>IF(A314="","",F314*G314)</f>
         <v/>
       </c>
     </row>
     <row r="315">
-      <c r="I315">
+      <c r="L315">
         <f>IF(A315="","",F315*G315)</f>
         <v/>
       </c>
     </row>
     <row r="316">
-      <c r="I316">
+      <c r="L316">
         <f>IF(A316="","",F316*G316)</f>
         <v/>
       </c>
     </row>
     <row r="317">
-      <c r="I317">
+      <c r="L317">
         <f>IF(A317="","",F317*G317)</f>
         <v/>
       </c>
     </row>
     <row r="318">
-      <c r="I318">
+      <c r="L318">
         <f>IF(A318="","",F318*G318)</f>
         <v/>
       </c>
     </row>
     <row r="319">
-      <c r="I319">
+      <c r="L319">
         <f>IF(A319="","",F319*G319)</f>
         <v/>
       </c>
     </row>
     <row r="320">
-      <c r="I320">
+      <c r="L320">
         <f>IF(A320="","",F320*G320)</f>
         <v/>
       </c>
     </row>
     <row r="321">
-      <c r="I321">
+      <c r="L321">
         <f>IF(A321="","",F321*G321)</f>
         <v/>
       </c>
     </row>
     <row r="322">
-      <c r="I322">
+      <c r="L322">
         <f>IF(A322="","",F322*G322)</f>
         <v/>
       </c>
     </row>
     <row r="323">
-      <c r="I323">
+      <c r="L323">
         <f>IF(A323="","",F323*G323)</f>
         <v/>
       </c>
     </row>
     <row r="324">
-      <c r="I324">
+      <c r="L324">
         <f>IF(A324="","",F324*G324)</f>
         <v/>
       </c>
     </row>
     <row r="325">
-      <c r="I325">
+      <c r="L325">
         <f>IF(A325="","",F325*G325)</f>
         <v/>
       </c>
     </row>
     <row r="326">
-      <c r="I326">
+      <c r="L326">
         <f>IF(A326="","",F326*G326)</f>
         <v/>
       </c>
     </row>
     <row r="327">
-      <c r="I327">
+      <c r="L327">
         <f>IF(A327="","",F327*G327)</f>
         <v/>
       </c>
     </row>
     <row r="328">
-      <c r="I328">
+      <c r="L328">
         <f>IF(A328="","",F328*G328)</f>
         <v/>
       </c>
     </row>
     <row r="329">
-      <c r="I329">
+      <c r="L329">
         <f>IF(A329="","",F329*G329)</f>
         <v/>
       </c>
     </row>
     <row r="330">
-      <c r="I330">
+      <c r="L330">
         <f>IF(A330="","",F330*G330)</f>
         <v/>
       </c>
     </row>
     <row r="331">
-      <c r="I331">
+      <c r="L331">
         <f>IF(A331="","",F331*G331)</f>
         <v/>
       </c>
     </row>
     <row r="332">
-      <c r="I332">
+      <c r="L332">
         <f>IF(A332="","",F332*G332)</f>
         <v/>
       </c>
     </row>
     <row r="333">
-      <c r="I333">
+      <c r="L333">
         <f>IF(A333="","",F333*G333)</f>
         <v/>
       </c>
     </row>
     <row r="334">
-      <c r="I334">
+      <c r="L334">
         <f>IF(A334="","",F334*G334)</f>
         <v/>
       </c>
     </row>
     <row r="335">
-      <c r="I335">
+      <c r="L335">
         <f>IF(A335="","",F335*G335)</f>
         <v/>
       </c>
     </row>
     <row r="336">
-      <c r="I336">
+      <c r="L336">
         <f>IF(A336="","",F336*G336)</f>
         <v/>
       </c>
     </row>
     <row r="337">
-      <c r="I337">
+      <c r="L337">
         <f>IF(A337="","",F337*G337)</f>
         <v/>
       </c>
     </row>
     <row r="338">
-      <c r="I338">
+      <c r="L338">
         <f>IF(A338="","",F338*G338)</f>
         <v/>
       </c>
     </row>
     <row r="339">
-      <c r="I339">
+      <c r="L339">
         <f>IF(A339="","",F339*G339)</f>
         <v/>
       </c>
     </row>
     <row r="340">
-      <c r="I340">
+      <c r="L340">
         <f>IF(A340="","",F340*G340)</f>
         <v/>
       </c>
     </row>
     <row r="341">
-      <c r="I341">
+      <c r="L341">
         <f>IF(A341="","",F341*G341)</f>
         <v/>
       </c>
     </row>
     <row r="342">
-      <c r="I342">
+      <c r="L342">
         <f>IF(A342="","",F342*G342)</f>
         <v/>
       </c>
     </row>
     <row r="343">
-      <c r="I343">
+      <c r="L343">
         <f>IF(A343="","",F343*G343)</f>
         <v/>
       </c>
     </row>
     <row r="344">
-      <c r="I344">
+      <c r="L344">
         <f>IF(A344="","",F344*G344)</f>
         <v/>
       </c>
     </row>
     <row r="345">
-      <c r="I345">
+      <c r="L345">
         <f>IF(A345="","",F345*G345)</f>
         <v/>
       </c>
     </row>
     <row r="346">
-      <c r="I346">
+      <c r="L346">
         <f>IF(A346="","",F346*G346)</f>
         <v/>
       </c>
     </row>
     <row r="347">
-      <c r="I347">
+      <c r="L347">
         <f>IF(A347="","",F347*G347)</f>
         <v/>
       </c>
     </row>
     <row r="348">
-      <c r="I348">
+      <c r="L348">
         <f>IF(A348="","",F348*G348)</f>
         <v/>
       </c>
     </row>
     <row r="349">
-      <c r="I349">
+      <c r="L349">
         <f>IF(A349="","",F349*G349)</f>
         <v/>
       </c>
     </row>
     <row r="350">
-      <c r="I350">
+      <c r="L350">
         <f>IF(A350="","",F350*G350)</f>
         <v/>
       </c>
     </row>
     <row r="351">
-      <c r="I351">
+      <c r="L351">
         <f>IF(A351="","",F351*G351)</f>
         <v/>
       </c>
     </row>
     <row r="352">
-      <c r="I352">
+      <c r="L352">
         <f>IF(A352="","",F352*G352)</f>
         <v/>
       </c>
     </row>
     <row r="353">
-      <c r="I353">
+      <c r="L353">
         <f>IF(A353="","",F353*G353)</f>
         <v/>
       </c>
     </row>
     <row r="354">
-      <c r="I354">
+      <c r="L354">
         <f>IF(A354="","",F354*G354)</f>
         <v/>
       </c>
     </row>
     <row r="355">
-      <c r="I355">
+      <c r="L355">
         <f>IF(A355="","",F355*G355)</f>
         <v/>
       </c>
     </row>
     <row r="356">
-      <c r="I356">
+      <c r="L356">
         <f>IF(A356="","",F356*G356)</f>
         <v/>
       </c>
     </row>
     <row r="357">
-      <c r="I357">
+      <c r="L357">
         <f>IF(A357="","",F357*G357)</f>
         <v/>
       </c>
     </row>
     <row r="358">
-      <c r="I358">
+      <c r="L358">
         <f>IF(A358="","",F358*G358)</f>
         <v/>
       </c>
     </row>
     <row r="359">
-      <c r="I359">
+      <c r="L359">
         <f>IF(A359="","",F359*G359)</f>
         <v/>
       </c>
     </row>
     <row r="360">
-      <c r="I360">
+      <c r="L360">
         <f>IF(A360="","",F360*G360)</f>
         <v/>
       </c>
     </row>
     <row r="361">
-      <c r="I361">
+      <c r="L361">
         <f>IF(A361="","",F361*G361)</f>
         <v/>
       </c>
     </row>
     <row r="362">
-      <c r="I362">
+      <c r="L362">
         <f>IF(A362="","",F362*G362)</f>
         <v/>
       </c>
     </row>
     <row r="363">
-      <c r="I363">
+      <c r="L363">
         <f>IF(A363="","",F363*G363)</f>
         <v/>
       </c>
     </row>
     <row r="364">
-      <c r="I364">
+      <c r="L364">
         <f>IF(A364="","",F364*G364)</f>
         <v/>
       </c>
     </row>
     <row r="365">
-      <c r="I365">
+      <c r="L365">
         <f>IF(A365="","",F365*G365)</f>
         <v/>
       </c>
     </row>
     <row r="366">
-      <c r="I366">
+      <c r="L366">
         <f>IF(A366="","",F366*G366)</f>
         <v/>
       </c>
     </row>
     <row r="367">
-      <c r="I367">
+      <c r="L367">
         <f>IF(A367="","",F367*G367)</f>
         <v/>
       </c>
     </row>
     <row r="368">
-      <c r="I368">
+      <c r="L368">
         <f>IF(A368="","",F368*G368)</f>
         <v/>
       </c>
     </row>
     <row r="369">
-      <c r="I369">
+      <c r="L369">
         <f>IF(A369="","",F369*G369)</f>
         <v/>
       </c>
     </row>
     <row r="370">
-      <c r="I370">
+      <c r="L370">
         <f>IF(A370="","",F370*G370)</f>
         <v/>
       </c>
     </row>
     <row r="371">
-      <c r="I371">
+      <c r="L371">
         <f>IF(A371="","",F371*G371)</f>
         <v/>
       </c>
     </row>
     <row r="372">
-      <c r="I372">
+      <c r="L372">
         <f>IF(A372="","",F372*G372)</f>
         <v/>
       </c>
     </row>
     <row r="373">
-      <c r="I373">
+      <c r="L373">
         <f>IF(A373="","",F373*G373)</f>
         <v/>
       </c>
     </row>
     <row r="374">
-      <c r="I374">
+      <c r="L374">
         <f>IF(A374="","",F374*G374)</f>
         <v/>
       </c>
     </row>
     <row r="375">
-      <c r="I375">
+      <c r="L375">
         <f>IF(A375="","",F375*G375)</f>
         <v/>
       </c>
     </row>
     <row r="376">
-      <c r="I376">
+      <c r="L376">
         <f>IF(A376="","",F376*G376)</f>
         <v/>
       </c>
     </row>
     <row r="377">
-      <c r="I377">
+      <c r="L377">
         <f>IF(A377="","",F377*G377)</f>
         <v/>
       </c>
     </row>
     <row r="378">
-      <c r="I378">
+      <c r="L378">
         <f>IF(A378="","",F378*G378)</f>
         <v/>
       </c>
     </row>
     <row r="379">
-      <c r="I379">
+      <c r="L379">
         <f>IF(A379="","",F379*G379)</f>
         <v/>
       </c>
     </row>
     <row r="380">
-      <c r="I380">
+      <c r="L380">
         <f>IF(A380="","",F380*G380)</f>
         <v/>
       </c>
     </row>
     <row r="381">
-      <c r="I381">
+      <c r="L381">
         <f>IF(A381="","",F381*G381)</f>
         <v/>
       </c>
     </row>
     <row r="382">
-      <c r="I382">
+      <c r="L382">
         <f>IF(A382="","",F382*G382)</f>
         <v/>
       </c>
     </row>
     <row r="383">
-      <c r="I383">
+      <c r="L383">
         <f>IF(A383="","",F383*G383)</f>
         <v/>
       </c>
     </row>
     <row r="384">
-      <c r="I384">
+      <c r="L384">
         <f>IF(A384="","",F384*G384)</f>
         <v/>
       </c>
     </row>
     <row r="385">
-      <c r="I385">
+      <c r="L385">
         <f>IF(A385="","",F385*G385)</f>
         <v/>
       </c>
     </row>
     <row r="386">
-      <c r="I386">
+      <c r="L386">
         <f>IF(A386="","",F386*G386)</f>
         <v/>
       </c>
     </row>
     <row r="387">
-      <c r="I387">
+      <c r="L387">
         <f>IF(A387="","",F387*G387)</f>
         <v/>
       </c>
     </row>
     <row r="388">
-      <c r="I388">
+      <c r="L388">
         <f>IF(A388="","",F388*G388)</f>
         <v/>
       </c>
     </row>
     <row r="389">
-      <c r="I389">
+      <c r="L389">
         <f>IF(A389="","",F389*G389)</f>
         <v/>
       </c>
     </row>
     <row r="390">
-      <c r="I390">
+      <c r="L390">
         <f>IF(A390="","",F390*G390)</f>
         <v/>
       </c>
     </row>
     <row r="391">
-      <c r="I391">
+      <c r="L391">
         <f>IF(A391="","",F391*G391)</f>
         <v/>
       </c>
     </row>
     <row r="392">
-      <c r="I392">
+      <c r="L392">
         <f>IF(A392="","",F392*G392)</f>
         <v/>
       </c>
     </row>
     <row r="393">
-      <c r="I393">
+      <c r="L393">
         <f>IF(A393="","",F393*G393)</f>
         <v/>
       </c>
     </row>
     <row r="394">
-      <c r="I394">
+      <c r="L394">
         <f>IF(A394="","",F394*G394)</f>
         <v/>
       </c>
     </row>
     <row r="395">
-      <c r="I395">
+      <c r="L395">
         <f>IF(A395="","",F395*G395)</f>
         <v/>
       </c>
     </row>
     <row r="396">
-      <c r="I396">
+      <c r="L396">
         <f>IF(A396="","",F396*G396)</f>
         <v/>
       </c>
     </row>
     <row r="397">
-      <c r="I397">
+      <c r="L397">
         <f>IF(A397="","",F397*G397)</f>
         <v/>
       </c>
     </row>
     <row r="398">
-      <c r="I398">
+      <c r="L398">
         <f>IF(A398="","",F398*G398)</f>
         <v/>
       </c>
     </row>
     <row r="399">
-      <c r="I399">
+      <c r="L399">
         <f>IF(A399="","",F399*G399)</f>
         <v/>
       </c>
     </row>
     <row r="400">
-      <c r="I400">
+      <c r="L400">
         <f>IF(A400="","",F400*G400)</f>
         <v/>
       </c>
     </row>
     <row r="401">
-      <c r="I401">
+      <c r="L401">
         <f>IF(A401="","",F401*G401)</f>
         <v/>
       </c>
     </row>
     <row r="402">
-      <c r="I402">
+      <c r="L402">
         <f>IF(A402="","",F402*G402)</f>
         <v/>
       </c>
     </row>
     <row r="403">
-      <c r="I403">
+      <c r="L403">
         <f>IF(A403="","",F403*G403)</f>
         <v/>
       </c>
     </row>
     <row r="404">
-      <c r="I404">
+      <c r="L404">
         <f>IF(A404="","",F404*G404)</f>
         <v/>
       </c>
     </row>
     <row r="405">
-      <c r="I405">
+      <c r="L405">
         <f>IF(A405="","",F405*G405)</f>
         <v/>
       </c>
     </row>
     <row r="406">
-      <c r="I406">
+      <c r="L406">
         <f>IF(A406="","",F406*G406)</f>
         <v/>
       </c>
     </row>
     <row r="407">
-      <c r="I407">
+      <c r="L407">
         <f>IF(A407="","",F407*G407)</f>
         <v/>
       </c>
     </row>
     <row r="408">
-      <c r="I408">
+      <c r="L408">
         <f>IF(A408="","",F408*G408)</f>
         <v/>
       </c>
     </row>
     <row r="409">
-      <c r="I409">
+      <c r="L409">
         <f>IF(A409="","",F409*G409)</f>
         <v/>
       </c>
     </row>
     <row r="410">
-      <c r="I410">
+      <c r="L410">
         <f>IF(A410="","",F410*G410)</f>
         <v/>
       </c>
     </row>
     <row r="411">
-      <c r="I411">
+      <c r="L411">
         <f>IF(A411="","",F411*G411)</f>
         <v/>
       </c>
     </row>
     <row r="412">
-      <c r="I412">
+      <c r="L412">
         <f>IF(A412="","",F412*G412)</f>
         <v/>
       </c>
     </row>
     <row r="413">
-      <c r="I413">
+      <c r="L413">
         <f>IF(A413="","",F413*G413)</f>
         <v/>
       </c>
     </row>
     <row r="414">
-      <c r="I414">
+      <c r="L414">
         <f>IF(A414="","",F414*G414)</f>
         <v/>
       </c>
     </row>
     <row r="415">
-      <c r="I415">
+      <c r="L415">
         <f>IF(A415="","",F415*G415)</f>
         <v/>
       </c>
     </row>
     <row r="416">
-      <c r="I416">
+      <c r="L416">
         <f>IF(A416="","",F416*G416)</f>
         <v/>
       </c>
     </row>
     <row r="417">
-      <c r="I417">
+      <c r="L417">
         <f>IF(A417="","",F417*G417)</f>
         <v/>
       </c>
     </row>
     <row r="418">
-      <c r="I418">
+      <c r="L418">
         <f>IF(A418="","",F418*G418)</f>
         <v/>
       </c>
     </row>
     <row r="419">
-      <c r="I419">
+      <c r="L419">
         <f>IF(A419="","",F419*G419)</f>
         <v/>
       </c>
     </row>
     <row r="420">
-      <c r="I420">
+      <c r="L420">
         <f>IF(A420="","",F420*G420)</f>
         <v/>
       </c>
     </row>
     <row r="421">
-      <c r="I421">
+      <c r="L421">
         <f>IF(A421="","",F421*G421)</f>
         <v/>
       </c>
     </row>
     <row r="422">
-      <c r="I422">
+      <c r="L422">
         <f>IF(A422="","",F422*G422)</f>
         <v/>
       </c>
     </row>
     <row r="423">
-      <c r="I423">
+      <c r="L423">
         <f>IF(A423="","",F423*G423)</f>
         <v/>
       </c>
     </row>
     <row r="424">
-      <c r="I424">
+      <c r="L424">
         <f>IF(A424="","",F424*G424)</f>
         <v/>
       </c>
     </row>
     <row r="425">
-      <c r="I425">
+      <c r="L425">
         <f>IF(A425="","",F425*G425)</f>
         <v/>
       </c>
     </row>
     <row r="426">
-      <c r="I426">
+      <c r="L426">
         <f>IF(A426="","",F426*G426)</f>
         <v/>
       </c>
     </row>
     <row r="427">
-      <c r="I427">
+      <c r="L427">
         <f>IF(A427="","",F427*G427)</f>
         <v/>
       </c>
     </row>
     <row r="428">
-      <c r="I428">
+      <c r="L428">
         <f>IF(A428="","",F428*G428)</f>
         <v/>
       </c>
     </row>
     <row r="429">
-      <c r="I429">
+      <c r="L429">
         <f>IF(A429="","",F429*G429)</f>
         <v/>
       </c>
     </row>
     <row r="430">
-      <c r="I430">
+      <c r="L430">
         <f>IF(A430="","",F430*G430)</f>
         <v/>
       </c>
     </row>
     <row r="431">
-      <c r="I431">
+      <c r="L431">
         <f>IF(A431="","",F431*G431)</f>
         <v/>
       </c>
     </row>
     <row r="432">
-      <c r="I432">
+      <c r="L432">
         <f>IF(A432="","",F432*G432)</f>
         <v/>
       </c>
     </row>
     <row r="433">
-      <c r="I433">
+      <c r="L433">
         <f>IF(A433="","",F433*G433)</f>
         <v/>
       </c>
     </row>
     <row r="434">
-      <c r="I434">
+      <c r="L434">
         <f>IF(A434="","",F434*G434)</f>
         <v/>
       </c>
     </row>
     <row r="435">
-      <c r="I435">
+      <c r="L435">
         <f>IF(A435="","",F435*G435)</f>
         <v/>
       </c>
     </row>
     <row r="436">
-      <c r="I436">
+      <c r="L436">
         <f>IF(A436="","",F436*G436)</f>
         <v/>
       </c>
     </row>
     <row r="437">
-      <c r="I437">
+      <c r="L437">
         <f>IF(A437="","",F437*G437)</f>
         <v/>
       </c>
     </row>
     <row r="438">
-      <c r="I438">
+      <c r="L438">
         <f>IF(A438="","",F438*G438)</f>
         <v/>
       </c>
     </row>
     <row r="439">
-      <c r="I439">
+      <c r="L439">
         <f>IF(A439="","",F439*G439)</f>
         <v/>
       </c>
     </row>
     <row r="440">
-      <c r="I440">
+      <c r="L440">
         <f>IF(A440="","",F440*G440)</f>
         <v/>
       </c>
     </row>
     <row r="441">
-      <c r="I441">
+      <c r="L441">
         <f>IF(A441="","",F441*G441)</f>
         <v/>
       </c>
     </row>
     <row r="442">
-      <c r="I442">
+      <c r="L442">
         <f>IF(A442="","",F442*G442)</f>
         <v/>
       </c>
     </row>
     <row r="443">
-      <c r="I443">
+      <c r="L443">
         <f>IF(A443="","",F443*G443)</f>
         <v/>
       </c>
     </row>
     <row r="444">
-      <c r="I444">
+      <c r="L444">
         <f>IF(A444="","",F444*G444)</f>
         <v/>
       </c>
     </row>
     <row r="445">
-      <c r="I445">
+      <c r="L445">
         <f>IF(A445="","",F445*G445)</f>
         <v/>
       </c>
     </row>
     <row r="446">
-      <c r="I446">
+      <c r="L446">
         <f>IF(A446="","",F446*G446)</f>
         <v/>
       </c>
     </row>
     <row r="447">
-      <c r="I447">
+      <c r="L447">
         <f>IF(A447="","",F447*G447)</f>
         <v/>
       </c>
     </row>
     <row r="448">
-      <c r="I448">
+      <c r="L448">
         <f>IF(A448="","",F448*G448)</f>
         <v/>
       </c>
     </row>
     <row r="449">
-      <c r="I449">
+      <c r="L449">
         <f>IF(A449="","",F449*G449)</f>
         <v/>
       </c>
     </row>
     <row r="450">
-      <c r="I450">
+      <c r="L450">
         <f>IF(A450="","",F450*G450)</f>
         <v/>
       </c>
     </row>
     <row r="451">
-      <c r="I451">
+      <c r="L451">
         <f>IF(A451="","",F451*G451)</f>
         <v/>
       </c>
     </row>
     <row r="452">
-      <c r="I452">
+      <c r="L452">
         <f>IF(A452="","",F452*G452)</f>
         <v/>
       </c>
     </row>
     <row r="453">
-      <c r="I453">
+      <c r="L453">
         <f>IF(A453="","",F453*G453)</f>
         <v/>
       </c>
     </row>
     <row r="454">
-      <c r="I454">
+      <c r="L454">
         <f>IF(A454="","",F454*G454)</f>
         <v/>
       </c>
     </row>
     <row r="455">
-      <c r="I455">
+      <c r="L455">
         <f>IF(A455="","",F455*G455)</f>
         <v/>
       </c>
     </row>
     <row r="456">
-      <c r="I456">
+      <c r="L456">
         <f>IF(A456="","",F456*G456)</f>
         <v/>
       </c>
     </row>
     <row r="457">
-      <c r="I457">
+      <c r="L457">
         <f>IF(A457="","",F457*G457)</f>
         <v/>
       </c>
     </row>
     <row r="458">
-      <c r="I458">
+      <c r="L458">
         <f>IF(A458="","",F458*G458)</f>
         <v/>
       </c>
     </row>
     <row r="459">
-      <c r="I459">
+      <c r="L459">
         <f>IF(A459="","",F459*G459)</f>
         <v/>
       </c>
     </row>
     <row r="460">
-      <c r="I460">
+      <c r="L460">
         <f>IF(A460="","",F460*G460)</f>
         <v/>
       </c>
     </row>
     <row r="461">
-      <c r="I461">
+      <c r="L461">
         <f>IF(A461="","",F461*G461)</f>
         <v/>
       </c>
     </row>
     <row r="462">
-      <c r="I462">
+      <c r="L462">
         <f>IF(A462="","",F462*G462)</f>
         <v/>
       </c>
     </row>
     <row r="463">
-      <c r="I463">
+      <c r="L463">
         <f>IF(A463="","",F463*G463)</f>
         <v/>
       </c>
     </row>
     <row r="464">
-      <c r="I464">
+      <c r="L464">
         <f>IF(A464="","",F464*G464)</f>
         <v/>
       </c>
     </row>
     <row r="465">
-      <c r="I465">
+      <c r="L465">
         <f>IF(A465="","",F465*G465)</f>
         <v/>
       </c>
     </row>
     <row r="466">
-      <c r="I466">
+      <c r="L466">
         <f>IF(A466="","",F466*G466)</f>
         <v/>
       </c>
     </row>
     <row r="467">
-      <c r="I467">
+      <c r="L467">
         <f>IF(A467="","",F467*G467)</f>
         <v/>
       </c>
     </row>
     <row r="468">
-      <c r="I468">
+      <c r="L468">
         <f>IF(A468="","",F468*G468)</f>
         <v/>
       </c>
     </row>
     <row r="469">
-      <c r="I469">
+      <c r="L469">
         <f>IF(A469="","",F469*G469)</f>
         <v/>
       </c>
     </row>
     <row r="470">
-      <c r="I470">
+      <c r="L470">
         <f>IF(A470="","",F470*G470)</f>
         <v/>
       </c>
     </row>
     <row r="471">
-      <c r="I471">
+      <c r="L471">
         <f>IF(A471="","",F471*G471)</f>
         <v/>
       </c>
     </row>
     <row r="472">
-      <c r="I472">
+      <c r="L472">
         <f>IF(A472="","",F472*G472)</f>
         <v/>
       </c>
     </row>
     <row r="473">
-      <c r="I473">
+      <c r="L473">
         <f>IF(A473="","",F473*G473)</f>
         <v/>
       </c>
     </row>
     <row r="474">
-      <c r="I474">
+      <c r="L474">
         <f>IF(A474="","",F474*G474)</f>
         <v/>
       </c>
     </row>
     <row r="475">
-      <c r="I475">
+      <c r="L475">
         <f>IF(A475="","",F475*G475)</f>
         <v/>
       </c>
     </row>
     <row r="476">
-      <c r="I476">
+      <c r="L476">
         <f>IF(A476="","",F476*G476)</f>
         <v/>
       </c>
     </row>
     <row r="477">
-      <c r="I477">
+      <c r="L477">
         <f>IF(A477="","",F477*G477)</f>
         <v/>
       </c>
     </row>
     <row r="478">
-      <c r="I478">
+      <c r="L478">
         <f>IF(A478="","",F478*G478)</f>
         <v/>
       </c>
     </row>
     <row r="479">
-      <c r="I479">
+      <c r="L479">
         <f>IF(A479="","",F479*G479)</f>
         <v/>
       </c>
     </row>
     <row r="480">
-      <c r="I480">
+      <c r="L480">
         <f>IF(A480="","",F480*G480)</f>
         <v/>
       </c>
     </row>
     <row r="481">
-      <c r="I481">
+      <c r="L481">
         <f>IF(A481="","",F481*G481)</f>
         <v/>
       </c>
     </row>
     <row r="482">
-      <c r="I482">
+      <c r="L482">
         <f>IF(A482="","",F482*G482)</f>
         <v/>
       </c>
     </row>
     <row r="483">
-      <c r="I483">
+      <c r="L483">
         <f>IF(A483="","",F483*G483)</f>
         <v/>
       </c>
     </row>
     <row r="484">
-      <c r="I484">
+      <c r="L484">
         <f>IF(A484="","",F484*G484)</f>
         <v/>
       </c>
     </row>
     <row r="485">
-      <c r="I485">
+      <c r="L485">
         <f>IF(A485="","",F485*G485)</f>
         <v/>
       </c>
     </row>
     <row r="486">
-      <c r="I486">
+      <c r="L486">
         <f>IF(A486="","",F486*G486)</f>
         <v/>
       </c>
     </row>
     <row r="487">
-      <c r="I487">
+      <c r="L487">
         <f>IF(A487="","",F487*G487)</f>
         <v/>
       </c>
     </row>
     <row r="488">
-      <c r="I488">
+      <c r="L488">
         <f>IF(A488="","",F488*G488)</f>
         <v/>
       </c>
     </row>
     <row r="489">
-      <c r="I489">
+      <c r="L489">
         <f>IF(A489="","",F489*G489)</f>
         <v/>
       </c>
     </row>
     <row r="490">
-      <c r="I490">
+      <c r="L490">
         <f>IF(A490="","",F490*G490)</f>
         <v/>
       </c>
     </row>
     <row r="491">
-      <c r="I491">
+      <c r="L491">
         <f>IF(A491="","",F491*G491)</f>
         <v/>
       </c>
     </row>
     <row r="492">
-      <c r="I492">
+      <c r="L492">
         <f>IF(A492="","",F492*G492)</f>
         <v/>
       </c>
     </row>
     <row r="493">
-      <c r="I493">
+      <c r="L493">
         <f>IF(A493="","",F493*G493)</f>
         <v/>
       </c>
     </row>
     <row r="494">
-      <c r="I494">
+      <c r="L494">
         <f>IF(A494="","",F494*G494)</f>
         <v/>
       </c>
     </row>
     <row r="495">
-      <c r="I495">
+      <c r="L495">
         <f>IF(A495="","",F495*G495)</f>
         <v/>
       </c>
     </row>
     <row r="496">
-      <c r="I496">
+      <c r="L496">
         <f>IF(A496="","",F496*G496)</f>
         <v/>
       </c>
     </row>
     <row r="497">
-      <c r="I497">
+      <c r="L497">
         <f>IF(A497="","",F497*G497)</f>
         <v/>
       </c>
     </row>
     <row r="498">
-      <c r="I498">
+      <c r="L498">
         <f>IF(A498="","",F498*G498)</f>
         <v/>
       </c>
     </row>
     <row r="499">
-      <c r="I499">
+      <c r="L499">
         <f>IF(A499="","",F499*G499)</f>
         <v/>
       </c>
     </row>
     <row r="500">
-      <c r="I500">
+      <c r="L500">
         <f>IF(A500="","",F500*G500)</f>
         <v/>
       </c>
     </row>
     <row r="501">
-      <c r="I501">
+      <c r="L501">
         <f>IF(A501="","",F501*G501)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"cash,upi,whatsapp,bank"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix MAXIFS prefix in template for Excel compatibility
</commit_message>
<xml_diff>
--- a/data/Ayyappa_Pooja_Store_Data.xlsx
+++ b/data/Ayyappa_Pooja_Store_Data.xlsx
@@ -15892,7 +15892,7 @@
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>IF(A2="","",IF(D2=0,"",MAXIFS(Sales!C:C,Sales!D:D,A2)))</f>
+        <f>IF(A2="","",IF(D2=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A2)))</f>
         <v/>
       </c>
       <c r="G2">
@@ -15926,7 +15926,7 @@
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>IF(A3="","",IF(D3=0,"",MAXIFS(Sales!C:C,Sales!D:D,A3)))</f>
+        <f>IF(A3="","",IF(D3=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A3)))</f>
         <v/>
       </c>
       <c r="G3">
@@ -15960,7 +15960,7 @@
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>IF(A4="","",IF(D4=0,"",MAXIFS(Sales!C:C,Sales!D:D,A4)))</f>
+        <f>IF(A4="","",IF(D4=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A4)))</f>
         <v/>
       </c>
       <c r="G4">
@@ -15994,7 +15994,7 @@
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>IF(A5="","",IF(D5=0,"",MAXIFS(Sales!C:C,Sales!D:D,A5)))</f>
+        <f>IF(A5="","",IF(D5=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A5)))</f>
         <v/>
       </c>
       <c r="G5">
@@ -16028,7 +16028,7 @@
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>IF(A6="","",IF(D6=0,"",MAXIFS(Sales!C:C,Sales!D:D,A6)))</f>
+        <f>IF(A6="","",IF(D6=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A6)))</f>
         <v/>
       </c>
       <c r="G6">
@@ -16062,7 +16062,7 @@
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>IF(A7="","",IF(D7=0,"",MAXIFS(Sales!C:C,Sales!D:D,A7)))</f>
+        <f>IF(A7="","",IF(D7=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A7)))</f>
         <v/>
       </c>
       <c r="G7">
@@ -16096,7 +16096,7 @@
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>IF(A8="","",IF(D8=0,"",MAXIFS(Sales!C:C,Sales!D:D,A8)))</f>
+        <f>IF(A8="","",IF(D8=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A8)))</f>
         <v/>
       </c>
       <c r="G8">
@@ -16130,7 +16130,7 @@
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>IF(A9="","",IF(D9=0,"",MAXIFS(Sales!C:C,Sales!D:D,A9)))</f>
+        <f>IF(A9="","",IF(D9=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A9)))</f>
         <v/>
       </c>
       <c r="G9">
@@ -16164,7 +16164,7 @@
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>IF(A10="","",IF(D10=0,"",MAXIFS(Sales!C:C,Sales!D:D,A10)))</f>
+        <f>IF(A10="","",IF(D10=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A10)))</f>
         <v/>
       </c>
       <c r="G10">
@@ -16198,7 +16198,7 @@
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>IF(A11="","",IF(D11=0,"",MAXIFS(Sales!C:C,Sales!D:D,A11)))</f>
+        <f>IF(A11="","",IF(D11=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A11)))</f>
         <v/>
       </c>
       <c r="G11">
@@ -16232,7 +16232,7 @@
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>IF(A12="","",IF(D12=0,"",MAXIFS(Sales!C:C,Sales!D:D,A12)))</f>
+        <f>IF(A12="","",IF(D12=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A12)))</f>
         <v/>
       </c>
       <c r="G12">
@@ -16266,7 +16266,7 @@
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>IF(A13="","",IF(D13=0,"",MAXIFS(Sales!C:C,Sales!D:D,A13)))</f>
+        <f>IF(A13="","",IF(D13=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A13)))</f>
         <v/>
       </c>
       <c r="G13">
@@ -16300,7 +16300,7 @@
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>IF(A14="","",IF(D14=0,"",MAXIFS(Sales!C:C,Sales!D:D,A14)))</f>
+        <f>IF(A14="","",IF(D14=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A14)))</f>
         <v/>
       </c>
       <c r="G14">
@@ -16334,7 +16334,7 @@
         <v/>
       </c>
       <c r="F15" s="3">
-        <f>IF(A15="","",IF(D15=0,"",MAXIFS(Sales!C:C,Sales!D:D,A15)))</f>
+        <f>IF(A15="","",IF(D15=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A15)))</f>
         <v/>
       </c>
       <c r="G15">
@@ -16368,7 +16368,7 @@
         <v/>
       </c>
       <c r="F16" s="3">
-        <f>IF(A16="","",IF(D16=0,"",MAXIFS(Sales!C:C,Sales!D:D,A16)))</f>
+        <f>IF(A16="","",IF(D16=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A16)))</f>
         <v/>
       </c>
       <c r="G16">
@@ -16402,7 +16402,7 @@
         <v/>
       </c>
       <c r="F17" s="3">
-        <f>IF(A17="","",IF(D17=0,"",MAXIFS(Sales!C:C,Sales!D:D,A17)))</f>
+        <f>IF(A17="","",IF(D17=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A17)))</f>
         <v/>
       </c>
       <c r="G17">
@@ -16436,7 +16436,7 @@
         <v/>
       </c>
       <c r="F18" s="3">
-        <f>IF(A18="","",IF(D18=0,"",MAXIFS(Sales!C:C,Sales!D:D,A18)))</f>
+        <f>IF(A18="","",IF(D18=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A18)))</f>
         <v/>
       </c>
       <c r="G18">
@@ -16470,7 +16470,7 @@
         <v/>
       </c>
       <c r="F19" s="3">
-        <f>IF(A19="","",IF(D19=0,"",MAXIFS(Sales!C:C,Sales!D:D,A19)))</f>
+        <f>IF(A19="","",IF(D19=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A19)))</f>
         <v/>
       </c>
       <c r="G19">
@@ -16504,7 +16504,7 @@
         <v/>
       </c>
       <c r="F20" s="3">
-        <f>IF(A20="","",IF(D20=0,"",MAXIFS(Sales!C:C,Sales!D:D,A20)))</f>
+        <f>IF(A20="","",IF(D20=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A20)))</f>
         <v/>
       </c>
       <c r="G20">
@@ -16538,7 +16538,7 @@
         <v/>
       </c>
       <c r="F21" s="3">
-        <f>IF(A21="","",IF(D21=0,"",MAXIFS(Sales!C:C,Sales!D:D,A21)))</f>
+        <f>IF(A21="","",IF(D21=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A21)))</f>
         <v/>
       </c>
       <c r="G21">
@@ -16572,7 +16572,7 @@
         <v/>
       </c>
       <c r="F22" s="3">
-        <f>IF(A22="","",IF(D22=0,"",MAXIFS(Sales!C:C,Sales!D:D,A22)))</f>
+        <f>IF(A22="","",IF(D22=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A22)))</f>
         <v/>
       </c>
       <c r="G22">
@@ -16606,7 +16606,7 @@
         <v/>
       </c>
       <c r="F23" s="3">
-        <f>IF(A23="","",IF(D23=0,"",MAXIFS(Sales!C:C,Sales!D:D,A23)))</f>
+        <f>IF(A23="","",IF(D23=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A23)))</f>
         <v/>
       </c>
       <c r="G23">
@@ -16640,7 +16640,7 @@
         <v/>
       </c>
       <c r="F24" s="3">
-        <f>IF(A24="","",IF(D24=0,"",MAXIFS(Sales!C:C,Sales!D:D,A24)))</f>
+        <f>IF(A24="","",IF(D24=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A24)))</f>
         <v/>
       </c>
       <c r="G24">
@@ -16674,7 +16674,7 @@
         <v/>
       </c>
       <c r="F25" s="3">
-        <f>IF(A25="","",IF(D25=0,"",MAXIFS(Sales!C:C,Sales!D:D,A25)))</f>
+        <f>IF(A25="","",IF(D25=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A25)))</f>
         <v/>
       </c>
       <c r="G25">
@@ -16708,7 +16708,7 @@
         <v/>
       </c>
       <c r="F26" s="3">
-        <f>IF(A26="","",IF(D26=0,"",MAXIFS(Sales!C:C,Sales!D:D,A26)))</f>
+        <f>IF(A26="","",IF(D26=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A26)))</f>
         <v/>
       </c>
       <c r="G26">
@@ -16742,7 +16742,7 @@
         <v/>
       </c>
       <c r="F27" s="3">
-        <f>IF(A27="","",IF(D27=0,"",MAXIFS(Sales!C:C,Sales!D:D,A27)))</f>
+        <f>IF(A27="","",IF(D27=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A27)))</f>
         <v/>
       </c>
       <c r="G27">
@@ -16776,7 +16776,7 @@
         <v/>
       </c>
       <c r="F28" s="3">
-        <f>IF(A28="","",IF(D28=0,"",MAXIFS(Sales!C:C,Sales!D:D,A28)))</f>
+        <f>IF(A28="","",IF(D28=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A28)))</f>
         <v/>
       </c>
       <c r="G28">
@@ -16810,7 +16810,7 @@
         <v/>
       </c>
       <c r="F29" s="3">
-        <f>IF(A29="","",IF(D29=0,"",MAXIFS(Sales!C:C,Sales!D:D,A29)))</f>
+        <f>IF(A29="","",IF(D29=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A29)))</f>
         <v/>
       </c>
       <c r="G29">
@@ -16844,7 +16844,7 @@
         <v/>
       </c>
       <c r="F30" s="3">
-        <f>IF(A30="","",IF(D30=0,"",MAXIFS(Sales!C:C,Sales!D:D,A30)))</f>
+        <f>IF(A30="","",IF(D30=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A30)))</f>
         <v/>
       </c>
       <c r="G30">
@@ -16878,7 +16878,7 @@
         <v/>
       </c>
       <c r="F31" s="3">
-        <f>IF(A31="","",IF(D31=0,"",MAXIFS(Sales!C:C,Sales!D:D,A31)))</f>
+        <f>IF(A31="","",IF(D31=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A31)))</f>
         <v/>
       </c>
       <c r="G31">
@@ -16912,7 +16912,7 @@
         <v/>
       </c>
       <c r="F32" s="3">
-        <f>IF(A32="","",IF(D32=0,"",MAXIFS(Sales!C:C,Sales!D:D,A32)))</f>
+        <f>IF(A32="","",IF(D32=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A32)))</f>
         <v/>
       </c>
       <c r="G32">
@@ -16946,7 +16946,7 @@
         <v/>
       </c>
       <c r="F33" s="3">
-        <f>IF(A33="","",IF(D33=0,"",MAXIFS(Sales!C:C,Sales!D:D,A33)))</f>
+        <f>IF(A33="","",IF(D33=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A33)))</f>
         <v/>
       </c>
       <c r="G33">
@@ -16980,7 +16980,7 @@
         <v/>
       </c>
       <c r="F34" s="3">
-        <f>IF(A34="","",IF(D34=0,"",MAXIFS(Sales!C:C,Sales!D:D,A34)))</f>
+        <f>IF(A34="","",IF(D34=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A34)))</f>
         <v/>
       </c>
       <c r="G34">
@@ -17014,7 +17014,7 @@
         <v/>
       </c>
       <c r="F35" s="3">
-        <f>IF(A35="","",IF(D35=0,"",MAXIFS(Sales!C:C,Sales!D:D,A35)))</f>
+        <f>IF(A35="","",IF(D35=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A35)))</f>
         <v/>
       </c>
       <c r="G35">
@@ -17048,7 +17048,7 @@
         <v/>
       </c>
       <c r="F36" s="3">
-        <f>IF(A36="","",IF(D36=0,"",MAXIFS(Sales!C:C,Sales!D:D,A36)))</f>
+        <f>IF(A36="","",IF(D36=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A36)))</f>
         <v/>
       </c>
       <c r="G36">
@@ -17082,7 +17082,7 @@
         <v/>
       </c>
       <c r="F37" s="3">
-        <f>IF(A37="","",IF(D37=0,"",MAXIFS(Sales!C:C,Sales!D:D,A37)))</f>
+        <f>IF(A37="","",IF(D37=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A37)))</f>
         <v/>
       </c>
       <c r="G37">
@@ -17116,7 +17116,7 @@
         <v/>
       </c>
       <c r="F38" s="3">
-        <f>IF(A38="","",IF(D38=0,"",MAXIFS(Sales!C:C,Sales!D:D,A38)))</f>
+        <f>IF(A38="","",IF(D38=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A38)))</f>
         <v/>
       </c>
       <c r="G38">
@@ -17150,7 +17150,7 @@
         <v/>
       </c>
       <c r="F39" s="3">
-        <f>IF(A39="","",IF(D39=0,"",MAXIFS(Sales!C:C,Sales!D:D,A39)))</f>
+        <f>IF(A39="","",IF(D39=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A39)))</f>
         <v/>
       </c>
       <c r="G39">
@@ -17184,7 +17184,7 @@
         <v/>
       </c>
       <c r="F40" s="3">
-        <f>IF(A40="","",IF(D40=0,"",MAXIFS(Sales!C:C,Sales!D:D,A40)))</f>
+        <f>IF(A40="","",IF(D40=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A40)))</f>
         <v/>
       </c>
       <c r="G40">
@@ -17218,7 +17218,7 @@
         <v/>
       </c>
       <c r="F41" s="3">
-        <f>IF(A41="","",IF(D41=0,"",MAXIFS(Sales!C:C,Sales!D:D,A41)))</f>
+        <f>IF(A41="","",IF(D41=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A41)))</f>
         <v/>
       </c>
       <c r="G41">
@@ -17252,7 +17252,7 @@
         <v/>
       </c>
       <c r="F42" s="3">
-        <f>IF(A42="","",IF(D42=0,"",MAXIFS(Sales!C:C,Sales!D:D,A42)))</f>
+        <f>IF(A42="","",IF(D42=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A42)))</f>
         <v/>
       </c>
       <c r="G42">
@@ -17286,7 +17286,7 @@
         <v/>
       </c>
       <c r="F43" s="3">
-        <f>IF(A43="","",IF(D43=0,"",MAXIFS(Sales!C:C,Sales!D:D,A43)))</f>
+        <f>IF(A43="","",IF(D43=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A43)))</f>
         <v/>
       </c>
       <c r="G43">
@@ -17320,7 +17320,7 @@
         <v/>
       </c>
       <c r="F44" s="3">
-        <f>IF(A44="","",IF(D44=0,"",MAXIFS(Sales!C:C,Sales!D:D,A44)))</f>
+        <f>IF(A44="","",IF(D44=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A44)))</f>
         <v/>
       </c>
       <c r="G44">
@@ -17354,7 +17354,7 @@
         <v/>
       </c>
       <c r="F45" s="3">
-        <f>IF(A45="","",IF(D45=0,"",MAXIFS(Sales!C:C,Sales!D:D,A45)))</f>
+        <f>IF(A45="","",IF(D45=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A45)))</f>
         <v/>
       </c>
       <c r="G45">
@@ -17388,7 +17388,7 @@
         <v/>
       </c>
       <c r="F46" s="3">
-        <f>IF(A46="","",IF(D46=0,"",MAXIFS(Sales!C:C,Sales!D:D,A46)))</f>
+        <f>IF(A46="","",IF(D46=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A46)))</f>
         <v/>
       </c>
       <c r="G46">
@@ -17422,7 +17422,7 @@
         <v/>
       </c>
       <c r="F47" s="3">
-        <f>IF(A47="","",IF(D47=0,"",MAXIFS(Sales!C:C,Sales!D:D,A47)))</f>
+        <f>IF(A47="","",IF(D47=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A47)))</f>
         <v/>
       </c>
       <c r="G47">
@@ -17456,7 +17456,7 @@
         <v/>
       </c>
       <c r="F48" s="3">
-        <f>IF(A48="","",IF(D48=0,"",MAXIFS(Sales!C:C,Sales!D:D,A48)))</f>
+        <f>IF(A48="","",IF(D48=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A48)))</f>
         <v/>
       </c>
       <c r="G48">
@@ -17490,7 +17490,7 @@
         <v/>
       </c>
       <c r="F49" s="3">
-        <f>IF(A49="","",IF(D49=0,"",MAXIFS(Sales!C:C,Sales!D:D,A49)))</f>
+        <f>IF(A49="","",IF(D49=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A49)))</f>
         <v/>
       </c>
       <c r="G49">
@@ -17524,7 +17524,7 @@
         <v/>
       </c>
       <c r="F50" s="3">
-        <f>IF(A50="","",IF(D50=0,"",MAXIFS(Sales!C:C,Sales!D:D,A50)))</f>
+        <f>IF(A50="","",IF(D50=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A50)))</f>
         <v/>
       </c>
       <c r="G50">
@@ -17558,7 +17558,7 @@
         <v/>
       </c>
       <c r="F51" s="3">
-        <f>IF(A51="","",IF(D51=0,"",MAXIFS(Sales!C:C,Sales!D:D,A51)))</f>
+        <f>IF(A51="","",IF(D51=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A51)))</f>
         <v/>
       </c>
       <c r="G51">
@@ -17592,7 +17592,7 @@
         <v/>
       </c>
       <c r="F52" s="3">
-        <f>IF(A52="","",IF(D52=0,"",MAXIFS(Sales!C:C,Sales!D:D,A52)))</f>
+        <f>IF(A52="","",IF(D52=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A52)))</f>
         <v/>
       </c>
       <c r="G52">
@@ -17626,7 +17626,7 @@
         <v/>
       </c>
       <c r="F53" s="3">
-        <f>IF(A53="","",IF(D53=0,"",MAXIFS(Sales!C:C,Sales!D:D,A53)))</f>
+        <f>IF(A53="","",IF(D53=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A53)))</f>
         <v/>
       </c>
       <c r="G53">
@@ -17660,7 +17660,7 @@
         <v/>
       </c>
       <c r="F54" s="3">
-        <f>IF(A54="","",IF(D54=0,"",MAXIFS(Sales!C:C,Sales!D:D,A54)))</f>
+        <f>IF(A54="","",IF(D54=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A54)))</f>
         <v/>
       </c>
       <c r="G54">
@@ -17694,7 +17694,7 @@
         <v/>
       </c>
       <c r="F55" s="3">
-        <f>IF(A55="","",IF(D55=0,"",MAXIFS(Sales!C:C,Sales!D:D,A55)))</f>
+        <f>IF(A55="","",IF(D55=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A55)))</f>
         <v/>
       </c>
       <c r="G55">
@@ -17728,7 +17728,7 @@
         <v/>
       </c>
       <c r="F56" s="3">
-        <f>IF(A56="","",IF(D56=0,"",MAXIFS(Sales!C:C,Sales!D:D,A56)))</f>
+        <f>IF(A56="","",IF(D56=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A56)))</f>
         <v/>
       </c>
       <c r="G56">
@@ -17762,7 +17762,7 @@
         <v/>
       </c>
       <c r="F57" s="3">
-        <f>IF(A57="","",IF(D57=0,"",MAXIFS(Sales!C:C,Sales!D:D,A57)))</f>
+        <f>IF(A57="","",IF(D57=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A57)))</f>
         <v/>
       </c>
       <c r="G57">
@@ -17796,7 +17796,7 @@
         <v/>
       </c>
       <c r="F58" s="3">
-        <f>IF(A58="","",IF(D58=0,"",MAXIFS(Sales!C:C,Sales!D:D,A58)))</f>
+        <f>IF(A58="","",IF(D58=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A58)))</f>
         <v/>
       </c>
       <c r="G58">
@@ -17830,7 +17830,7 @@
         <v/>
       </c>
       <c r="F59" s="3">
-        <f>IF(A59="","",IF(D59=0,"",MAXIFS(Sales!C:C,Sales!D:D,A59)))</f>
+        <f>IF(A59="","",IF(D59=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A59)))</f>
         <v/>
       </c>
       <c r="G59">
@@ -17864,7 +17864,7 @@
         <v/>
       </c>
       <c r="F60" s="3">
-        <f>IF(A60="","",IF(D60=0,"",MAXIFS(Sales!C:C,Sales!D:D,A60)))</f>
+        <f>IF(A60="","",IF(D60=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A60)))</f>
         <v/>
       </c>
       <c r="G60">
@@ -17898,7 +17898,7 @@
         <v/>
       </c>
       <c r="F61" s="3">
-        <f>IF(A61="","",IF(D61=0,"",MAXIFS(Sales!C:C,Sales!D:D,A61)))</f>
+        <f>IF(A61="","",IF(D61=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A61)))</f>
         <v/>
       </c>
       <c r="G61">
@@ -17932,7 +17932,7 @@
         <v/>
       </c>
       <c r="F62" s="3">
-        <f>IF(A62="","",IF(D62=0,"",MAXIFS(Sales!C:C,Sales!D:D,A62)))</f>
+        <f>IF(A62="","",IF(D62=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A62)))</f>
         <v/>
       </c>
       <c r="G62">
@@ -17966,7 +17966,7 @@
         <v/>
       </c>
       <c r="F63" s="3">
-        <f>IF(A63="","",IF(D63=0,"",MAXIFS(Sales!C:C,Sales!D:D,A63)))</f>
+        <f>IF(A63="","",IF(D63=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A63)))</f>
         <v/>
       </c>
       <c r="G63">
@@ -18000,7 +18000,7 @@
         <v/>
       </c>
       <c r="F64" s="3">
-        <f>IF(A64="","",IF(D64=0,"",MAXIFS(Sales!C:C,Sales!D:D,A64)))</f>
+        <f>IF(A64="","",IF(D64=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A64)))</f>
         <v/>
       </c>
       <c r="G64">
@@ -18034,7 +18034,7 @@
         <v/>
       </c>
       <c r="F65" s="3">
-        <f>IF(A65="","",IF(D65=0,"",MAXIFS(Sales!C:C,Sales!D:D,A65)))</f>
+        <f>IF(A65="","",IF(D65=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A65)))</f>
         <v/>
       </c>
       <c r="G65">
@@ -18068,7 +18068,7 @@
         <v/>
       </c>
       <c r="F66" s="3">
-        <f>IF(A66="","",IF(D66=0,"",MAXIFS(Sales!C:C,Sales!D:D,A66)))</f>
+        <f>IF(A66="","",IF(D66=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A66)))</f>
         <v/>
       </c>
       <c r="G66">
@@ -18102,7 +18102,7 @@
         <v/>
       </c>
       <c r="F67" s="3">
-        <f>IF(A67="","",IF(D67=0,"",MAXIFS(Sales!C:C,Sales!D:D,A67)))</f>
+        <f>IF(A67="","",IF(D67=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A67)))</f>
         <v/>
       </c>
       <c r="G67">
@@ -18136,7 +18136,7 @@
         <v/>
       </c>
       <c r="F68" s="3">
-        <f>IF(A68="","",IF(D68=0,"",MAXIFS(Sales!C:C,Sales!D:D,A68)))</f>
+        <f>IF(A68="","",IF(D68=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A68)))</f>
         <v/>
       </c>
       <c r="G68">
@@ -18170,7 +18170,7 @@
         <v/>
       </c>
       <c r="F69" s="3">
-        <f>IF(A69="","",IF(D69=0,"",MAXIFS(Sales!C:C,Sales!D:D,A69)))</f>
+        <f>IF(A69="","",IF(D69=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A69)))</f>
         <v/>
       </c>
       <c r="G69">
@@ -18204,7 +18204,7 @@
         <v/>
       </c>
       <c r="F70" s="3">
-        <f>IF(A70="","",IF(D70=0,"",MAXIFS(Sales!C:C,Sales!D:D,A70)))</f>
+        <f>IF(A70="","",IF(D70=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A70)))</f>
         <v/>
       </c>
       <c r="G70">
@@ -18238,7 +18238,7 @@
         <v/>
       </c>
       <c r="F71" s="3">
-        <f>IF(A71="","",IF(D71=0,"",MAXIFS(Sales!C:C,Sales!D:D,A71)))</f>
+        <f>IF(A71="","",IF(D71=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A71)))</f>
         <v/>
       </c>
       <c r="G71">
@@ -18272,7 +18272,7 @@
         <v/>
       </c>
       <c r="F72" s="3">
-        <f>IF(A72="","",IF(D72=0,"",MAXIFS(Sales!C:C,Sales!D:D,A72)))</f>
+        <f>IF(A72="","",IF(D72=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A72)))</f>
         <v/>
       </c>
       <c r="G72">
@@ -18306,7 +18306,7 @@
         <v/>
       </c>
       <c r="F73" s="3">
-        <f>IF(A73="","",IF(D73=0,"",MAXIFS(Sales!C:C,Sales!D:D,A73)))</f>
+        <f>IF(A73="","",IF(D73=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A73)))</f>
         <v/>
       </c>
       <c r="G73">
@@ -18340,7 +18340,7 @@
         <v/>
       </c>
       <c r="F74" s="3">
-        <f>IF(A74="","",IF(D74=0,"",MAXIFS(Sales!C:C,Sales!D:D,A74)))</f>
+        <f>IF(A74="","",IF(D74=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A74)))</f>
         <v/>
       </c>
       <c r="G74">
@@ -18374,7 +18374,7 @@
         <v/>
       </c>
       <c r="F75" s="3">
-        <f>IF(A75="","",IF(D75=0,"",MAXIFS(Sales!C:C,Sales!D:D,A75)))</f>
+        <f>IF(A75="","",IF(D75=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A75)))</f>
         <v/>
       </c>
       <c r="G75">
@@ -18408,7 +18408,7 @@
         <v/>
       </c>
       <c r="F76" s="3">
-        <f>IF(A76="","",IF(D76=0,"",MAXIFS(Sales!C:C,Sales!D:D,A76)))</f>
+        <f>IF(A76="","",IF(D76=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A76)))</f>
         <v/>
       </c>
       <c r="G76">
@@ -18442,7 +18442,7 @@
         <v/>
       </c>
       <c r="F77" s="3">
-        <f>IF(A77="","",IF(D77=0,"",MAXIFS(Sales!C:C,Sales!D:D,A77)))</f>
+        <f>IF(A77="","",IF(D77=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A77)))</f>
         <v/>
       </c>
       <c r="G77">
@@ -18476,7 +18476,7 @@
         <v/>
       </c>
       <c r="F78" s="3">
-        <f>IF(A78="","",IF(D78=0,"",MAXIFS(Sales!C:C,Sales!D:D,A78)))</f>
+        <f>IF(A78="","",IF(D78=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A78)))</f>
         <v/>
       </c>
       <c r="G78">
@@ -18510,7 +18510,7 @@
         <v/>
       </c>
       <c r="F79" s="3">
-        <f>IF(A79="","",IF(D79=0,"",MAXIFS(Sales!C:C,Sales!D:D,A79)))</f>
+        <f>IF(A79="","",IF(D79=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A79)))</f>
         <v/>
       </c>
       <c r="G79">
@@ -18544,7 +18544,7 @@
         <v/>
       </c>
       <c r="F80" s="3">
-        <f>IF(A80="","",IF(D80=0,"",MAXIFS(Sales!C:C,Sales!D:D,A80)))</f>
+        <f>IF(A80="","",IF(D80=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A80)))</f>
         <v/>
       </c>
       <c r="G80">
@@ -18578,7 +18578,7 @@
         <v/>
       </c>
       <c r="F81" s="3">
-        <f>IF(A81="","",IF(D81=0,"",MAXIFS(Sales!C:C,Sales!D:D,A81)))</f>
+        <f>IF(A81="","",IF(D81=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A81)))</f>
         <v/>
       </c>
       <c r="G81">
@@ -18612,7 +18612,7 @@
         <v/>
       </c>
       <c r="F82" s="3">
-        <f>IF(A82="","",IF(D82=0,"",MAXIFS(Sales!C:C,Sales!D:D,A82)))</f>
+        <f>IF(A82="","",IF(D82=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A82)))</f>
         <v/>
       </c>
       <c r="G82">
@@ -18646,7 +18646,7 @@
         <v/>
       </c>
       <c r="F83" s="3">
-        <f>IF(A83="","",IF(D83=0,"",MAXIFS(Sales!C:C,Sales!D:D,A83)))</f>
+        <f>IF(A83="","",IF(D83=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A83)))</f>
         <v/>
       </c>
       <c r="G83">
@@ -18680,7 +18680,7 @@
         <v/>
       </c>
       <c r="F84" s="3">
-        <f>IF(A84="","",IF(D84=0,"",MAXIFS(Sales!C:C,Sales!D:D,A84)))</f>
+        <f>IF(A84="","",IF(D84=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A84)))</f>
         <v/>
       </c>
       <c r="G84">
@@ -18714,7 +18714,7 @@
         <v/>
       </c>
       <c r="F85" s="3">
-        <f>IF(A85="","",IF(D85=0,"",MAXIFS(Sales!C:C,Sales!D:D,A85)))</f>
+        <f>IF(A85="","",IF(D85=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A85)))</f>
         <v/>
       </c>
       <c r="G85">
@@ -18748,7 +18748,7 @@
         <v/>
       </c>
       <c r="F86" s="3">
-        <f>IF(A86="","",IF(D86=0,"",MAXIFS(Sales!C:C,Sales!D:D,A86)))</f>
+        <f>IF(A86="","",IF(D86=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A86)))</f>
         <v/>
       </c>
       <c r="G86">
@@ -18782,7 +18782,7 @@
         <v/>
       </c>
       <c r="F87" s="3">
-        <f>IF(A87="","",IF(D87=0,"",MAXIFS(Sales!C:C,Sales!D:D,A87)))</f>
+        <f>IF(A87="","",IF(D87=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A87)))</f>
         <v/>
       </c>
       <c r="G87">
@@ -18816,7 +18816,7 @@
         <v/>
       </c>
       <c r="F88" s="3">
-        <f>IF(A88="","",IF(D88=0,"",MAXIFS(Sales!C:C,Sales!D:D,A88)))</f>
+        <f>IF(A88="","",IF(D88=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A88)))</f>
         <v/>
       </c>
       <c r="G88">
@@ -18850,7 +18850,7 @@
         <v/>
       </c>
       <c r="F89" s="3">
-        <f>IF(A89="","",IF(D89=0,"",MAXIFS(Sales!C:C,Sales!D:D,A89)))</f>
+        <f>IF(A89="","",IF(D89=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A89)))</f>
         <v/>
       </c>
       <c r="G89">
@@ -18884,7 +18884,7 @@
         <v/>
       </c>
       <c r="F90" s="3">
-        <f>IF(A90="","",IF(D90=0,"",MAXIFS(Sales!C:C,Sales!D:D,A90)))</f>
+        <f>IF(A90="","",IF(D90=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A90)))</f>
         <v/>
       </c>
       <c r="G90">
@@ -18918,7 +18918,7 @@
         <v/>
       </c>
       <c r="F91" s="3">
-        <f>IF(A91="","",IF(D91=0,"",MAXIFS(Sales!C:C,Sales!D:D,A91)))</f>
+        <f>IF(A91="","",IF(D91=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A91)))</f>
         <v/>
       </c>
       <c r="G91">
@@ -18952,7 +18952,7 @@
         <v/>
       </c>
       <c r="F92" s="3">
-        <f>IF(A92="","",IF(D92=0,"",MAXIFS(Sales!C:C,Sales!D:D,A92)))</f>
+        <f>IF(A92="","",IF(D92=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A92)))</f>
         <v/>
       </c>
       <c r="G92">
@@ -18986,7 +18986,7 @@
         <v/>
       </c>
       <c r="F93" s="3">
-        <f>IF(A93="","",IF(D93=0,"",MAXIFS(Sales!C:C,Sales!D:D,A93)))</f>
+        <f>IF(A93="","",IF(D93=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A93)))</f>
         <v/>
       </c>
       <c r="G93">
@@ -19020,7 +19020,7 @@
         <v/>
       </c>
       <c r="F94" s="3">
-        <f>IF(A94="","",IF(D94=0,"",MAXIFS(Sales!C:C,Sales!D:D,A94)))</f>
+        <f>IF(A94="","",IF(D94=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A94)))</f>
         <v/>
       </c>
       <c r="G94">
@@ -19054,7 +19054,7 @@
         <v/>
       </c>
       <c r="F95" s="3">
-        <f>IF(A95="","",IF(D95=0,"",MAXIFS(Sales!C:C,Sales!D:D,A95)))</f>
+        <f>IF(A95="","",IF(D95=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A95)))</f>
         <v/>
       </c>
       <c r="G95">
@@ -19088,7 +19088,7 @@
         <v/>
       </c>
       <c r="F96" s="3">
-        <f>IF(A96="","",IF(D96=0,"",MAXIFS(Sales!C:C,Sales!D:D,A96)))</f>
+        <f>IF(A96="","",IF(D96=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A96)))</f>
         <v/>
       </c>
       <c r="G96">
@@ -19122,7 +19122,7 @@
         <v/>
       </c>
       <c r="F97" s="3">
-        <f>IF(A97="","",IF(D97=0,"",MAXIFS(Sales!C:C,Sales!D:D,A97)))</f>
+        <f>IF(A97="","",IF(D97=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A97)))</f>
         <v/>
       </c>
       <c r="G97">
@@ -19156,7 +19156,7 @@
         <v/>
       </c>
       <c r="F98" s="3">
-        <f>IF(A98="","",IF(D98=0,"",MAXIFS(Sales!C:C,Sales!D:D,A98)))</f>
+        <f>IF(A98="","",IF(D98=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A98)))</f>
         <v/>
       </c>
       <c r="G98">
@@ -19190,7 +19190,7 @@
         <v/>
       </c>
       <c r="F99" s="3">
-        <f>IF(A99="","",IF(D99=0,"",MAXIFS(Sales!C:C,Sales!D:D,A99)))</f>
+        <f>IF(A99="","",IF(D99=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A99)))</f>
         <v/>
       </c>
       <c r="G99">
@@ -19224,7 +19224,7 @@
         <v/>
       </c>
       <c r="F100" s="3">
-        <f>IF(A100="","",IF(D100=0,"",MAXIFS(Sales!C:C,Sales!D:D,A100)))</f>
+        <f>IF(A100="","",IF(D100=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A100)))</f>
         <v/>
       </c>
       <c r="G100">
@@ -19258,7 +19258,7 @@
         <v/>
       </c>
       <c r="F101" s="3">
-        <f>IF(A101="","",IF(D101=0,"",MAXIFS(Sales!C:C,Sales!D:D,A101)))</f>
+        <f>IF(A101="","",IF(D101=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A101)))</f>
         <v/>
       </c>
       <c r="G101">
@@ -19292,7 +19292,7 @@
         <v/>
       </c>
       <c r="F102" s="3">
-        <f>IF(A102="","",IF(D102=0,"",MAXIFS(Sales!C:C,Sales!D:D,A102)))</f>
+        <f>IF(A102="","",IF(D102=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A102)))</f>
         <v/>
       </c>
       <c r="G102">
@@ -19326,7 +19326,7 @@
         <v/>
       </c>
       <c r="F103" s="3">
-        <f>IF(A103="","",IF(D103=0,"",MAXIFS(Sales!C:C,Sales!D:D,A103)))</f>
+        <f>IF(A103="","",IF(D103=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A103)))</f>
         <v/>
       </c>
       <c r="G103">
@@ -19360,7 +19360,7 @@
         <v/>
       </c>
       <c r="F104" s="3">
-        <f>IF(A104="","",IF(D104=0,"",MAXIFS(Sales!C:C,Sales!D:D,A104)))</f>
+        <f>IF(A104="","",IF(D104=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A104)))</f>
         <v/>
       </c>
       <c r="G104">
@@ -19394,7 +19394,7 @@
         <v/>
       </c>
       <c r="F105" s="3">
-        <f>IF(A105="","",IF(D105=0,"",MAXIFS(Sales!C:C,Sales!D:D,A105)))</f>
+        <f>IF(A105="","",IF(D105=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A105)))</f>
         <v/>
       </c>
       <c r="G105">
@@ -19428,7 +19428,7 @@
         <v/>
       </c>
       <c r="F106" s="3">
-        <f>IF(A106="","",IF(D106=0,"",MAXIFS(Sales!C:C,Sales!D:D,A106)))</f>
+        <f>IF(A106="","",IF(D106=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A106)))</f>
         <v/>
       </c>
       <c r="G106">
@@ -19462,7 +19462,7 @@
         <v/>
       </c>
       <c r="F107" s="3">
-        <f>IF(A107="","",IF(D107=0,"",MAXIFS(Sales!C:C,Sales!D:D,A107)))</f>
+        <f>IF(A107="","",IF(D107=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A107)))</f>
         <v/>
       </c>
       <c r="G107">
@@ -19496,7 +19496,7 @@
         <v/>
       </c>
       <c r="F108" s="3">
-        <f>IF(A108="","",IF(D108=0,"",MAXIFS(Sales!C:C,Sales!D:D,A108)))</f>
+        <f>IF(A108="","",IF(D108=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A108)))</f>
         <v/>
       </c>
       <c r="G108">
@@ -19530,7 +19530,7 @@
         <v/>
       </c>
       <c r="F109" s="3">
-        <f>IF(A109="","",IF(D109=0,"",MAXIFS(Sales!C:C,Sales!D:D,A109)))</f>
+        <f>IF(A109="","",IF(D109=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A109)))</f>
         <v/>
       </c>
       <c r="G109">
@@ -19564,7 +19564,7 @@
         <v/>
       </c>
       <c r="F110" s="3">
-        <f>IF(A110="","",IF(D110=0,"",MAXIFS(Sales!C:C,Sales!D:D,A110)))</f>
+        <f>IF(A110="","",IF(D110=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A110)))</f>
         <v/>
       </c>
       <c r="G110">
@@ -19598,7 +19598,7 @@
         <v/>
       </c>
       <c r="F111" s="3">
-        <f>IF(A111="","",IF(D111=0,"",MAXIFS(Sales!C:C,Sales!D:D,A111)))</f>
+        <f>IF(A111="","",IF(D111=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A111)))</f>
         <v/>
       </c>
       <c r="G111">
@@ -19632,7 +19632,7 @@
         <v/>
       </c>
       <c r="F112" s="3">
-        <f>IF(A112="","",IF(D112=0,"",MAXIFS(Sales!C:C,Sales!D:D,A112)))</f>
+        <f>IF(A112="","",IF(D112=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A112)))</f>
         <v/>
       </c>
       <c r="G112">
@@ -19666,7 +19666,7 @@
         <v/>
       </c>
       <c r="F113" s="3">
-        <f>IF(A113="","",IF(D113=0,"",MAXIFS(Sales!C:C,Sales!D:D,A113)))</f>
+        <f>IF(A113="","",IF(D113=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A113)))</f>
         <v/>
       </c>
       <c r="G113">
@@ -19700,7 +19700,7 @@
         <v/>
       </c>
       <c r="F114" s="3">
-        <f>IF(A114="","",IF(D114=0,"",MAXIFS(Sales!C:C,Sales!D:D,A114)))</f>
+        <f>IF(A114="","",IF(D114=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A114)))</f>
         <v/>
       </c>
       <c r="G114">
@@ -19734,7 +19734,7 @@
         <v/>
       </c>
       <c r="F115" s="3">
-        <f>IF(A115="","",IF(D115=0,"",MAXIFS(Sales!C:C,Sales!D:D,A115)))</f>
+        <f>IF(A115="","",IF(D115=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A115)))</f>
         <v/>
       </c>
       <c r="G115">
@@ -19768,7 +19768,7 @@
         <v/>
       </c>
       <c r="F116" s="3">
-        <f>IF(A116="","",IF(D116=0,"",MAXIFS(Sales!C:C,Sales!D:D,A116)))</f>
+        <f>IF(A116="","",IF(D116=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A116)))</f>
         <v/>
       </c>
       <c r="G116">
@@ -19802,7 +19802,7 @@
         <v/>
       </c>
       <c r="F117" s="3">
-        <f>IF(A117="","",IF(D117=0,"",MAXIFS(Sales!C:C,Sales!D:D,A117)))</f>
+        <f>IF(A117="","",IF(D117=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A117)))</f>
         <v/>
       </c>
       <c r="G117">
@@ -19836,7 +19836,7 @@
         <v/>
       </c>
       <c r="F118" s="3">
-        <f>IF(A118="","",IF(D118=0,"",MAXIFS(Sales!C:C,Sales!D:D,A118)))</f>
+        <f>IF(A118="","",IF(D118=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A118)))</f>
         <v/>
       </c>
       <c r="G118">
@@ -19870,7 +19870,7 @@
         <v/>
       </c>
       <c r="F119" s="3">
-        <f>IF(A119="","",IF(D119=0,"",MAXIFS(Sales!C:C,Sales!D:D,A119)))</f>
+        <f>IF(A119="","",IF(D119=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A119)))</f>
         <v/>
       </c>
       <c r="G119">
@@ -19904,7 +19904,7 @@
         <v/>
       </c>
       <c r="F120" s="3">
-        <f>IF(A120="","",IF(D120=0,"",MAXIFS(Sales!C:C,Sales!D:D,A120)))</f>
+        <f>IF(A120="","",IF(D120=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A120)))</f>
         <v/>
       </c>
       <c r="G120">
@@ -19938,7 +19938,7 @@
         <v/>
       </c>
       <c r="F121" s="3">
-        <f>IF(A121="","",IF(D121=0,"",MAXIFS(Sales!C:C,Sales!D:D,A121)))</f>
+        <f>IF(A121="","",IF(D121=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A121)))</f>
         <v/>
       </c>
       <c r="G121">
@@ -19972,7 +19972,7 @@
         <v/>
       </c>
       <c r="F122" s="3">
-        <f>IF(A122="","",IF(D122=0,"",MAXIFS(Sales!C:C,Sales!D:D,A122)))</f>
+        <f>IF(A122="","",IF(D122=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A122)))</f>
         <v/>
       </c>
       <c r="G122">
@@ -20006,7 +20006,7 @@
         <v/>
       </c>
       <c r="F123" s="3">
-        <f>IF(A123="","",IF(D123=0,"",MAXIFS(Sales!C:C,Sales!D:D,A123)))</f>
+        <f>IF(A123="","",IF(D123=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A123)))</f>
         <v/>
       </c>
       <c r="G123">
@@ -20040,7 +20040,7 @@
         <v/>
       </c>
       <c r="F124" s="3">
-        <f>IF(A124="","",IF(D124=0,"",MAXIFS(Sales!C:C,Sales!D:D,A124)))</f>
+        <f>IF(A124="","",IF(D124=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A124)))</f>
         <v/>
       </c>
       <c r="G124">
@@ -20074,7 +20074,7 @@
         <v/>
       </c>
       <c r="F125" s="3">
-        <f>IF(A125="","",IF(D125=0,"",MAXIFS(Sales!C:C,Sales!D:D,A125)))</f>
+        <f>IF(A125="","",IF(D125=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A125)))</f>
         <v/>
       </c>
       <c r="G125">
@@ -20108,7 +20108,7 @@
         <v/>
       </c>
       <c r="F126" s="3">
-        <f>IF(A126="","",IF(D126=0,"",MAXIFS(Sales!C:C,Sales!D:D,A126)))</f>
+        <f>IF(A126="","",IF(D126=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A126)))</f>
         <v/>
       </c>
       <c r="G126">
@@ -20142,7 +20142,7 @@
         <v/>
       </c>
       <c r="F127" s="3">
-        <f>IF(A127="","",IF(D127=0,"",MAXIFS(Sales!C:C,Sales!D:D,A127)))</f>
+        <f>IF(A127="","",IF(D127=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A127)))</f>
         <v/>
       </c>
       <c r="G127">
@@ -20176,7 +20176,7 @@
         <v/>
       </c>
       <c r="F128" s="3">
-        <f>IF(A128="","",IF(D128=0,"",MAXIFS(Sales!C:C,Sales!D:D,A128)))</f>
+        <f>IF(A128="","",IF(D128=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A128)))</f>
         <v/>
       </c>
       <c r="G128">
@@ -20210,7 +20210,7 @@
         <v/>
       </c>
       <c r="F129" s="3">
-        <f>IF(A129="","",IF(D129=0,"",MAXIFS(Sales!C:C,Sales!D:D,A129)))</f>
+        <f>IF(A129="","",IF(D129=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A129)))</f>
         <v/>
       </c>
       <c r="G129">
@@ -20244,7 +20244,7 @@
         <v/>
       </c>
       <c r="F130" s="3">
-        <f>IF(A130="","",IF(D130=0,"",MAXIFS(Sales!C:C,Sales!D:D,A130)))</f>
+        <f>IF(A130="","",IF(D130=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A130)))</f>
         <v/>
       </c>
       <c r="G130">
@@ -20278,7 +20278,7 @@
         <v/>
       </c>
       <c r="F131" s="3">
-        <f>IF(A131="","",IF(D131=0,"",MAXIFS(Sales!C:C,Sales!D:D,A131)))</f>
+        <f>IF(A131="","",IF(D131=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A131)))</f>
         <v/>
       </c>
       <c r="G131">
@@ -20312,7 +20312,7 @@
         <v/>
       </c>
       <c r="F132" s="3">
-        <f>IF(A132="","",IF(D132=0,"",MAXIFS(Sales!C:C,Sales!D:D,A132)))</f>
+        <f>IF(A132="","",IF(D132=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A132)))</f>
         <v/>
       </c>
       <c r="G132">
@@ -20346,7 +20346,7 @@
         <v/>
       </c>
       <c r="F133" s="3">
-        <f>IF(A133="","",IF(D133=0,"",MAXIFS(Sales!C:C,Sales!D:D,A133)))</f>
+        <f>IF(A133="","",IF(D133=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A133)))</f>
         <v/>
       </c>
       <c r="G133">
@@ -20380,7 +20380,7 @@
         <v/>
       </c>
       <c r="F134" s="3">
-        <f>IF(A134="","",IF(D134=0,"",MAXIFS(Sales!C:C,Sales!D:D,A134)))</f>
+        <f>IF(A134="","",IF(D134=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A134)))</f>
         <v/>
       </c>
       <c r="G134">
@@ -20414,7 +20414,7 @@
         <v/>
       </c>
       <c r="F135" s="3">
-        <f>IF(A135="","",IF(D135=0,"",MAXIFS(Sales!C:C,Sales!D:D,A135)))</f>
+        <f>IF(A135="","",IF(D135=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A135)))</f>
         <v/>
       </c>
       <c r="G135">
@@ -20448,7 +20448,7 @@
         <v/>
       </c>
       <c r="F136" s="3">
-        <f>IF(A136="","",IF(D136=0,"",MAXIFS(Sales!C:C,Sales!D:D,A136)))</f>
+        <f>IF(A136="","",IF(D136=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A136)))</f>
         <v/>
       </c>
       <c r="G136">
@@ -20482,7 +20482,7 @@
         <v/>
       </c>
       <c r="F137" s="3">
-        <f>IF(A137="","",IF(D137=0,"",MAXIFS(Sales!C:C,Sales!D:D,A137)))</f>
+        <f>IF(A137="","",IF(D137=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A137)))</f>
         <v/>
       </c>
       <c r="G137">
@@ -20516,7 +20516,7 @@
         <v/>
       </c>
       <c r="F138" s="3">
-        <f>IF(A138="","",IF(D138=0,"",MAXIFS(Sales!C:C,Sales!D:D,A138)))</f>
+        <f>IF(A138="","",IF(D138=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A138)))</f>
         <v/>
       </c>
       <c r="G138">
@@ -20550,7 +20550,7 @@
         <v/>
       </c>
       <c r="F139" s="3">
-        <f>IF(A139="","",IF(D139=0,"",MAXIFS(Sales!C:C,Sales!D:D,A139)))</f>
+        <f>IF(A139="","",IF(D139=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A139)))</f>
         <v/>
       </c>
       <c r="G139">
@@ -20584,7 +20584,7 @@
         <v/>
       </c>
       <c r="F140" s="3">
-        <f>IF(A140="","",IF(D140=0,"",MAXIFS(Sales!C:C,Sales!D:D,A140)))</f>
+        <f>IF(A140="","",IF(D140=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A140)))</f>
         <v/>
       </c>
       <c r="G140">
@@ -20618,7 +20618,7 @@
         <v/>
       </c>
       <c r="F141" s="3">
-        <f>IF(A141="","",IF(D141=0,"",MAXIFS(Sales!C:C,Sales!D:D,A141)))</f>
+        <f>IF(A141="","",IF(D141=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A141)))</f>
         <v/>
       </c>
       <c r="G141">
@@ -20652,7 +20652,7 @@
         <v/>
       </c>
       <c r="F142" s="3">
-        <f>IF(A142="","",IF(D142=0,"",MAXIFS(Sales!C:C,Sales!D:D,A142)))</f>
+        <f>IF(A142="","",IF(D142=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A142)))</f>
         <v/>
       </c>
       <c r="G142">
@@ -20686,7 +20686,7 @@
         <v/>
       </c>
       <c r="F143" s="3">
-        <f>IF(A143="","",IF(D143=0,"",MAXIFS(Sales!C:C,Sales!D:D,A143)))</f>
+        <f>IF(A143="","",IF(D143=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A143)))</f>
         <v/>
       </c>
       <c r="G143">
@@ -20720,7 +20720,7 @@
         <v/>
       </c>
       <c r="F144" s="3">
-        <f>IF(A144="","",IF(D144=0,"",MAXIFS(Sales!C:C,Sales!D:D,A144)))</f>
+        <f>IF(A144="","",IF(D144=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A144)))</f>
         <v/>
       </c>
       <c r="G144">
@@ -20754,7 +20754,7 @@
         <v/>
       </c>
       <c r="F145" s="3">
-        <f>IF(A145="","",IF(D145=0,"",MAXIFS(Sales!C:C,Sales!D:D,A145)))</f>
+        <f>IF(A145="","",IF(D145=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A145)))</f>
         <v/>
       </c>
       <c r="G145">
@@ -20788,7 +20788,7 @@
         <v/>
       </c>
       <c r="F146" s="3">
-        <f>IF(A146="","",IF(D146=0,"",MAXIFS(Sales!C:C,Sales!D:D,A146)))</f>
+        <f>IF(A146="","",IF(D146=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A146)))</f>
         <v/>
       </c>
       <c r="G146">
@@ -20822,7 +20822,7 @@
         <v/>
       </c>
       <c r="F147" s="3">
-        <f>IF(A147="","",IF(D147=0,"",MAXIFS(Sales!C:C,Sales!D:D,A147)))</f>
+        <f>IF(A147="","",IF(D147=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A147)))</f>
         <v/>
       </c>
       <c r="G147">
@@ -20856,7 +20856,7 @@
         <v/>
       </c>
       <c r="F148" s="3">
-        <f>IF(A148="","",IF(D148=0,"",MAXIFS(Sales!C:C,Sales!D:D,A148)))</f>
+        <f>IF(A148="","",IF(D148=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A148)))</f>
         <v/>
       </c>
       <c r="G148">
@@ -20890,7 +20890,7 @@
         <v/>
       </c>
       <c r="F149" s="3">
-        <f>IF(A149="","",IF(D149=0,"",MAXIFS(Sales!C:C,Sales!D:D,A149)))</f>
+        <f>IF(A149="","",IF(D149=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A149)))</f>
         <v/>
       </c>
       <c r="G149">
@@ -20924,7 +20924,7 @@
         <v/>
       </c>
       <c r="F150" s="3">
-        <f>IF(A150="","",IF(D150=0,"",MAXIFS(Sales!C:C,Sales!D:D,A150)))</f>
+        <f>IF(A150="","",IF(D150=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A150)))</f>
         <v/>
       </c>
       <c r="G150">
@@ -20958,7 +20958,7 @@
         <v/>
       </c>
       <c r="F151" s="3">
-        <f>IF(A151="","",IF(D151=0,"",MAXIFS(Sales!C:C,Sales!D:D,A151)))</f>
+        <f>IF(A151="","",IF(D151=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A151)))</f>
         <v/>
       </c>
       <c r="G151">
@@ -20992,7 +20992,7 @@
         <v/>
       </c>
       <c r="F152" s="3">
-        <f>IF(A152="","",IF(D152=0,"",MAXIFS(Sales!C:C,Sales!D:D,A152)))</f>
+        <f>IF(A152="","",IF(D152=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A152)))</f>
         <v/>
       </c>
       <c r="G152">
@@ -21026,7 +21026,7 @@
         <v/>
       </c>
       <c r="F153" s="3">
-        <f>IF(A153="","",IF(D153=0,"",MAXIFS(Sales!C:C,Sales!D:D,A153)))</f>
+        <f>IF(A153="","",IF(D153=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A153)))</f>
         <v/>
       </c>
       <c r="G153">
@@ -21060,7 +21060,7 @@
         <v/>
       </c>
       <c r="F154" s="3">
-        <f>IF(A154="","",IF(D154=0,"",MAXIFS(Sales!C:C,Sales!D:D,A154)))</f>
+        <f>IF(A154="","",IF(D154=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A154)))</f>
         <v/>
       </c>
       <c r="G154">
@@ -21094,7 +21094,7 @@
         <v/>
       </c>
       <c r="F155" s="3">
-        <f>IF(A155="","",IF(D155=0,"",MAXIFS(Sales!C:C,Sales!D:D,A155)))</f>
+        <f>IF(A155="","",IF(D155=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A155)))</f>
         <v/>
       </c>
       <c r="G155">
@@ -21128,7 +21128,7 @@
         <v/>
       </c>
       <c r="F156" s="3">
-        <f>IF(A156="","",IF(D156=0,"",MAXIFS(Sales!C:C,Sales!D:D,A156)))</f>
+        <f>IF(A156="","",IF(D156=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A156)))</f>
         <v/>
       </c>
       <c r="G156">
@@ -21162,7 +21162,7 @@
         <v/>
       </c>
       <c r="F157" s="3">
-        <f>IF(A157="","",IF(D157=0,"",MAXIFS(Sales!C:C,Sales!D:D,A157)))</f>
+        <f>IF(A157="","",IF(D157=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A157)))</f>
         <v/>
       </c>
       <c r="G157">
@@ -21196,7 +21196,7 @@
         <v/>
       </c>
       <c r="F158" s="3">
-        <f>IF(A158="","",IF(D158=0,"",MAXIFS(Sales!C:C,Sales!D:D,A158)))</f>
+        <f>IF(A158="","",IF(D158=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A158)))</f>
         <v/>
       </c>
       <c r="G158">
@@ -21230,7 +21230,7 @@
         <v/>
       </c>
       <c r="F159" s="3">
-        <f>IF(A159="","",IF(D159=0,"",MAXIFS(Sales!C:C,Sales!D:D,A159)))</f>
+        <f>IF(A159="","",IF(D159=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A159)))</f>
         <v/>
       </c>
       <c r="G159">
@@ -21264,7 +21264,7 @@
         <v/>
       </c>
       <c r="F160" s="3">
-        <f>IF(A160="","",IF(D160=0,"",MAXIFS(Sales!C:C,Sales!D:D,A160)))</f>
+        <f>IF(A160="","",IF(D160=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A160)))</f>
         <v/>
       </c>
       <c r="G160">
@@ -21298,7 +21298,7 @@
         <v/>
       </c>
       <c r="F161" s="3">
-        <f>IF(A161="","",IF(D161=0,"",MAXIFS(Sales!C:C,Sales!D:D,A161)))</f>
+        <f>IF(A161="","",IF(D161=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A161)))</f>
         <v/>
       </c>
       <c r="G161">
@@ -21332,7 +21332,7 @@
         <v/>
       </c>
       <c r="F162" s="3">
-        <f>IF(A162="","",IF(D162=0,"",MAXIFS(Sales!C:C,Sales!D:D,A162)))</f>
+        <f>IF(A162="","",IF(D162=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A162)))</f>
         <v/>
       </c>
       <c r="G162">
@@ -21366,7 +21366,7 @@
         <v/>
       </c>
       <c r="F163" s="3">
-        <f>IF(A163="","",IF(D163=0,"",MAXIFS(Sales!C:C,Sales!D:D,A163)))</f>
+        <f>IF(A163="","",IF(D163=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A163)))</f>
         <v/>
       </c>
       <c r="G163">
@@ -21400,7 +21400,7 @@
         <v/>
       </c>
       <c r="F164" s="3">
-        <f>IF(A164="","",IF(D164=0,"",MAXIFS(Sales!C:C,Sales!D:D,A164)))</f>
+        <f>IF(A164="","",IF(D164=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A164)))</f>
         <v/>
       </c>
       <c r="G164">
@@ -21434,7 +21434,7 @@
         <v/>
       </c>
       <c r="F165" s="3">
-        <f>IF(A165="","",IF(D165=0,"",MAXIFS(Sales!C:C,Sales!D:D,A165)))</f>
+        <f>IF(A165="","",IF(D165=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A165)))</f>
         <v/>
       </c>
       <c r="G165">
@@ -21468,7 +21468,7 @@
         <v/>
       </c>
       <c r="F166" s="3">
-        <f>IF(A166="","",IF(D166=0,"",MAXIFS(Sales!C:C,Sales!D:D,A166)))</f>
+        <f>IF(A166="","",IF(D166=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A166)))</f>
         <v/>
       </c>
       <c r="G166">
@@ -21502,7 +21502,7 @@
         <v/>
       </c>
       <c r="F167" s="3">
-        <f>IF(A167="","",IF(D167=0,"",MAXIFS(Sales!C:C,Sales!D:D,A167)))</f>
+        <f>IF(A167="","",IF(D167=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A167)))</f>
         <v/>
       </c>
       <c r="G167">
@@ -21536,7 +21536,7 @@
         <v/>
       </c>
       <c r="F168" s="3">
-        <f>IF(A168="","",IF(D168=0,"",MAXIFS(Sales!C:C,Sales!D:D,A168)))</f>
+        <f>IF(A168="","",IF(D168=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A168)))</f>
         <v/>
       </c>
       <c r="G168">
@@ -21570,7 +21570,7 @@
         <v/>
       </c>
       <c r="F169" s="3">
-        <f>IF(A169="","",IF(D169=0,"",MAXIFS(Sales!C:C,Sales!D:D,A169)))</f>
+        <f>IF(A169="","",IF(D169=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A169)))</f>
         <v/>
       </c>
       <c r="G169">
@@ -21604,7 +21604,7 @@
         <v/>
       </c>
       <c r="F170" s="3">
-        <f>IF(A170="","",IF(D170=0,"",MAXIFS(Sales!C:C,Sales!D:D,A170)))</f>
+        <f>IF(A170="","",IF(D170=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A170)))</f>
         <v/>
       </c>
       <c r="G170">
@@ -21638,7 +21638,7 @@
         <v/>
       </c>
       <c r="F171" s="3">
-        <f>IF(A171="","",IF(D171=0,"",MAXIFS(Sales!C:C,Sales!D:D,A171)))</f>
+        <f>IF(A171="","",IF(D171=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A171)))</f>
         <v/>
       </c>
       <c r="G171">
@@ -21672,7 +21672,7 @@
         <v/>
       </c>
       <c r="F172" s="3">
-        <f>IF(A172="","",IF(D172=0,"",MAXIFS(Sales!C:C,Sales!D:D,A172)))</f>
+        <f>IF(A172="","",IF(D172=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A172)))</f>
         <v/>
       </c>
       <c r="G172">
@@ -21706,7 +21706,7 @@
         <v/>
       </c>
       <c r="F173" s="3">
-        <f>IF(A173="","",IF(D173=0,"",MAXIFS(Sales!C:C,Sales!D:D,A173)))</f>
+        <f>IF(A173="","",IF(D173=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A173)))</f>
         <v/>
       </c>
       <c r="G173">
@@ -21740,7 +21740,7 @@
         <v/>
       </c>
       <c r="F174" s="3">
-        <f>IF(A174="","",IF(D174=0,"",MAXIFS(Sales!C:C,Sales!D:D,A174)))</f>
+        <f>IF(A174="","",IF(D174=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A174)))</f>
         <v/>
       </c>
       <c r="G174">
@@ -21774,7 +21774,7 @@
         <v/>
       </c>
       <c r="F175" s="3">
-        <f>IF(A175="","",IF(D175=0,"",MAXIFS(Sales!C:C,Sales!D:D,A175)))</f>
+        <f>IF(A175="","",IF(D175=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A175)))</f>
         <v/>
       </c>
       <c r="G175">
@@ -21808,7 +21808,7 @@
         <v/>
       </c>
       <c r="F176" s="3">
-        <f>IF(A176="","",IF(D176=0,"",MAXIFS(Sales!C:C,Sales!D:D,A176)))</f>
+        <f>IF(A176="","",IF(D176=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A176)))</f>
         <v/>
       </c>
       <c r="G176">
@@ -21842,7 +21842,7 @@
         <v/>
       </c>
       <c r="F177" s="3">
-        <f>IF(A177="","",IF(D177=0,"",MAXIFS(Sales!C:C,Sales!D:D,A177)))</f>
+        <f>IF(A177="","",IF(D177=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A177)))</f>
         <v/>
       </c>
       <c r="G177">
@@ -21876,7 +21876,7 @@
         <v/>
       </c>
       <c r="F178" s="3">
-        <f>IF(A178="","",IF(D178=0,"",MAXIFS(Sales!C:C,Sales!D:D,A178)))</f>
+        <f>IF(A178="","",IF(D178=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A178)))</f>
         <v/>
       </c>
       <c r="G178">
@@ -21910,7 +21910,7 @@
         <v/>
       </c>
       <c r="F179" s="3">
-        <f>IF(A179="","",IF(D179=0,"",MAXIFS(Sales!C:C,Sales!D:D,A179)))</f>
+        <f>IF(A179="","",IF(D179=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A179)))</f>
         <v/>
       </c>
       <c r="G179">
@@ -21944,7 +21944,7 @@
         <v/>
       </c>
       <c r="F180" s="3">
-        <f>IF(A180="","",IF(D180=0,"",MAXIFS(Sales!C:C,Sales!D:D,A180)))</f>
+        <f>IF(A180="","",IF(D180=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A180)))</f>
         <v/>
       </c>
       <c r="G180">
@@ -21978,7 +21978,7 @@
         <v/>
       </c>
       <c r="F181" s="3">
-        <f>IF(A181="","",IF(D181=0,"",MAXIFS(Sales!C:C,Sales!D:D,A181)))</f>
+        <f>IF(A181="","",IF(D181=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A181)))</f>
         <v/>
       </c>
       <c r="G181">
@@ -22012,7 +22012,7 @@
         <v/>
       </c>
       <c r="F182" s="3">
-        <f>IF(A182="","",IF(D182=0,"",MAXIFS(Sales!C:C,Sales!D:D,A182)))</f>
+        <f>IF(A182="","",IF(D182=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A182)))</f>
         <v/>
       </c>
       <c r="G182">
@@ -22046,7 +22046,7 @@
         <v/>
       </c>
       <c r="F183" s="3">
-        <f>IF(A183="","",IF(D183=0,"",MAXIFS(Sales!C:C,Sales!D:D,A183)))</f>
+        <f>IF(A183="","",IF(D183=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A183)))</f>
         <v/>
       </c>
       <c r="G183">
@@ -22080,7 +22080,7 @@
         <v/>
       </c>
       <c r="F184" s="3">
-        <f>IF(A184="","",IF(D184=0,"",MAXIFS(Sales!C:C,Sales!D:D,A184)))</f>
+        <f>IF(A184="","",IF(D184=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A184)))</f>
         <v/>
       </c>
       <c r="G184">
@@ -22114,7 +22114,7 @@
         <v/>
       </c>
       <c r="F185" s="3">
-        <f>IF(A185="","",IF(D185=0,"",MAXIFS(Sales!C:C,Sales!D:D,A185)))</f>
+        <f>IF(A185="","",IF(D185=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A185)))</f>
         <v/>
       </c>
       <c r="G185">
@@ -22148,7 +22148,7 @@
         <v/>
       </c>
       <c r="F186" s="3">
-        <f>IF(A186="","",IF(D186=0,"",MAXIFS(Sales!C:C,Sales!D:D,A186)))</f>
+        <f>IF(A186="","",IF(D186=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A186)))</f>
         <v/>
       </c>
       <c r="G186">
@@ -22182,7 +22182,7 @@
         <v/>
       </c>
       <c r="F187" s="3">
-        <f>IF(A187="","",IF(D187=0,"",MAXIFS(Sales!C:C,Sales!D:D,A187)))</f>
+        <f>IF(A187="","",IF(D187=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A187)))</f>
         <v/>
       </c>
       <c r="G187">
@@ -22216,7 +22216,7 @@
         <v/>
       </c>
       <c r="F188" s="3">
-        <f>IF(A188="","",IF(D188=0,"",MAXIFS(Sales!C:C,Sales!D:D,A188)))</f>
+        <f>IF(A188="","",IF(D188=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A188)))</f>
         <v/>
       </c>
       <c r="G188">
@@ -22250,7 +22250,7 @@
         <v/>
       </c>
       <c r="F189" s="3">
-        <f>IF(A189="","",IF(D189=0,"",MAXIFS(Sales!C:C,Sales!D:D,A189)))</f>
+        <f>IF(A189="","",IF(D189=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A189)))</f>
         <v/>
       </c>
       <c r="G189">
@@ -22284,7 +22284,7 @@
         <v/>
       </c>
       <c r="F190" s="3">
-        <f>IF(A190="","",IF(D190=0,"",MAXIFS(Sales!C:C,Sales!D:D,A190)))</f>
+        <f>IF(A190="","",IF(D190=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A190)))</f>
         <v/>
       </c>
       <c r="G190">
@@ -22318,7 +22318,7 @@
         <v/>
       </c>
       <c r="F191" s="3">
-        <f>IF(A191="","",IF(D191=0,"",MAXIFS(Sales!C:C,Sales!D:D,A191)))</f>
+        <f>IF(A191="","",IF(D191=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A191)))</f>
         <v/>
       </c>
       <c r="G191">
@@ -22352,7 +22352,7 @@
         <v/>
       </c>
       <c r="F192" s="3">
-        <f>IF(A192="","",IF(D192=0,"",MAXIFS(Sales!C:C,Sales!D:D,A192)))</f>
+        <f>IF(A192="","",IF(D192=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A192)))</f>
         <v/>
       </c>
       <c r="G192">
@@ -22386,7 +22386,7 @@
         <v/>
       </c>
       <c r="F193" s="3">
-        <f>IF(A193="","",IF(D193=0,"",MAXIFS(Sales!C:C,Sales!D:D,A193)))</f>
+        <f>IF(A193="","",IF(D193=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A193)))</f>
         <v/>
       </c>
       <c r="G193">
@@ -22420,7 +22420,7 @@
         <v/>
       </c>
       <c r="F194" s="3">
-        <f>IF(A194="","",IF(D194=0,"",MAXIFS(Sales!C:C,Sales!D:D,A194)))</f>
+        <f>IF(A194="","",IF(D194=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A194)))</f>
         <v/>
       </c>
       <c r="G194">
@@ -22454,7 +22454,7 @@
         <v/>
       </c>
       <c r="F195" s="3">
-        <f>IF(A195="","",IF(D195=0,"",MAXIFS(Sales!C:C,Sales!D:D,A195)))</f>
+        <f>IF(A195="","",IF(D195=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A195)))</f>
         <v/>
       </c>
       <c r="G195">
@@ -22488,7 +22488,7 @@
         <v/>
       </c>
       <c r="F196" s="3">
-        <f>IF(A196="","",IF(D196=0,"",MAXIFS(Sales!C:C,Sales!D:D,A196)))</f>
+        <f>IF(A196="","",IF(D196=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A196)))</f>
         <v/>
       </c>
       <c r="G196">
@@ -22522,7 +22522,7 @@
         <v/>
       </c>
       <c r="F197" s="3">
-        <f>IF(A197="","",IF(D197=0,"",MAXIFS(Sales!C:C,Sales!D:D,A197)))</f>
+        <f>IF(A197="","",IF(D197=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A197)))</f>
         <v/>
       </c>
       <c r="G197">
@@ -22556,7 +22556,7 @@
         <v/>
       </c>
       <c r="F198" s="3">
-        <f>IF(A198="","",IF(D198=0,"",MAXIFS(Sales!C:C,Sales!D:D,A198)))</f>
+        <f>IF(A198="","",IF(D198=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A198)))</f>
         <v/>
       </c>
       <c r="G198">
@@ -22590,7 +22590,7 @@
         <v/>
       </c>
       <c r="F199" s="3">
-        <f>IF(A199="","",IF(D199=0,"",MAXIFS(Sales!C:C,Sales!D:D,A199)))</f>
+        <f>IF(A199="","",IF(D199=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A199)))</f>
         <v/>
       </c>
       <c r="G199">
@@ -22624,7 +22624,7 @@
         <v/>
       </c>
       <c r="F200" s="3">
-        <f>IF(A200="","",IF(D200=0,"",MAXIFS(Sales!C:C,Sales!D:D,A200)))</f>
+        <f>IF(A200="","",IF(D200=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A200)))</f>
         <v/>
       </c>
       <c r="G200">
@@ -22658,7 +22658,7 @@
         <v/>
       </c>
       <c r="F201" s="3">
-        <f>IF(A201="","",IF(D201=0,"",MAXIFS(Sales!C:C,Sales!D:D,A201)))</f>
+        <f>IF(A201="","",IF(D201=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A201)))</f>
         <v/>
       </c>
       <c r="G201">
@@ -22692,7 +22692,7 @@
         <v/>
       </c>
       <c r="F202" s="3">
-        <f>IF(A202="","",IF(D202=0,"",MAXIFS(Sales!C:C,Sales!D:D,A202)))</f>
+        <f>IF(A202="","",IF(D202=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A202)))</f>
         <v/>
       </c>
       <c r="G202">
@@ -22726,7 +22726,7 @@
         <v/>
       </c>
       <c r="F203" s="3">
-        <f>IF(A203="","",IF(D203=0,"",MAXIFS(Sales!C:C,Sales!D:D,A203)))</f>
+        <f>IF(A203="","",IF(D203=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A203)))</f>
         <v/>
       </c>
       <c r="G203">
@@ -22760,7 +22760,7 @@
         <v/>
       </c>
       <c r="F204" s="3">
-        <f>IF(A204="","",IF(D204=0,"",MAXIFS(Sales!C:C,Sales!D:D,A204)))</f>
+        <f>IF(A204="","",IF(D204=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A204)))</f>
         <v/>
       </c>
       <c r="G204">
@@ -22794,7 +22794,7 @@
         <v/>
       </c>
       <c r="F205" s="3">
-        <f>IF(A205="","",IF(D205=0,"",MAXIFS(Sales!C:C,Sales!D:D,A205)))</f>
+        <f>IF(A205="","",IF(D205=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A205)))</f>
         <v/>
       </c>
       <c r="G205">
@@ -22828,7 +22828,7 @@
         <v/>
       </c>
       <c r="F206" s="3">
-        <f>IF(A206="","",IF(D206=0,"",MAXIFS(Sales!C:C,Sales!D:D,A206)))</f>
+        <f>IF(A206="","",IF(D206=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A206)))</f>
         <v/>
       </c>
       <c r="G206">
@@ -22862,7 +22862,7 @@
         <v/>
       </c>
       <c r="F207" s="3">
-        <f>IF(A207="","",IF(D207=0,"",MAXIFS(Sales!C:C,Sales!D:D,A207)))</f>
+        <f>IF(A207="","",IF(D207=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A207)))</f>
         <v/>
       </c>
       <c r="G207">
@@ -22896,7 +22896,7 @@
         <v/>
       </c>
       <c r="F208" s="3">
-        <f>IF(A208="","",IF(D208=0,"",MAXIFS(Sales!C:C,Sales!D:D,A208)))</f>
+        <f>IF(A208="","",IF(D208=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A208)))</f>
         <v/>
       </c>
       <c r="G208">
@@ -22930,7 +22930,7 @@
         <v/>
       </c>
       <c r="F209" s="3">
-        <f>IF(A209="","",IF(D209=0,"",MAXIFS(Sales!C:C,Sales!D:D,A209)))</f>
+        <f>IF(A209="","",IF(D209=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A209)))</f>
         <v/>
       </c>
       <c r="G209">
@@ -22964,7 +22964,7 @@
         <v/>
       </c>
       <c r="F210" s="3">
-        <f>IF(A210="","",IF(D210=0,"",MAXIFS(Sales!C:C,Sales!D:D,A210)))</f>
+        <f>IF(A210="","",IF(D210=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A210)))</f>
         <v/>
       </c>
       <c r="G210">
@@ -22998,7 +22998,7 @@
         <v/>
       </c>
       <c r="F211" s="3">
-        <f>IF(A211="","",IF(D211=0,"",MAXIFS(Sales!C:C,Sales!D:D,A211)))</f>
+        <f>IF(A211="","",IF(D211=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A211)))</f>
         <v/>
       </c>
       <c r="G211">
@@ -23032,7 +23032,7 @@
         <v/>
       </c>
       <c r="F212" s="3">
-        <f>IF(A212="","",IF(D212=0,"",MAXIFS(Sales!C:C,Sales!D:D,A212)))</f>
+        <f>IF(A212="","",IF(D212=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A212)))</f>
         <v/>
       </c>
       <c r="G212">
@@ -23066,7 +23066,7 @@
         <v/>
       </c>
       <c r="F213" s="3">
-        <f>IF(A213="","",IF(D213=0,"",MAXIFS(Sales!C:C,Sales!D:D,A213)))</f>
+        <f>IF(A213="","",IF(D213=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A213)))</f>
         <v/>
       </c>
       <c r="G213">
@@ -23100,7 +23100,7 @@
         <v/>
       </c>
       <c r="F214" s="3">
-        <f>IF(A214="","",IF(D214=0,"",MAXIFS(Sales!C:C,Sales!D:D,A214)))</f>
+        <f>IF(A214="","",IF(D214=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A214)))</f>
         <v/>
       </c>
       <c r="G214">
@@ -23134,7 +23134,7 @@
         <v/>
       </c>
       <c r="F215" s="3">
-        <f>IF(A215="","",IF(D215=0,"",MAXIFS(Sales!C:C,Sales!D:D,A215)))</f>
+        <f>IF(A215="","",IF(D215=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A215)))</f>
         <v/>
       </c>
       <c r="G215">
@@ -23168,7 +23168,7 @@
         <v/>
       </c>
       <c r="F216" s="3">
-        <f>IF(A216="","",IF(D216=0,"",MAXIFS(Sales!C:C,Sales!D:D,A216)))</f>
+        <f>IF(A216="","",IF(D216=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A216)))</f>
         <v/>
       </c>
       <c r="G216">
@@ -23202,7 +23202,7 @@
         <v/>
       </c>
       <c r="F217" s="3">
-        <f>IF(A217="","",IF(D217=0,"",MAXIFS(Sales!C:C,Sales!D:D,A217)))</f>
+        <f>IF(A217="","",IF(D217=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A217)))</f>
         <v/>
       </c>
       <c r="G217">
@@ -23236,7 +23236,7 @@
         <v/>
       </c>
       <c r="F218" s="3">
-        <f>IF(A218="","",IF(D218=0,"",MAXIFS(Sales!C:C,Sales!D:D,A218)))</f>
+        <f>IF(A218="","",IF(D218=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A218)))</f>
         <v/>
       </c>
       <c r="G218">
@@ -23270,7 +23270,7 @@
         <v/>
       </c>
       <c r="F219" s="3">
-        <f>IF(A219="","",IF(D219=0,"",MAXIFS(Sales!C:C,Sales!D:D,A219)))</f>
+        <f>IF(A219="","",IF(D219=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A219)))</f>
         <v/>
       </c>
       <c r="G219">
@@ -23304,7 +23304,7 @@
         <v/>
       </c>
       <c r="F220" s="3">
-        <f>IF(A220="","",IF(D220=0,"",MAXIFS(Sales!C:C,Sales!D:D,A220)))</f>
+        <f>IF(A220="","",IF(D220=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A220)))</f>
         <v/>
       </c>
       <c r="G220">
@@ -23338,7 +23338,7 @@
         <v/>
       </c>
       <c r="F221" s="3">
-        <f>IF(A221="","",IF(D221=0,"",MAXIFS(Sales!C:C,Sales!D:D,A221)))</f>
+        <f>IF(A221="","",IF(D221=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A221)))</f>
         <v/>
       </c>
       <c r="G221">
@@ -23372,7 +23372,7 @@
         <v/>
       </c>
       <c r="F222" s="3">
-        <f>IF(A222="","",IF(D222=0,"",MAXIFS(Sales!C:C,Sales!D:D,A222)))</f>
+        <f>IF(A222="","",IF(D222=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A222)))</f>
         <v/>
       </c>
       <c r="G222">
@@ -23406,7 +23406,7 @@
         <v/>
       </c>
       <c r="F223" s="3">
-        <f>IF(A223="","",IF(D223=0,"",MAXIFS(Sales!C:C,Sales!D:D,A223)))</f>
+        <f>IF(A223="","",IF(D223=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A223)))</f>
         <v/>
       </c>
       <c r="G223">
@@ -23440,7 +23440,7 @@
         <v/>
       </c>
       <c r="F224" s="3">
-        <f>IF(A224="","",IF(D224=0,"",MAXIFS(Sales!C:C,Sales!D:D,A224)))</f>
+        <f>IF(A224="","",IF(D224=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A224)))</f>
         <v/>
       </c>
       <c r="G224">
@@ -23474,7 +23474,7 @@
         <v/>
       </c>
       <c r="F225" s="3">
-        <f>IF(A225="","",IF(D225=0,"",MAXIFS(Sales!C:C,Sales!D:D,A225)))</f>
+        <f>IF(A225="","",IF(D225=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A225)))</f>
         <v/>
       </c>
       <c r="G225">
@@ -23508,7 +23508,7 @@
         <v/>
       </c>
       <c r="F226" s="3">
-        <f>IF(A226="","",IF(D226=0,"",MAXIFS(Sales!C:C,Sales!D:D,A226)))</f>
+        <f>IF(A226="","",IF(D226=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A226)))</f>
         <v/>
       </c>
       <c r="G226">
@@ -23542,7 +23542,7 @@
         <v/>
       </c>
       <c r="F227" s="3">
-        <f>IF(A227="","",IF(D227=0,"",MAXIFS(Sales!C:C,Sales!D:D,A227)))</f>
+        <f>IF(A227="","",IF(D227=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A227)))</f>
         <v/>
       </c>
       <c r="G227">
@@ -23576,7 +23576,7 @@
         <v/>
       </c>
       <c r="F228" s="3">
-        <f>IF(A228="","",IF(D228=0,"",MAXIFS(Sales!C:C,Sales!D:D,A228)))</f>
+        <f>IF(A228="","",IF(D228=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A228)))</f>
         <v/>
       </c>
       <c r="G228">
@@ -23610,7 +23610,7 @@
         <v/>
       </c>
       <c r="F229" s="3">
-        <f>IF(A229="","",IF(D229=0,"",MAXIFS(Sales!C:C,Sales!D:D,A229)))</f>
+        <f>IF(A229="","",IF(D229=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A229)))</f>
         <v/>
       </c>
       <c r="G229">
@@ -23644,7 +23644,7 @@
         <v/>
       </c>
       <c r="F230" s="3">
-        <f>IF(A230="","",IF(D230=0,"",MAXIFS(Sales!C:C,Sales!D:D,A230)))</f>
+        <f>IF(A230="","",IF(D230=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A230)))</f>
         <v/>
       </c>
       <c r="G230">
@@ -23678,7 +23678,7 @@
         <v/>
       </c>
       <c r="F231" s="3">
-        <f>IF(A231="","",IF(D231=0,"",MAXIFS(Sales!C:C,Sales!D:D,A231)))</f>
+        <f>IF(A231="","",IF(D231=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A231)))</f>
         <v/>
       </c>
       <c r="G231">
@@ -23712,7 +23712,7 @@
         <v/>
       </c>
       <c r="F232" s="3">
-        <f>IF(A232="","",IF(D232=0,"",MAXIFS(Sales!C:C,Sales!D:D,A232)))</f>
+        <f>IF(A232="","",IF(D232=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A232)))</f>
         <v/>
       </c>
       <c r="G232">
@@ -23746,7 +23746,7 @@
         <v/>
       </c>
       <c r="F233" s="3">
-        <f>IF(A233="","",IF(D233=0,"",MAXIFS(Sales!C:C,Sales!D:D,A233)))</f>
+        <f>IF(A233="","",IF(D233=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A233)))</f>
         <v/>
       </c>
       <c r="G233">
@@ -23780,7 +23780,7 @@
         <v/>
       </c>
       <c r="F234" s="3">
-        <f>IF(A234="","",IF(D234=0,"",MAXIFS(Sales!C:C,Sales!D:D,A234)))</f>
+        <f>IF(A234="","",IF(D234=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A234)))</f>
         <v/>
       </c>
       <c r="G234">
@@ -23814,7 +23814,7 @@
         <v/>
       </c>
       <c r="F235" s="3">
-        <f>IF(A235="","",IF(D235=0,"",MAXIFS(Sales!C:C,Sales!D:D,A235)))</f>
+        <f>IF(A235="","",IF(D235=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A235)))</f>
         <v/>
       </c>
       <c r="G235">
@@ -23848,7 +23848,7 @@
         <v/>
       </c>
       <c r="F236" s="3">
-        <f>IF(A236="","",IF(D236=0,"",MAXIFS(Sales!C:C,Sales!D:D,A236)))</f>
+        <f>IF(A236="","",IF(D236=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A236)))</f>
         <v/>
       </c>
       <c r="G236">
@@ -23882,7 +23882,7 @@
         <v/>
       </c>
       <c r="F237" s="3">
-        <f>IF(A237="","",IF(D237=0,"",MAXIFS(Sales!C:C,Sales!D:D,A237)))</f>
+        <f>IF(A237="","",IF(D237=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A237)))</f>
         <v/>
       </c>
       <c r="G237">
@@ -23916,7 +23916,7 @@
         <v/>
       </c>
       <c r="F238" s="3">
-        <f>IF(A238="","",IF(D238=0,"",MAXIFS(Sales!C:C,Sales!D:D,A238)))</f>
+        <f>IF(A238="","",IF(D238=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A238)))</f>
         <v/>
       </c>
       <c r="G238">
@@ -23950,7 +23950,7 @@
         <v/>
       </c>
       <c r="F239" s="3">
-        <f>IF(A239="","",IF(D239=0,"",MAXIFS(Sales!C:C,Sales!D:D,A239)))</f>
+        <f>IF(A239="","",IF(D239=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A239)))</f>
         <v/>
       </c>
       <c r="G239">
@@ -23984,7 +23984,7 @@
         <v/>
       </c>
       <c r="F240" s="3">
-        <f>IF(A240="","",IF(D240=0,"",MAXIFS(Sales!C:C,Sales!D:D,A240)))</f>
+        <f>IF(A240="","",IF(D240=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A240)))</f>
         <v/>
       </c>
       <c r="G240">
@@ -24018,7 +24018,7 @@
         <v/>
       </c>
       <c r="F241" s="3">
-        <f>IF(A241="","",IF(D241=0,"",MAXIFS(Sales!C:C,Sales!D:D,A241)))</f>
+        <f>IF(A241="","",IF(D241=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A241)))</f>
         <v/>
       </c>
       <c r="G241">
@@ -24052,7 +24052,7 @@
         <v/>
       </c>
       <c r="F242" s="3">
-        <f>IF(A242="","",IF(D242=0,"",MAXIFS(Sales!C:C,Sales!D:D,A242)))</f>
+        <f>IF(A242="","",IF(D242=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A242)))</f>
         <v/>
       </c>
       <c r="G242">
@@ -24086,7 +24086,7 @@
         <v/>
       </c>
       <c r="F243" s="3">
-        <f>IF(A243="","",IF(D243=0,"",MAXIFS(Sales!C:C,Sales!D:D,A243)))</f>
+        <f>IF(A243="","",IF(D243=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A243)))</f>
         <v/>
       </c>
       <c r="G243">
@@ -24120,7 +24120,7 @@
         <v/>
       </c>
       <c r="F244" s="3">
-        <f>IF(A244="","",IF(D244=0,"",MAXIFS(Sales!C:C,Sales!D:D,A244)))</f>
+        <f>IF(A244="","",IF(D244=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A244)))</f>
         <v/>
       </c>
       <c r="G244">
@@ -24154,7 +24154,7 @@
         <v/>
       </c>
       <c r="F245" s="3">
-        <f>IF(A245="","",IF(D245=0,"",MAXIFS(Sales!C:C,Sales!D:D,A245)))</f>
+        <f>IF(A245="","",IF(D245=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A245)))</f>
         <v/>
       </c>
       <c r="G245">
@@ -24188,7 +24188,7 @@
         <v/>
       </c>
       <c r="F246" s="3">
-        <f>IF(A246="","",IF(D246=0,"",MAXIFS(Sales!C:C,Sales!D:D,A246)))</f>
+        <f>IF(A246="","",IF(D246=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A246)))</f>
         <v/>
       </c>
       <c r="G246">
@@ -24222,7 +24222,7 @@
         <v/>
       </c>
       <c r="F247" s="3">
-        <f>IF(A247="","",IF(D247=0,"",MAXIFS(Sales!C:C,Sales!D:D,A247)))</f>
+        <f>IF(A247="","",IF(D247=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A247)))</f>
         <v/>
       </c>
       <c r="G247">
@@ -24256,7 +24256,7 @@
         <v/>
       </c>
       <c r="F248" s="3">
-        <f>IF(A248="","",IF(D248=0,"",MAXIFS(Sales!C:C,Sales!D:D,A248)))</f>
+        <f>IF(A248="","",IF(D248=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A248)))</f>
         <v/>
       </c>
       <c r="G248">
@@ -24290,7 +24290,7 @@
         <v/>
       </c>
       <c r="F249" s="3">
-        <f>IF(A249="","",IF(D249=0,"",MAXIFS(Sales!C:C,Sales!D:D,A249)))</f>
+        <f>IF(A249="","",IF(D249=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A249)))</f>
         <v/>
       </c>
       <c r="G249">
@@ -24324,7 +24324,7 @@
         <v/>
       </c>
       <c r="F250" s="3">
-        <f>IF(A250="","",IF(D250=0,"",MAXIFS(Sales!C:C,Sales!D:D,A250)))</f>
+        <f>IF(A250="","",IF(D250=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A250)))</f>
         <v/>
       </c>
       <c r="G250">
@@ -24358,7 +24358,7 @@
         <v/>
       </c>
       <c r="F251" s="3">
-        <f>IF(A251="","",IF(D251=0,"",MAXIFS(Sales!C:C,Sales!D:D,A251)))</f>
+        <f>IF(A251="","",IF(D251=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A251)))</f>
         <v/>
       </c>
       <c r="G251">
@@ -24392,7 +24392,7 @@
         <v/>
       </c>
       <c r="F252" s="3">
-        <f>IF(A252="","",IF(D252=0,"",MAXIFS(Sales!C:C,Sales!D:D,A252)))</f>
+        <f>IF(A252="","",IF(D252=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A252)))</f>
         <v/>
       </c>
       <c r="G252">
@@ -24426,7 +24426,7 @@
         <v/>
       </c>
       <c r="F253" s="3">
-        <f>IF(A253="","",IF(D253=0,"",MAXIFS(Sales!C:C,Sales!D:D,A253)))</f>
+        <f>IF(A253="","",IF(D253=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A253)))</f>
         <v/>
       </c>
       <c r="G253">
@@ -24460,7 +24460,7 @@
         <v/>
       </c>
       <c r="F254" s="3">
-        <f>IF(A254="","",IF(D254=0,"",MAXIFS(Sales!C:C,Sales!D:D,A254)))</f>
+        <f>IF(A254="","",IF(D254=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A254)))</f>
         <v/>
       </c>
       <c r="G254">
@@ -24494,7 +24494,7 @@
         <v/>
       </c>
       <c r="F255" s="3">
-        <f>IF(A255="","",IF(D255=0,"",MAXIFS(Sales!C:C,Sales!D:D,A255)))</f>
+        <f>IF(A255="","",IF(D255=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A255)))</f>
         <v/>
       </c>
       <c r="G255">
@@ -24528,7 +24528,7 @@
         <v/>
       </c>
       <c r="F256" s="3">
-        <f>IF(A256="","",IF(D256=0,"",MAXIFS(Sales!C:C,Sales!D:D,A256)))</f>
+        <f>IF(A256="","",IF(D256=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A256)))</f>
         <v/>
       </c>
       <c r="G256">
@@ -24562,7 +24562,7 @@
         <v/>
       </c>
       <c r="F257" s="3">
-        <f>IF(A257="","",IF(D257=0,"",MAXIFS(Sales!C:C,Sales!D:D,A257)))</f>
+        <f>IF(A257="","",IF(D257=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A257)))</f>
         <v/>
       </c>
       <c r="G257">
@@ -24596,7 +24596,7 @@
         <v/>
       </c>
       <c r="F258" s="3">
-        <f>IF(A258="","",IF(D258=0,"",MAXIFS(Sales!C:C,Sales!D:D,A258)))</f>
+        <f>IF(A258="","",IF(D258=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A258)))</f>
         <v/>
       </c>
       <c r="G258">
@@ -24630,7 +24630,7 @@
         <v/>
       </c>
       <c r="F259" s="3">
-        <f>IF(A259="","",IF(D259=0,"",MAXIFS(Sales!C:C,Sales!D:D,A259)))</f>
+        <f>IF(A259="","",IF(D259=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A259)))</f>
         <v/>
       </c>
       <c r="G259">
@@ -24664,7 +24664,7 @@
         <v/>
       </c>
       <c r="F260" s="3">
-        <f>IF(A260="","",IF(D260=0,"",MAXIFS(Sales!C:C,Sales!D:D,A260)))</f>
+        <f>IF(A260="","",IF(D260=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A260)))</f>
         <v/>
       </c>
       <c r="G260">
@@ -24698,7 +24698,7 @@
         <v/>
       </c>
       <c r="F261" s="3">
-        <f>IF(A261="","",IF(D261=0,"",MAXIFS(Sales!C:C,Sales!D:D,A261)))</f>
+        <f>IF(A261="","",IF(D261=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A261)))</f>
         <v/>
       </c>
       <c r="G261">
@@ -24732,7 +24732,7 @@
         <v/>
       </c>
       <c r="F262" s="3">
-        <f>IF(A262="","",IF(D262=0,"",MAXIFS(Sales!C:C,Sales!D:D,A262)))</f>
+        <f>IF(A262="","",IF(D262=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A262)))</f>
         <v/>
       </c>
       <c r="G262">
@@ -24766,7 +24766,7 @@
         <v/>
       </c>
       <c r="F263" s="3">
-        <f>IF(A263="","",IF(D263=0,"",MAXIFS(Sales!C:C,Sales!D:D,A263)))</f>
+        <f>IF(A263="","",IF(D263=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A263)))</f>
         <v/>
       </c>
       <c r="G263">
@@ -24800,7 +24800,7 @@
         <v/>
       </c>
       <c r="F264" s="3">
-        <f>IF(A264="","",IF(D264=0,"",MAXIFS(Sales!C:C,Sales!D:D,A264)))</f>
+        <f>IF(A264="","",IF(D264=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A264)))</f>
         <v/>
       </c>
       <c r="G264">
@@ -24834,7 +24834,7 @@
         <v/>
       </c>
       <c r="F265" s="3">
-        <f>IF(A265="","",IF(D265=0,"",MAXIFS(Sales!C:C,Sales!D:D,A265)))</f>
+        <f>IF(A265="","",IF(D265=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A265)))</f>
         <v/>
       </c>
       <c r="G265">
@@ -24868,7 +24868,7 @@
         <v/>
       </c>
       <c r="F266" s="3">
-        <f>IF(A266="","",IF(D266=0,"",MAXIFS(Sales!C:C,Sales!D:D,A266)))</f>
+        <f>IF(A266="","",IF(D266=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A266)))</f>
         <v/>
       </c>
       <c r="G266">
@@ -24902,7 +24902,7 @@
         <v/>
       </c>
       <c r="F267" s="3">
-        <f>IF(A267="","",IF(D267=0,"",MAXIFS(Sales!C:C,Sales!D:D,A267)))</f>
+        <f>IF(A267="","",IF(D267=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A267)))</f>
         <v/>
       </c>
       <c r="G267">
@@ -24936,7 +24936,7 @@
         <v/>
       </c>
       <c r="F268" s="3">
-        <f>IF(A268="","",IF(D268=0,"",MAXIFS(Sales!C:C,Sales!D:D,A268)))</f>
+        <f>IF(A268="","",IF(D268=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A268)))</f>
         <v/>
       </c>
       <c r="G268">
@@ -24970,7 +24970,7 @@
         <v/>
       </c>
       <c r="F269" s="3">
-        <f>IF(A269="","",IF(D269=0,"",MAXIFS(Sales!C:C,Sales!D:D,A269)))</f>
+        <f>IF(A269="","",IF(D269=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A269)))</f>
         <v/>
       </c>
       <c r="G269">
@@ -25004,7 +25004,7 @@
         <v/>
       </c>
       <c r="F270" s="3">
-        <f>IF(A270="","",IF(D270=0,"",MAXIFS(Sales!C:C,Sales!D:D,A270)))</f>
+        <f>IF(A270="","",IF(D270=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A270)))</f>
         <v/>
       </c>
       <c r="G270">
@@ -25038,7 +25038,7 @@
         <v/>
       </c>
       <c r="F271" s="3">
-        <f>IF(A271="","",IF(D271=0,"",MAXIFS(Sales!C:C,Sales!D:D,A271)))</f>
+        <f>IF(A271="","",IF(D271=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A271)))</f>
         <v/>
       </c>
       <c r="G271">
@@ -25072,7 +25072,7 @@
         <v/>
       </c>
       <c r="F272" s="3">
-        <f>IF(A272="","",IF(D272=0,"",MAXIFS(Sales!C:C,Sales!D:D,A272)))</f>
+        <f>IF(A272="","",IF(D272=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A272)))</f>
         <v/>
       </c>
       <c r="G272">
@@ -25106,7 +25106,7 @@
         <v/>
       </c>
       <c r="F273" s="3">
-        <f>IF(A273="","",IF(D273=0,"",MAXIFS(Sales!C:C,Sales!D:D,A273)))</f>
+        <f>IF(A273="","",IF(D273=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A273)))</f>
         <v/>
       </c>
       <c r="G273">
@@ -25140,7 +25140,7 @@
         <v/>
       </c>
       <c r="F274" s="3">
-        <f>IF(A274="","",IF(D274=0,"",MAXIFS(Sales!C:C,Sales!D:D,A274)))</f>
+        <f>IF(A274="","",IF(D274=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A274)))</f>
         <v/>
       </c>
       <c r="G274">
@@ -25174,7 +25174,7 @@
         <v/>
       </c>
       <c r="F275" s="3">
-        <f>IF(A275="","",IF(D275=0,"",MAXIFS(Sales!C:C,Sales!D:D,A275)))</f>
+        <f>IF(A275="","",IF(D275=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A275)))</f>
         <v/>
       </c>
       <c r="G275">
@@ -25208,7 +25208,7 @@
         <v/>
       </c>
       <c r="F276" s="3">
-        <f>IF(A276="","",IF(D276=0,"",MAXIFS(Sales!C:C,Sales!D:D,A276)))</f>
+        <f>IF(A276="","",IF(D276=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A276)))</f>
         <v/>
       </c>
       <c r="G276">
@@ -25242,7 +25242,7 @@
         <v/>
       </c>
       <c r="F277" s="3">
-        <f>IF(A277="","",IF(D277=0,"",MAXIFS(Sales!C:C,Sales!D:D,A277)))</f>
+        <f>IF(A277="","",IF(D277=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A277)))</f>
         <v/>
       </c>
       <c r="G277">
@@ -25276,7 +25276,7 @@
         <v/>
       </c>
       <c r="F278" s="3">
-        <f>IF(A278="","",IF(D278=0,"",MAXIFS(Sales!C:C,Sales!D:D,A278)))</f>
+        <f>IF(A278="","",IF(D278=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A278)))</f>
         <v/>
       </c>
       <c r="G278">
@@ -25310,7 +25310,7 @@
         <v/>
       </c>
       <c r="F279" s="3">
-        <f>IF(A279="","",IF(D279=0,"",MAXIFS(Sales!C:C,Sales!D:D,A279)))</f>
+        <f>IF(A279="","",IF(D279=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A279)))</f>
         <v/>
       </c>
       <c r="G279">
@@ -25344,7 +25344,7 @@
         <v/>
       </c>
       <c r="F280" s="3">
-        <f>IF(A280="","",IF(D280=0,"",MAXIFS(Sales!C:C,Sales!D:D,A280)))</f>
+        <f>IF(A280="","",IF(D280=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A280)))</f>
         <v/>
       </c>
       <c r="G280">
@@ -25378,7 +25378,7 @@
         <v/>
       </c>
       <c r="F281" s="3">
-        <f>IF(A281="","",IF(D281=0,"",MAXIFS(Sales!C:C,Sales!D:D,A281)))</f>
+        <f>IF(A281="","",IF(D281=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A281)))</f>
         <v/>
       </c>
       <c r="G281">
@@ -25412,7 +25412,7 @@
         <v/>
       </c>
       <c r="F282" s="3">
-        <f>IF(A282="","",IF(D282=0,"",MAXIFS(Sales!C:C,Sales!D:D,A282)))</f>
+        <f>IF(A282="","",IF(D282=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A282)))</f>
         <v/>
       </c>
       <c r="G282">
@@ -25446,7 +25446,7 @@
         <v/>
       </c>
       <c r="F283" s="3">
-        <f>IF(A283="","",IF(D283=0,"",MAXIFS(Sales!C:C,Sales!D:D,A283)))</f>
+        <f>IF(A283="","",IF(D283=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A283)))</f>
         <v/>
       </c>
       <c r="G283">
@@ -25480,7 +25480,7 @@
         <v/>
       </c>
       <c r="F284" s="3">
-        <f>IF(A284="","",IF(D284=0,"",MAXIFS(Sales!C:C,Sales!D:D,A284)))</f>
+        <f>IF(A284="","",IF(D284=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A284)))</f>
         <v/>
       </c>
       <c r="G284">
@@ -25514,7 +25514,7 @@
         <v/>
       </c>
       <c r="F285" s="3">
-        <f>IF(A285="","",IF(D285=0,"",MAXIFS(Sales!C:C,Sales!D:D,A285)))</f>
+        <f>IF(A285="","",IF(D285=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A285)))</f>
         <v/>
       </c>
       <c r="G285">
@@ -25548,7 +25548,7 @@
         <v/>
       </c>
       <c r="F286" s="3">
-        <f>IF(A286="","",IF(D286=0,"",MAXIFS(Sales!C:C,Sales!D:D,A286)))</f>
+        <f>IF(A286="","",IF(D286=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A286)))</f>
         <v/>
       </c>
       <c r="G286">
@@ -25582,7 +25582,7 @@
         <v/>
       </c>
       <c r="F287" s="3">
-        <f>IF(A287="","",IF(D287=0,"",MAXIFS(Sales!C:C,Sales!D:D,A287)))</f>
+        <f>IF(A287="","",IF(D287=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A287)))</f>
         <v/>
       </c>
       <c r="G287">
@@ -25616,7 +25616,7 @@
         <v/>
       </c>
       <c r="F288" s="3">
-        <f>IF(A288="","",IF(D288=0,"",MAXIFS(Sales!C:C,Sales!D:D,A288)))</f>
+        <f>IF(A288="","",IF(D288=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A288)))</f>
         <v/>
       </c>
       <c r="G288">
@@ -25650,7 +25650,7 @@
         <v/>
       </c>
       <c r="F289" s="3">
-        <f>IF(A289="","",IF(D289=0,"",MAXIFS(Sales!C:C,Sales!D:D,A289)))</f>
+        <f>IF(A289="","",IF(D289=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A289)))</f>
         <v/>
       </c>
       <c r="G289">
@@ -25684,7 +25684,7 @@
         <v/>
       </c>
       <c r="F290" s="3">
-        <f>IF(A290="","",IF(D290=0,"",MAXIFS(Sales!C:C,Sales!D:D,A290)))</f>
+        <f>IF(A290="","",IF(D290=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A290)))</f>
         <v/>
       </c>
       <c r="G290">
@@ -25718,7 +25718,7 @@
         <v/>
       </c>
       <c r="F291" s="3">
-        <f>IF(A291="","",IF(D291=0,"",MAXIFS(Sales!C:C,Sales!D:D,A291)))</f>
+        <f>IF(A291="","",IF(D291=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A291)))</f>
         <v/>
       </c>
       <c r="G291">
@@ -25752,7 +25752,7 @@
         <v/>
       </c>
       <c r="F292" s="3">
-        <f>IF(A292="","",IF(D292=0,"",MAXIFS(Sales!C:C,Sales!D:D,A292)))</f>
+        <f>IF(A292="","",IF(D292=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A292)))</f>
         <v/>
       </c>
       <c r="G292">
@@ -25786,7 +25786,7 @@
         <v/>
       </c>
       <c r="F293" s="3">
-        <f>IF(A293="","",IF(D293=0,"",MAXIFS(Sales!C:C,Sales!D:D,A293)))</f>
+        <f>IF(A293="","",IF(D293=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A293)))</f>
         <v/>
       </c>
       <c r="G293">
@@ -25820,7 +25820,7 @@
         <v/>
       </c>
       <c r="F294" s="3">
-        <f>IF(A294="","",IF(D294=0,"",MAXIFS(Sales!C:C,Sales!D:D,A294)))</f>
+        <f>IF(A294="","",IF(D294=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A294)))</f>
         <v/>
       </c>
       <c r="G294">
@@ -25854,7 +25854,7 @@
         <v/>
       </c>
       <c r="F295" s="3">
-        <f>IF(A295="","",IF(D295=0,"",MAXIFS(Sales!C:C,Sales!D:D,A295)))</f>
+        <f>IF(A295="","",IF(D295=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A295)))</f>
         <v/>
       </c>
       <c r="G295">
@@ -25888,7 +25888,7 @@
         <v/>
       </c>
       <c r="F296" s="3">
-        <f>IF(A296="","",IF(D296=0,"",MAXIFS(Sales!C:C,Sales!D:D,A296)))</f>
+        <f>IF(A296="","",IF(D296=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A296)))</f>
         <v/>
       </c>
       <c r="G296">
@@ -25922,7 +25922,7 @@
         <v/>
       </c>
       <c r="F297" s="3">
-        <f>IF(A297="","",IF(D297=0,"",MAXIFS(Sales!C:C,Sales!D:D,A297)))</f>
+        <f>IF(A297="","",IF(D297=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A297)))</f>
         <v/>
       </c>
       <c r="G297">
@@ -25956,7 +25956,7 @@
         <v/>
       </c>
       <c r="F298" s="3">
-        <f>IF(A298="","",IF(D298=0,"",MAXIFS(Sales!C:C,Sales!D:D,A298)))</f>
+        <f>IF(A298="","",IF(D298=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A298)))</f>
         <v/>
       </c>
       <c r="G298">
@@ -25990,7 +25990,7 @@
         <v/>
       </c>
       <c r="F299" s="3">
-        <f>IF(A299="","",IF(D299=0,"",MAXIFS(Sales!C:C,Sales!D:D,A299)))</f>
+        <f>IF(A299="","",IF(D299=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A299)))</f>
         <v/>
       </c>
       <c r="G299">
@@ -26024,7 +26024,7 @@
         <v/>
       </c>
       <c r="F300" s="3">
-        <f>IF(A300="","",IF(D300=0,"",MAXIFS(Sales!C:C,Sales!D:D,A300)))</f>
+        <f>IF(A300="","",IF(D300=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A300)))</f>
         <v/>
       </c>
       <c r="G300">
@@ -26058,7 +26058,7 @@
         <v/>
       </c>
       <c r="F301" s="3">
-        <f>IF(A301="","",IF(D301=0,"",MAXIFS(Sales!C:C,Sales!D:D,A301)))</f>
+        <f>IF(A301="","",IF(D301=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A301)))</f>
         <v/>
       </c>
       <c r="G301">
@@ -26092,7 +26092,7 @@
         <v/>
       </c>
       <c r="F302" s="3">
-        <f>IF(A302="","",IF(D302=0,"",MAXIFS(Sales!C:C,Sales!D:D,A302)))</f>
+        <f>IF(A302="","",IF(D302=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A302)))</f>
         <v/>
       </c>
       <c r="G302">
@@ -26126,7 +26126,7 @@
         <v/>
       </c>
       <c r="F303" s="3">
-        <f>IF(A303="","",IF(D303=0,"",MAXIFS(Sales!C:C,Sales!D:D,A303)))</f>
+        <f>IF(A303="","",IF(D303=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A303)))</f>
         <v/>
       </c>
       <c r="G303">
@@ -26160,7 +26160,7 @@
         <v/>
       </c>
       <c r="F304" s="3">
-        <f>IF(A304="","",IF(D304=0,"",MAXIFS(Sales!C:C,Sales!D:D,A304)))</f>
+        <f>IF(A304="","",IF(D304=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A304)))</f>
         <v/>
       </c>
       <c r="G304">
@@ -26194,7 +26194,7 @@
         <v/>
       </c>
       <c r="F305" s="3">
-        <f>IF(A305="","",IF(D305=0,"",MAXIFS(Sales!C:C,Sales!D:D,A305)))</f>
+        <f>IF(A305="","",IF(D305=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A305)))</f>
         <v/>
       </c>
       <c r="G305">
@@ -26228,7 +26228,7 @@
         <v/>
       </c>
       <c r="F306" s="3">
-        <f>IF(A306="","",IF(D306=0,"",MAXIFS(Sales!C:C,Sales!D:D,A306)))</f>
+        <f>IF(A306="","",IF(D306=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A306)))</f>
         <v/>
       </c>
       <c r="G306">
@@ -26262,7 +26262,7 @@
         <v/>
       </c>
       <c r="F307" s="3">
-        <f>IF(A307="","",IF(D307=0,"",MAXIFS(Sales!C:C,Sales!D:D,A307)))</f>
+        <f>IF(A307="","",IF(D307=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A307)))</f>
         <v/>
       </c>
       <c r="G307">
@@ -26296,7 +26296,7 @@
         <v/>
       </c>
       <c r="F308" s="3">
-        <f>IF(A308="","",IF(D308=0,"",MAXIFS(Sales!C:C,Sales!D:D,A308)))</f>
+        <f>IF(A308="","",IF(D308=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A308)))</f>
         <v/>
       </c>
       <c r="G308">
@@ -26330,7 +26330,7 @@
         <v/>
       </c>
       <c r="F309" s="3">
-        <f>IF(A309="","",IF(D309=0,"",MAXIFS(Sales!C:C,Sales!D:D,A309)))</f>
+        <f>IF(A309="","",IF(D309=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A309)))</f>
         <v/>
       </c>
       <c r="G309">
@@ -26364,7 +26364,7 @@
         <v/>
       </c>
       <c r="F310" s="3">
-        <f>IF(A310="","",IF(D310=0,"",MAXIFS(Sales!C:C,Sales!D:D,A310)))</f>
+        <f>IF(A310="","",IF(D310=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A310)))</f>
         <v/>
       </c>
       <c r="G310">
@@ -26398,7 +26398,7 @@
         <v/>
       </c>
       <c r="F311" s="3">
-        <f>IF(A311="","",IF(D311=0,"",MAXIFS(Sales!C:C,Sales!D:D,A311)))</f>
+        <f>IF(A311="","",IF(D311=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A311)))</f>
         <v/>
       </c>
       <c r="G311">
@@ -26432,7 +26432,7 @@
         <v/>
       </c>
       <c r="F312" s="3">
-        <f>IF(A312="","",IF(D312=0,"",MAXIFS(Sales!C:C,Sales!D:D,A312)))</f>
+        <f>IF(A312="","",IF(D312=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A312)))</f>
         <v/>
       </c>
       <c r="G312">
@@ -26466,7 +26466,7 @@
         <v/>
       </c>
       <c r="F313" s="3">
-        <f>IF(A313="","",IF(D313=0,"",MAXIFS(Sales!C:C,Sales!D:D,A313)))</f>
+        <f>IF(A313="","",IF(D313=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A313)))</f>
         <v/>
       </c>
       <c r="G313">
@@ -26500,7 +26500,7 @@
         <v/>
       </c>
       <c r="F314" s="3">
-        <f>IF(A314="","",IF(D314=0,"",MAXIFS(Sales!C:C,Sales!D:D,A314)))</f>
+        <f>IF(A314="","",IF(D314=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A314)))</f>
         <v/>
       </c>
       <c r="G314">
@@ -26534,7 +26534,7 @@
         <v/>
       </c>
       <c r="F315" s="3">
-        <f>IF(A315="","",IF(D315=0,"",MAXIFS(Sales!C:C,Sales!D:D,A315)))</f>
+        <f>IF(A315="","",IF(D315=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A315)))</f>
         <v/>
       </c>
       <c r="G315">
@@ -26568,7 +26568,7 @@
         <v/>
       </c>
       <c r="F316" s="3">
-        <f>IF(A316="","",IF(D316=0,"",MAXIFS(Sales!C:C,Sales!D:D,A316)))</f>
+        <f>IF(A316="","",IF(D316=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A316)))</f>
         <v/>
       </c>
       <c r="G316">
@@ -26602,7 +26602,7 @@
         <v/>
       </c>
       <c r="F317" s="3">
-        <f>IF(A317="","",IF(D317=0,"",MAXIFS(Sales!C:C,Sales!D:D,A317)))</f>
+        <f>IF(A317="","",IF(D317=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A317)))</f>
         <v/>
       </c>
       <c r="G317">
@@ -26636,7 +26636,7 @@
         <v/>
       </c>
       <c r="F318" s="3">
-        <f>IF(A318="","",IF(D318=0,"",MAXIFS(Sales!C:C,Sales!D:D,A318)))</f>
+        <f>IF(A318="","",IF(D318=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A318)))</f>
         <v/>
       </c>
       <c r="G318">
@@ -26670,7 +26670,7 @@
         <v/>
       </c>
       <c r="F319" s="3">
-        <f>IF(A319="","",IF(D319=0,"",MAXIFS(Sales!C:C,Sales!D:D,A319)))</f>
+        <f>IF(A319="","",IF(D319=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A319)))</f>
         <v/>
       </c>
       <c r="G319">
@@ -26704,7 +26704,7 @@
         <v/>
       </c>
       <c r="F320" s="3">
-        <f>IF(A320="","",IF(D320=0,"",MAXIFS(Sales!C:C,Sales!D:D,A320)))</f>
+        <f>IF(A320="","",IF(D320=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A320)))</f>
         <v/>
       </c>
       <c r="G320">
@@ -26738,7 +26738,7 @@
         <v/>
       </c>
       <c r="F321" s="3">
-        <f>IF(A321="","",IF(D321=0,"",MAXIFS(Sales!C:C,Sales!D:D,A321)))</f>
+        <f>IF(A321="","",IF(D321=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A321)))</f>
         <v/>
       </c>
       <c r="G321">
@@ -26772,7 +26772,7 @@
         <v/>
       </c>
       <c r="F322" s="3">
-        <f>IF(A322="","",IF(D322=0,"",MAXIFS(Sales!C:C,Sales!D:D,A322)))</f>
+        <f>IF(A322="","",IF(D322=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A322)))</f>
         <v/>
       </c>
       <c r="G322">
@@ -26806,7 +26806,7 @@
         <v/>
       </c>
       <c r="F323" s="3">
-        <f>IF(A323="","",IF(D323=0,"",MAXIFS(Sales!C:C,Sales!D:D,A323)))</f>
+        <f>IF(A323="","",IF(D323=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A323)))</f>
         <v/>
       </c>
       <c r="G323">
@@ -26840,7 +26840,7 @@
         <v/>
       </c>
       <c r="F324" s="3">
-        <f>IF(A324="","",IF(D324=0,"",MAXIFS(Sales!C:C,Sales!D:D,A324)))</f>
+        <f>IF(A324="","",IF(D324=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A324)))</f>
         <v/>
       </c>
       <c r="G324">
@@ -26874,7 +26874,7 @@
         <v/>
       </c>
       <c r="F325" s="3">
-        <f>IF(A325="","",IF(D325=0,"",MAXIFS(Sales!C:C,Sales!D:D,A325)))</f>
+        <f>IF(A325="","",IF(D325=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A325)))</f>
         <v/>
       </c>
       <c r="G325">
@@ -26908,7 +26908,7 @@
         <v/>
       </c>
       <c r="F326" s="3">
-        <f>IF(A326="","",IF(D326=0,"",MAXIFS(Sales!C:C,Sales!D:D,A326)))</f>
+        <f>IF(A326="","",IF(D326=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A326)))</f>
         <v/>
       </c>
       <c r="G326">
@@ -26942,7 +26942,7 @@
         <v/>
       </c>
       <c r="F327" s="3">
-        <f>IF(A327="","",IF(D327=0,"",MAXIFS(Sales!C:C,Sales!D:D,A327)))</f>
+        <f>IF(A327="","",IF(D327=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A327)))</f>
         <v/>
       </c>
       <c r="G327">
@@ -26976,7 +26976,7 @@
         <v/>
       </c>
       <c r="F328" s="3">
-        <f>IF(A328="","",IF(D328=0,"",MAXIFS(Sales!C:C,Sales!D:D,A328)))</f>
+        <f>IF(A328="","",IF(D328=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A328)))</f>
         <v/>
       </c>
       <c r="G328">
@@ -27010,7 +27010,7 @@
         <v/>
       </c>
       <c r="F329" s="3">
-        <f>IF(A329="","",IF(D329=0,"",MAXIFS(Sales!C:C,Sales!D:D,A329)))</f>
+        <f>IF(A329="","",IF(D329=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A329)))</f>
         <v/>
       </c>
       <c r="G329">
@@ -27044,7 +27044,7 @@
         <v/>
       </c>
       <c r="F330" s="3">
-        <f>IF(A330="","",IF(D330=0,"",MAXIFS(Sales!C:C,Sales!D:D,A330)))</f>
+        <f>IF(A330="","",IF(D330=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A330)))</f>
         <v/>
       </c>
       <c r="G330">
@@ -27078,7 +27078,7 @@
         <v/>
       </c>
       <c r="F331" s="3">
-        <f>IF(A331="","",IF(D331=0,"",MAXIFS(Sales!C:C,Sales!D:D,A331)))</f>
+        <f>IF(A331="","",IF(D331=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A331)))</f>
         <v/>
       </c>
       <c r="G331">
@@ -27112,7 +27112,7 @@
         <v/>
       </c>
       <c r="F332" s="3">
-        <f>IF(A332="","",IF(D332=0,"",MAXIFS(Sales!C:C,Sales!D:D,A332)))</f>
+        <f>IF(A332="","",IF(D332=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A332)))</f>
         <v/>
       </c>
       <c r="G332">
@@ -27146,7 +27146,7 @@
         <v/>
       </c>
       <c r="F333" s="3">
-        <f>IF(A333="","",IF(D333=0,"",MAXIFS(Sales!C:C,Sales!D:D,A333)))</f>
+        <f>IF(A333="","",IF(D333=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A333)))</f>
         <v/>
       </c>
       <c r="G333">
@@ -27180,7 +27180,7 @@
         <v/>
       </c>
       <c r="F334" s="3">
-        <f>IF(A334="","",IF(D334=0,"",MAXIFS(Sales!C:C,Sales!D:D,A334)))</f>
+        <f>IF(A334="","",IF(D334=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A334)))</f>
         <v/>
       </c>
       <c r="G334">
@@ -27214,7 +27214,7 @@
         <v/>
       </c>
       <c r="F335" s="3">
-        <f>IF(A335="","",IF(D335=0,"",MAXIFS(Sales!C:C,Sales!D:D,A335)))</f>
+        <f>IF(A335="","",IF(D335=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A335)))</f>
         <v/>
       </c>
       <c r="G335">
@@ -27248,7 +27248,7 @@
         <v/>
       </c>
       <c r="F336" s="3">
-        <f>IF(A336="","",IF(D336=0,"",MAXIFS(Sales!C:C,Sales!D:D,A336)))</f>
+        <f>IF(A336="","",IF(D336=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A336)))</f>
         <v/>
       </c>
       <c r="G336">
@@ -27282,7 +27282,7 @@
         <v/>
       </c>
       <c r="F337" s="3">
-        <f>IF(A337="","",IF(D337=0,"",MAXIFS(Sales!C:C,Sales!D:D,A337)))</f>
+        <f>IF(A337="","",IF(D337=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A337)))</f>
         <v/>
       </c>
       <c r="G337">
@@ -27316,7 +27316,7 @@
         <v/>
       </c>
       <c r="F338" s="3">
-        <f>IF(A338="","",IF(D338=0,"",MAXIFS(Sales!C:C,Sales!D:D,A338)))</f>
+        <f>IF(A338="","",IF(D338=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A338)))</f>
         <v/>
       </c>
       <c r="G338">
@@ -27350,7 +27350,7 @@
         <v/>
       </c>
       <c r="F339" s="3">
-        <f>IF(A339="","",IF(D339=0,"",MAXIFS(Sales!C:C,Sales!D:D,A339)))</f>
+        <f>IF(A339="","",IF(D339=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A339)))</f>
         <v/>
       </c>
       <c r="G339">
@@ -27384,7 +27384,7 @@
         <v/>
       </c>
       <c r="F340" s="3">
-        <f>IF(A340="","",IF(D340=0,"",MAXIFS(Sales!C:C,Sales!D:D,A340)))</f>
+        <f>IF(A340="","",IF(D340=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A340)))</f>
         <v/>
       </c>
       <c r="G340">
@@ -27418,7 +27418,7 @@
         <v/>
       </c>
       <c r="F341" s="3">
-        <f>IF(A341="","",IF(D341=0,"",MAXIFS(Sales!C:C,Sales!D:D,A341)))</f>
+        <f>IF(A341="","",IF(D341=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A341)))</f>
         <v/>
       </c>
       <c r="G341">
@@ -27452,7 +27452,7 @@
         <v/>
       </c>
       <c r="F342" s="3">
-        <f>IF(A342="","",IF(D342=0,"",MAXIFS(Sales!C:C,Sales!D:D,A342)))</f>
+        <f>IF(A342="","",IF(D342=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A342)))</f>
         <v/>
       </c>
       <c r="G342">
@@ -27486,7 +27486,7 @@
         <v/>
       </c>
       <c r="F343" s="3">
-        <f>IF(A343="","",IF(D343=0,"",MAXIFS(Sales!C:C,Sales!D:D,A343)))</f>
+        <f>IF(A343="","",IF(D343=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A343)))</f>
         <v/>
       </c>
       <c r="G343">
@@ -27520,7 +27520,7 @@
         <v/>
       </c>
       <c r="F344" s="3">
-        <f>IF(A344="","",IF(D344=0,"",MAXIFS(Sales!C:C,Sales!D:D,A344)))</f>
+        <f>IF(A344="","",IF(D344=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A344)))</f>
         <v/>
       </c>
       <c r="G344">
@@ -27554,7 +27554,7 @@
         <v/>
       </c>
       <c r="F345" s="3">
-        <f>IF(A345="","",IF(D345=0,"",MAXIFS(Sales!C:C,Sales!D:D,A345)))</f>
+        <f>IF(A345="","",IF(D345=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A345)))</f>
         <v/>
       </c>
       <c r="G345">
@@ -27588,7 +27588,7 @@
         <v/>
       </c>
       <c r="F346" s="3">
-        <f>IF(A346="","",IF(D346=0,"",MAXIFS(Sales!C:C,Sales!D:D,A346)))</f>
+        <f>IF(A346="","",IF(D346=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A346)))</f>
         <v/>
       </c>
       <c r="G346">
@@ -27622,7 +27622,7 @@
         <v/>
       </c>
       <c r="F347" s="3">
-        <f>IF(A347="","",IF(D347=0,"",MAXIFS(Sales!C:C,Sales!D:D,A347)))</f>
+        <f>IF(A347="","",IF(D347=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A347)))</f>
         <v/>
       </c>
       <c r="G347">
@@ -27656,7 +27656,7 @@
         <v/>
       </c>
       <c r="F348" s="3">
-        <f>IF(A348="","",IF(D348=0,"",MAXIFS(Sales!C:C,Sales!D:D,A348)))</f>
+        <f>IF(A348="","",IF(D348=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A348)))</f>
         <v/>
       </c>
       <c r="G348">
@@ -27690,7 +27690,7 @@
         <v/>
       </c>
       <c r="F349" s="3">
-        <f>IF(A349="","",IF(D349=0,"",MAXIFS(Sales!C:C,Sales!D:D,A349)))</f>
+        <f>IF(A349="","",IF(D349=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A349)))</f>
         <v/>
       </c>
       <c r="G349">
@@ -27724,7 +27724,7 @@
         <v/>
       </c>
       <c r="F350" s="3">
-        <f>IF(A350="","",IF(D350=0,"",MAXIFS(Sales!C:C,Sales!D:D,A350)))</f>
+        <f>IF(A350="","",IF(D350=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A350)))</f>
         <v/>
       </c>
       <c r="G350">
@@ -27758,7 +27758,7 @@
         <v/>
       </c>
       <c r="F351" s="3">
-        <f>IF(A351="","",IF(D351=0,"",MAXIFS(Sales!C:C,Sales!D:D,A351)))</f>
+        <f>IF(A351="","",IF(D351=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A351)))</f>
         <v/>
       </c>
       <c r="G351">
@@ -27792,7 +27792,7 @@
         <v/>
       </c>
       <c r="F352" s="3">
-        <f>IF(A352="","",IF(D352=0,"",MAXIFS(Sales!C:C,Sales!D:D,A352)))</f>
+        <f>IF(A352="","",IF(D352=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A352)))</f>
         <v/>
       </c>
       <c r="G352">
@@ -27826,7 +27826,7 @@
         <v/>
       </c>
       <c r="F353" s="3">
-        <f>IF(A353="","",IF(D353=0,"",MAXIFS(Sales!C:C,Sales!D:D,A353)))</f>
+        <f>IF(A353="","",IF(D353=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A353)))</f>
         <v/>
       </c>
       <c r="G353">
@@ -27860,7 +27860,7 @@
         <v/>
       </c>
       <c r="F354" s="3">
-        <f>IF(A354="","",IF(D354=0,"",MAXIFS(Sales!C:C,Sales!D:D,A354)))</f>
+        <f>IF(A354="","",IF(D354=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A354)))</f>
         <v/>
       </c>
       <c r="G354">
@@ -27894,7 +27894,7 @@
         <v/>
       </c>
       <c r="F355" s="3">
-        <f>IF(A355="","",IF(D355=0,"",MAXIFS(Sales!C:C,Sales!D:D,A355)))</f>
+        <f>IF(A355="","",IF(D355=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A355)))</f>
         <v/>
       </c>
       <c r="G355">
@@ -27928,7 +27928,7 @@
         <v/>
       </c>
       <c r="F356" s="3">
-        <f>IF(A356="","",IF(D356=0,"",MAXIFS(Sales!C:C,Sales!D:D,A356)))</f>
+        <f>IF(A356="","",IF(D356=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A356)))</f>
         <v/>
       </c>
       <c r="G356">
@@ -27962,7 +27962,7 @@
         <v/>
       </c>
       <c r="F357" s="3">
-        <f>IF(A357="","",IF(D357=0,"",MAXIFS(Sales!C:C,Sales!D:D,A357)))</f>
+        <f>IF(A357="","",IF(D357=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A357)))</f>
         <v/>
       </c>
       <c r="G357">
@@ -27996,7 +27996,7 @@
         <v/>
       </c>
       <c r="F358" s="3">
-        <f>IF(A358="","",IF(D358=0,"",MAXIFS(Sales!C:C,Sales!D:D,A358)))</f>
+        <f>IF(A358="","",IF(D358=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A358)))</f>
         <v/>
       </c>
       <c r="G358">
@@ -28030,7 +28030,7 @@
         <v/>
       </c>
       <c r="F359" s="3">
-        <f>IF(A359="","",IF(D359=0,"",MAXIFS(Sales!C:C,Sales!D:D,A359)))</f>
+        <f>IF(A359="","",IF(D359=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A359)))</f>
         <v/>
       </c>
       <c r="G359">
@@ -28064,7 +28064,7 @@
         <v/>
       </c>
       <c r="F360" s="3">
-        <f>IF(A360="","",IF(D360=0,"",MAXIFS(Sales!C:C,Sales!D:D,A360)))</f>
+        <f>IF(A360="","",IF(D360=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A360)))</f>
         <v/>
       </c>
       <c r="G360">
@@ -28098,7 +28098,7 @@
         <v/>
       </c>
       <c r="F361" s="3">
-        <f>IF(A361="","",IF(D361=0,"",MAXIFS(Sales!C:C,Sales!D:D,A361)))</f>
+        <f>IF(A361="","",IF(D361=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A361)))</f>
         <v/>
       </c>
       <c r="G361">
@@ -28132,7 +28132,7 @@
         <v/>
       </c>
       <c r="F362" s="3">
-        <f>IF(A362="","",IF(D362=0,"",MAXIFS(Sales!C:C,Sales!D:D,A362)))</f>
+        <f>IF(A362="","",IF(D362=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A362)))</f>
         <v/>
       </c>
       <c r="G362">
@@ -28166,7 +28166,7 @@
         <v/>
       </c>
       <c r="F363" s="3">
-        <f>IF(A363="","",IF(D363=0,"",MAXIFS(Sales!C:C,Sales!D:D,A363)))</f>
+        <f>IF(A363="","",IF(D363=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A363)))</f>
         <v/>
       </c>
       <c r="G363">
@@ -28200,7 +28200,7 @@
         <v/>
       </c>
       <c r="F364" s="3">
-        <f>IF(A364="","",IF(D364=0,"",MAXIFS(Sales!C:C,Sales!D:D,A364)))</f>
+        <f>IF(A364="","",IF(D364=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A364)))</f>
         <v/>
       </c>
       <c r="G364">
@@ -28234,7 +28234,7 @@
         <v/>
       </c>
       <c r="F365" s="3">
-        <f>IF(A365="","",IF(D365=0,"",MAXIFS(Sales!C:C,Sales!D:D,A365)))</f>
+        <f>IF(A365="","",IF(D365=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A365)))</f>
         <v/>
       </c>
       <c r="G365">
@@ -28268,7 +28268,7 @@
         <v/>
       </c>
       <c r="F366" s="3">
-        <f>IF(A366="","",IF(D366=0,"",MAXIFS(Sales!C:C,Sales!D:D,A366)))</f>
+        <f>IF(A366="","",IF(D366=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A366)))</f>
         <v/>
       </c>
       <c r="G366">
@@ -28302,7 +28302,7 @@
         <v/>
       </c>
       <c r="F367" s="3">
-        <f>IF(A367="","",IF(D367=0,"",MAXIFS(Sales!C:C,Sales!D:D,A367)))</f>
+        <f>IF(A367="","",IF(D367=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A367)))</f>
         <v/>
       </c>
       <c r="G367">
@@ -28336,7 +28336,7 @@
         <v/>
       </c>
       <c r="F368" s="3">
-        <f>IF(A368="","",IF(D368=0,"",MAXIFS(Sales!C:C,Sales!D:D,A368)))</f>
+        <f>IF(A368="","",IF(D368=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A368)))</f>
         <v/>
       </c>
       <c r="G368">
@@ -28370,7 +28370,7 @@
         <v/>
       </c>
       <c r="F369" s="3">
-        <f>IF(A369="","",IF(D369=0,"",MAXIFS(Sales!C:C,Sales!D:D,A369)))</f>
+        <f>IF(A369="","",IF(D369=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A369)))</f>
         <v/>
       </c>
       <c r="G369">
@@ -28404,7 +28404,7 @@
         <v/>
       </c>
       <c r="F370" s="3">
-        <f>IF(A370="","",IF(D370=0,"",MAXIFS(Sales!C:C,Sales!D:D,A370)))</f>
+        <f>IF(A370="","",IF(D370=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A370)))</f>
         <v/>
       </c>
       <c r="G370">
@@ -28438,7 +28438,7 @@
         <v/>
       </c>
       <c r="F371" s="3">
-        <f>IF(A371="","",IF(D371=0,"",MAXIFS(Sales!C:C,Sales!D:D,A371)))</f>
+        <f>IF(A371="","",IF(D371=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A371)))</f>
         <v/>
       </c>
       <c r="G371">
@@ -28472,7 +28472,7 @@
         <v/>
       </c>
       <c r="F372" s="3">
-        <f>IF(A372="","",IF(D372=0,"",MAXIFS(Sales!C:C,Sales!D:D,A372)))</f>
+        <f>IF(A372="","",IF(D372=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A372)))</f>
         <v/>
       </c>
       <c r="G372">
@@ -28506,7 +28506,7 @@
         <v/>
       </c>
       <c r="F373" s="3">
-        <f>IF(A373="","",IF(D373=0,"",MAXIFS(Sales!C:C,Sales!D:D,A373)))</f>
+        <f>IF(A373="","",IF(D373=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A373)))</f>
         <v/>
       </c>
       <c r="G373">
@@ -28540,7 +28540,7 @@
         <v/>
       </c>
       <c r="F374" s="3">
-        <f>IF(A374="","",IF(D374=0,"",MAXIFS(Sales!C:C,Sales!D:D,A374)))</f>
+        <f>IF(A374="","",IF(D374=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A374)))</f>
         <v/>
       </c>
       <c r="G374">
@@ -28574,7 +28574,7 @@
         <v/>
       </c>
       <c r="F375" s="3">
-        <f>IF(A375="","",IF(D375=0,"",MAXIFS(Sales!C:C,Sales!D:D,A375)))</f>
+        <f>IF(A375="","",IF(D375=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A375)))</f>
         <v/>
       </c>
       <c r="G375">
@@ -28608,7 +28608,7 @@
         <v/>
       </c>
       <c r="F376" s="3">
-        <f>IF(A376="","",IF(D376=0,"",MAXIFS(Sales!C:C,Sales!D:D,A376)))</f>
+        <f>IF(A376="","",IF(D376=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A376)))</f>
         <v/>
       </c>
       <c r="G376">
@@ -28642,7 +28642,7 @@
         <v/>
       </c>
       <c r="F377" s="3">
-        <f>IF(A377="","",IF(D377=0,"",MAXIFS(Sales!C:C,Sales!D:D,A377)))</f>
+        <f>IF(A377="","",IF(D377=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A377)))</f>
         <v/>
       </c>
       <c r="G377">
@@ -28676,7 +28676,7 @@
         <v/>
       </c>
       <c r="F378" s="3">
-        <f>IF(A378="","",IF(D378=0,"",MAXIFS(Sales!C:C,Sales!D:D,A378)))</f>
+        <f>IF(A378="","",IF(D378=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A378)))</f>
         <v/>
       </c>
       <c r="G378">
@@ -28710,7 +28710,7 @@
         <v/>
       </c>
       <c r="F379" s="3">
-        <f>IF(A379="","",IF(D379=0,"",MAXIFS(Sales!C:C,Sales!D:D,A379)))</f>
+        <f>IF(A379="","",IF(D379=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A379)))</f>
         <v/>
       </c>
       <c r="G379">
@@ -28744,7 +28744,7 @@
         <v/>
       </c>
       <c r="F380" s="3">
-        <f>IF(A380="","",IF(D380=0,"",MAXIFS(Sales!C:C,Sales!D:D,A380)))</f>
+        <f>IF(A380="","",IF(D380=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A380)))</f>
         <v/>
       </c>
       <c r="G380">
@@ -28778,7 +28778,7 @@
         <v/>
       </c>
       <c r="F381" s="3">
-        <f>IF(A381="","",IF(D381=0,"",MAXIFS(Sales!C:C,Sales!D:D,A381)))</f>
+        <f>IF(A381="","",IF(D381=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A381)))</f>
         <v/>
       </c>
       <c r="G381">
@@ -28812,7 +28812,7 @@
         <v/>
       </c>
       <c r="F382" s="3">
-        <f>IF(A382="","",IF(D382=0,"",MAXIFS(Sales!C:C,Sales!D:D,A382)))</f>
+        <f>IF(A382="","",IF(D382=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A382)))</f>
         <v/>
       </c>
       <c r="G382">
@@ -28846,7 +28846,7 @@
         <v/>
       </c>
       <c r="F383" s="3">
-        <f>IF(A383="","",IF(D383=0,"",MAXIFS(Sales!C:C,Sales!D:D,A383)))</f>
+        <f>IF(A383="","",IF(D383=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A383)))</f>
         <v/>
       </c>
       <c r="G383">
@@ -28880,7 +28880,7 @@
         <v/>
       </c>
       <c r="F384" s="3">
-        <f>IF(A384="","",IF(D384=0,"",MAXIFS(Sales!C:C,Sales!D:D,A384)))</f>
+        <f>IF(A384="","",IF(D384=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A384)))</f>
         <v/>
       </c>
       <c r="G384">
@@ -28914,7 +28914,7 @@
         <v/>
       </c>
       <c r="F385" s="3">
-        <f>IF(A385="","",IF(D385=0,"",MAXIFS(Sales!C:C,Sales!D:D,A385)))</f>
+        <f>IF(A385="","",IF(D385=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A385)))</f>
         <v/>
       </c>
       <c r="G385">
@@ -28948,7 +28948,7 @@
         <v/>
       </c>
       <c r="F386" s="3">
-        <f>IF(A386="","",IF(D386=0,"",MAXIFS(Sales!C:C,Sales!D:D,A386)))</f>
+        <f>IF(A386="","",IF(D386=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A386)))</f>
         <v/>
       </c>
       <c r="G386">
@@ -28982,7 +28982,7 @@
         <v/>
       </c>
       <c r="F387" s="3">
-        <f>IF(A387="","",IF(D387=0,"",MAXIFS(Sales!C:C,Sales!D:D,A387)))</f>
+        <f>IF(A387="","",IF(D387=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A387)))</f>
         <v/>
       </c>
       <c r="G387">
@@ -29016,7 +29016,7 @@
         <v/>
       </c>
       <c r="F388" s="3">
-        <f>IF(A388="","",IF(D388=0,"",MAXIFS(Sales!C:C,Sales!D:D,A388)))</f>
+        <f>IF(A388="","",IF(D388=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A388)))</f>
         <v/>
       </c>
       <c r="G388">
@@ -29050,7 +29050,7 @@
         <v/>
       </c>
       <c r="F389" s="3">
-        <f>IF(A389="","",IF(D389=0,"",MAXIFS(Sales!C:C,Sales!D:D,A389)))</f>
+        <f>IF(A389="","",IF(D389=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A389)))</f>
         <v/>
       </c>
       <c r="G389">
@@ -29084,7 +29084,7 @@
         <v/>
       </c>
       <c r="F390" s="3">
-        <f>IF(A390="","",IF(D390=0,"",MAXIFS(Sales!C:C,Sales!D:D,A390)))</f>
+        <f>IF(A390="","",IF(D390=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A390)))</f>
         <v/>
       </c>
       <c r="G390">
@@ -29118,7 +29118,7 @@
         <v/>
       </c>
       <c r="F391" s="3">
-        <f>IF(A391="","",IF(D391=0,"",MAXIFS(Sales!C:C,Sales!D:D,A391)))</f>
+        <f>IF(A391="","",IF(D391=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A391)))</f>
         <v/>
       </c>
       <c r="G391">
@@ -29152,7 +29152,7 @@
         <v/>
       </c>
       <c r="F392" s="3">
-        <f>IF(A392="","",IF(D392=0,"",MAXIFS(Sales!C:C,Sales!D:D,A392)))</f>
+        <f>IF(A392="","",IF(D392=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A392)))</f>
         <v/>
       </c>
       <c r="G392">
@@ -29186,7 +29186,7 @@
         <v/>
       </c>
       <c r="F393" s="3">
-        <f>IF(A393="","",IF(D393=0,"",MAXIFS(Sales!C:C,Sales!D:D,A393)))</f>
+        <f>IF(A393="","",IF(D393=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A393)))</f>
         <v/>
       </c>
       <c r="G393">
@@ -29220,7 +29220,7 @@
         <v/>
       </c>
       <c r="F394" s="3">
-        <f>IF(A394="","",IF(D394=0,"",MAXIFS(Sales!C:C,Sales!D:D,A394)))</f>
+        <f>IF(A394="","",IF(D394=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A394)))</f>
         <v/>
       </c>
       <c r="G394">
@@ -29254,7 +29254,7 @@
         <v/>
       </c>
       <c r="F395" s="3">
-        <f>IF(A395="","",IF(D395=0,"",MAXIFS(Sales!C:C,Sales!D:D,A395)))</f>
+        <f>IF(A395="","",IF(D395=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A395)))</f>
         <v/>
       </c>
       <c r="G395">
@@ -29288,7 +29288,7 @@
         <v/>
       </c>
       <c r="F396" s="3">
-        <f>IF(A396="","",IF(D396=0,"",MAXIFS(Sales!C:C,Sales!D:D,A396)))</f>
+        <f>IF(A396="","",IF(D396=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A396)))</f>
         <v/>
       </c>
       <c r="G396">
@@ -29322,7 +29322,7 @@
         <v/>
       </c>
       <c r="F397" s="3">
-        <f>IF(A397="","",IF(D397=0,"",MAXIFS(Sales!C:C,Sales!D:D,A397)))</f>
+        <f>IF(A397="","",IF(D397=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A397)))</f>
         <v/>
       </c>
       <c r="G397">
@@ -29356,7 +29356,7 @@
         <v/>
       </c>
       <c r="F398" s="3">
-        <f>IF(A398="","",IF(D398=0,"",MAXIFS(Sales!C:C,Sales!D:D,A398)))</f>
+        <f>IF(A398="","",IF(D398=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A398)))</f>
         <v/>
       </c>
       <c r="G398">
@@ -29390,7 +29390,7 @@
         <v/>
       </c>
       <c r="F399" s="3">
-        <f>IF(A399="","",IF(D399=0,"",MAXIFS(Sales!C:C,Sales!D:D,A399)))</f>
+        <f>IF(A399="","",IF(D399=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A399)))</f>
         <v/>
       </c>
       <c r="G399">
@@ -29424,7 +29424,7 @@
         <v/>
       </c>
       <c r="F400" s="3">
-        <f>IF(A400="","",IF(D400=0,"",MAXIFS(Sales!C:C,Sales!D:D,A400)))</f>
+        <f>IF(A400="","",IF(D400=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A400)))</f>
         <v/>
       </c>
       <c r="G400">
@@ -29458,7 +29458,7 @@
         <v/>
       </c>
       <c r="F401" s="3">
-        <f>IF(A401="","",IF(D401=0,"",MAXIFS(Sales!C:C,Sales!D:D,A401)))</f>
+        <f>IF(A401="","",IF(D401=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A401)))</f>
         <v/>
       </c>
       <c r="G401">
@@ -29492,7 +29492,7 @@
         <v/>
       </c>
       <c r="F402" s="3">
-        <f>IF(A402="","",IF(D402=0,"",MAXIFS(Sales!C:C,Sales!D:D,A402)))</f>
+        <f>IF(A402="","",IF(D402=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A402)))</f>
         <v/>
       </c>
       <c r="G402">
@@ -29526,7 +29526,7 @@
         <v/>
       </c>
       <c r="F403" s="3">
-        <f>IF(A403="","",IF(D403=0,"",MAXIFS(Sales!C:C,Sales!D:D,A403)))</f>
+        <f>IF(A403="","",IF(D403=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A403)))</f>
         <v/>
       </c>
       <c r="G403">
@@ -29560,7 +29560,7 @@
         <v/>
       </c>
       <c r="F404" s="3">
-        <f>IF(A404="","",IF(D404=0,"",MAXIFS(Sales!C:C,Sales!D:D,A404)))</f>
+        <f>IF(A404="","",IF(D404=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A404)))</f>
         <v/>
       </c>
       <c r="G404">
@@ -29594,7 +29594,7 @@
         <v/>
       </c>
       <c r="F405" s="3">
-        <f>IF(A405="","",IF(D405=0,"",MAXIFS(Sales!C:C,Sales!D:D,A405)))</f>
+        <f>IF(A405="","",IF(D405=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A405)))</f>
         <v/>
       </c>
       <c r="G405">
@@ -29628,7 +29628,7 @@
         <v/>
       </c>
       <c r="F406" s="3">
-        <f>IF(A406="","",IF(D406=0,"",MAXIFS(Sales!C:C,Sales!D:D,A406)))</f>
+        <f>IF(A406="","",IF(D406=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A406)))</f>
         <v/>
       </c>
       <c r="G406">
@@ -29662,7 +29662,7 @@
         <v/>
       </c>
       <c r="F407" s="3">
-        <f>IF(A407="","",IF(D407=0,"",MAXIFS(Sales!C:C,Sales!D:D,A407)))</f>
+        <f>IF(A407="","",IF(D407=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A407)))</f>
         <v/>
       </c>
       <c r="G407">
@@ -29696,7 +29696,7 @@
         <v/>
       </c>
       <c r="F408" s="3">
-        <f>IF(A408="","",IF(D408=0,"",MAXIFS(Sales!C:C,Sales!D:D,A408)))</f>
+        <f>IF(A408="","",IF(D408=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A408)))</f>
         <v/>
       </c>
       <c r="G408">
@@ -29730,7 +29730,7 @@
         <v/>
       </c>
       <c r="F409" s="3">
-        <f>IF(A409="","",IF(D409=0,"",MAXIFS(Sales!C:C,Sales!D:D,A409)))</f>
+        <f>IF(A409="","",IF(D409=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A409)))</f>
         <v/>
       </c>
       <c r="G409">
@@ -29764,7 +29764,7 @@
         <v/>
       </c>
       <c r="F410" s="3">
-        <f>IF(A410="","",IF(D410=0,"",MAXIFS(Sales!C:C,Sales!D:D,A410)))</f>
+        <f>IF(A410="","",IF(D410=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A410)))</f>
         <v/>
       </c>
       <c r="G410">
@@ -29798,7 +29798,7 @@
         <v/>
       </c>
       <c r="F411" s="3">
-        <f>IF(A411="","",IF(D411=0,"",MAXIFS(Sales!C:C,Sales!D:D,A411)))</f>
+        <f>IF(A411="","",IF(D411=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A411)))</f>
         <v/>
       </c>
       <c r="G411">
@@ -29832,7 +29832,7 @@
         <v/>
       </c>
       <c r="F412" s="3">
-        <f>IF(A412="","",IF(D412=0,"",MAXIFS(Sales!C:C,Sales!D:D,A412)))</f>
+        <f>IF(A412="","",IF(D412=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A412)))</f>
         <v/>
       </c>
       <c r="G412">
@@ -29866,7 +29866,7 @@
         <v/>
       </c>
       <c r="F413" s="3">
-        <f>IF(A413="","",IF(D413=0,"",MAXIFS(Sales!C:C,Sales!D:D,A413)))</f>
+        <f>IF(A413="","",IF(D413=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A413)))</f>
         <v/>
       </c>
       <c r="G413">
@@ -29900,7 +29900,7 @@
         <v/>
       </c>
       <c r="F414" s="3">
-        <f>IF(A414="","",IF(D414=0,"",MAXIFS(Sales!C:C,Sales!D:D,A414)))</f>
+        <f>IF(A414="","",IF(D414=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A414)))</f>
         <v/>
       </c>
       <c r="G414">
@@ -29934,7 +29934,7 @@
         <v/>
       </c>
       <c r="F415" s="3">
-        <f>IF(A415="","",IF(D415=0,"",MAXIFS(Sales!C:C,Sales!D:D,A415)))</f>
+        <f>IF(A415="","",IF(D415=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A415)))</f>
         <v/>
       </c>
       <c r="G415">
@@ -29968,7 +29968,7 @@
         <v/>
       </c>
       <c r="F416" s="3">
-        <f>IF(A416="","",IF(D416=0,"",MAXIFS(Sales!C:C,Sales!D:D,A416)))</f>
+        <f>IF(A416="","",IF(D416=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A416)))</f>
         <v/>
       </c>
       <c r="G416">
@@ -30002,7 +30002,7 @@
         <v/>
       </c>
       <c r="F417" s="3">
-        <f>IF(A417="","",IF(D417=0,"",MAXIFS(Sales!C:C,Sales!D:D,A417)))</f>
+        <f>IF(A417="","",IF(D417=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A417)))</f>
         <v/>
       </c>
       <c r="G417">
@@ -30036,7 +30036,7 @@
         <v/>
       </c>
       <c r="F418" s="3">
-        <f>IF(A418="","",IF(D418=0,"",MAXIFS(Sales!C:C,Sales!D:D,A418)))</f>
+        <f>IF(A418="","",IF(D418=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A418)))</f>
         <v/>
       </c>
       <c r="G418">
@@ -30070,7 +30070,7 @@
         <v/>
       </c>
       <c r="F419" s="3">
-        <f>IF(A419="","",IF(D419=0,"",MAXIFS(Sales!C:C,Sales!D:D,A419)))</f>
+        <f>IF(A419="","",IF(D419=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A419)))</f>
         <v/>
       </c>
       <c r="G419">
@@ -30104,7 +30104,7 @@
         <v/>
       </c>
       <c r="F420" s="3">
-        <f>IF(A420="","",IF(D420=0,"",MAXIFS(Sales!C:C,Sales!D:D,A420)))</f>
+        <f>IF(A420="","",IF(D420=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A420)))</f>
         <v/>
       </c>
       <c r="G420">
@@ -30138,7 +30138,7 @@
         <v/>
       </c>
       <c r="F421" s="3">
-        <f>IF(A421="","",IF(D421=0,"",MAXIFS(Sales!C:C,Sales!D:D,A421)))</f>
+        <f>IF(A421="","",IF(D421=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A421)))</f>
         <v/>
       </c>
       <c r="G421">
@@ -30172,7 +30172,7 @@
         <v/>
       </c>
       <c r="F422" s="3">
-        <f>IF(A422="","",IF(D422=0,"",MAXIFS(Sales!C:C,Sales!D:D,A422)))</f>
+        <f>IF(A422="","",IF(D422=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A422)))</f>
         <v/>
       </c>
       <c r="G422">
@@ -30206,7 +30206,7 @@
         <v/>
       </c>
       <c r="F423" s="3">
-        <f>IF(A423="","",IF(D423=0,"",MAXIFS(Sales!C:C,Sales!D:D,A423)))</f>
+        <f>IF(A423="","",IF(D423=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A423)))</f>
         <v/>
       </c>
       <c r="G423">
@@ -30240,7 +30240,7 @@
         <v/>
       </c>
       <c r="F424" s="3">
-        <f>IF(A424="","",IF(D424=0,"",MAXIFS(Sales!C:C,Sales!D:D,A424)))</f>
+        <f>IF(A424="","",IF(D424=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A424)))</f>
         <v/>
       </c>
       <c r="G424">
@@ -30274,7 +30274,7 @@
         <v/>
       </c>
       <c r="F425" s="3">
-        <f>IF(A425="","",IF(D425=0,"",MAXIFS(Sales!C:C,Sales!D:D,A425)))</f>
+        <f>IF(A425="","",IF(D425=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A425)))</f>
         <v/>
       </c>
       <c r="G425">
@@ -30308,7 +30308,7 @@
         <v/>
       </c>
       <c r="F426" s="3">
-        <f>IF(A426="","",IF(D426=0,"",MAXIFS(Sales!C:C,Sales!D:D,A426)))</f>
+        <f>IF(A426="","",IF(D426=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A426)))</f>
         <v/>
       </c>
       <c r="G426">
@@ -30342,7 +30342,7 @@
         <v/>
       </c>
       <c r="F427" s="3">
-        <f>IF(A427="","",IF(D427=0,"",MAXIFS(Sales!C:C,Sales!D:D,A427)))</f>
+        <f>IF(A427="","",IF(D427=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A427)))</f>
         <v/>
       </c>
       <c r="G427">
@@ -30376,7 +30376,7 @@
         <v/>
       </c>
       <c r="F428" s="3">
-        <f>IF(A428="","",IF(D428=0,"",MAXIFS(Sales!C:C,Sales!D:D,A428)))</f>
+        <f>IF(A428="","",IF(D428=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A428)))</f>
         <v/>
       </c>
       <c r="G428">
@@ -30410,7 +30410,7 @@
         <v/>
       </c>
       <c r="F429" s="3">
-        <f>IF(A429="","",IF(D429=0,"",MAXIFS(Sales!C:C,Sales!D:D,A429)))</f>
+        <f>IF(A429="","",IF(D429=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A429)))</f>
         <v/>
       </c>
       <c r="G429">
@@ -30444,7 +30444,7 @@
         <v/>
       </c>
       <c r="F430" s="3">
-        <f>IF(A430="","",IF(D430=0,"",MAXIFS(Sales!C:C,Sales!D:D,A430)))</f>
+        <f>IF(A430="","",IF(D430=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A430)))</f>
         <v/>
       </c>
       <c r="G430">
@@ -30478,7 +30478,7 @@
         <v/>
       </c>
       <c r="F431" s="3">
-        <f>IF(A431="","",IF(D431=0,"",MAXIFS(Sales!C:C,Sales!D:D,A431)))</f>
+        <f>IF(A431="","",IF(D431=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A431)))</f>
         <v/>
       </c>
       <c r="G431">
@@ -30512,7 +30512,7 @@
         <v/>
       </c>
       <c r="F432" s="3">
-        <f>IF(A432="","",IF(D432=0,"",MAXIFS(Sales!C:C,Sales!D:D,A432)))</f>
+        <f>IF(A432="","",IF(D432=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A432)))</f>
         <v/>
       </c>
       <c r="G432">
@@ -30546,7 +30546,7 @@
         <v/>
       </c>
       <c r="F433" s="3">
-        <f>IF(A433="","",IF(D433=0,"",MAXIFS(Sales!C:C,Sales!D:D,A433)))</f>
+        <f>IF(A433="","",IF(D433=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A433)))</f>
         <v/>
       </c>
       <c r="G433">
@@ -30580,7 +30580,7 @@
         <v/>
       </c>
       <c r="F434" s="3">
-        <f>IF(A434="","",IF(D434=0,"",MAXIFS(Sales!C:C,Sales!D:D,A434)))</f>
+        <f>IF(A434="","",IF(D434=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A434)))</f>
         <v/>
       </c>
       <c r="G434">
@@ -30614,7 +30614,7 @@
         <v/>
       </c>
       <c r="F435" s="3">
-        <f>IF(A435="","",IF(D435=0,"",MAXIFS(Sales!C:C,Sales!D:D,A435)))</f>
+        <f>IF(A435="","",IF(D435=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A435)))</f>
         <v/>
       </c>
       <c r="G435">
@@ -30648,7 +30648,7 @@
         <v/>
       </c>
       <c r="F436" s="3">
-        <f>IF(A436="","",IF(D436=0,"",MAXIFS(Sales!C:C,Sales!D:D,A436)))</f>
+        <f>IF(A436="","",IF(D436=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A436)))</f>
         <v/>
       </c>
       <c r="G436">
@@ -30682,7 +30682,7 @@
         <v/>
       </c>
       <c r="F437" s="3">
-        <f>IF(A437="","",IF(D437=0,"",MAXIFS(Sales!C:C,Sales!D:D,A437)))</f>
+        <f>IF(A437="","",IF(D437=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A437)))</f>
         <v/>
       </c>
       <c r="G437">
@@ -30716,7 +30716,7 @@
         <v/>
       </c>
       <c r="F438" s="3">
-        <f>IF(A438="","",IF(D438=0,"",MAXIFS(Sales!C:C,Sales!D:D,A438)))</f>
+        <f>IF(A438="","",IF(D438=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A438)))</f>
         <v/>
       </c>
       <c r="G438">
@@ -30750,7 +30750,7 @@
         <v/>
       </c>
       <c r="F439" s="3">
-        <f>IF(A439="","",IF(D439=0,"",MAXIFS(Sales!C:C,Sales!D:D,A439)))</f>
+        <f>IF(A439="","",IF(D439=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A439)))</f>
         <v/>
       </c>
       <c r="G439">
@@ -30784,7 +30784,7 @@
         <v/>
       </c>
       <c r="F440" s="3">
-        <f>IF(A440="","",IF(D440=0,"",MAXIFS(Sales!C:C,Sales!D:D,A440)))</f>
+        <f>IF(A440="","",IF(D440=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A440)))</f>
         <v/>
       </c>
       <c r="G440">
@@ -30818,7 +30818,7 @@
         <v/>
       </c>
       <c r="F441" s="3">
-        <f>IF(A441="","",IF(D441=0,"",MAXIFS(Sales!C:C,Sales!D:D,A441)))</f>
+        <f>IF(A441="","",IF(D441=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A441)))</f>
         <v/>
       </c>
       <c r="G441">
@@ -30852,7 +30852,7 @@
         <v/>
       </c>
       <c r="F442" s="3">
-        <f>IF(A442="","",IF(D442=0,"",MAXIFS(Sales!C:C,Sales!D:D,A442)))</f>
+        <f>IF(A442="","",IF(D442=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A442)))</f>
         <v/>
       </c>
       <c r="G442">
@@ -30886,7 +30886,7 @@
         <v/>
       </c>
       <c r="F443" s="3">
-        <f>IF(A443="","",IF(D443=0,"",MAXIFS(Sales!C:C,Sales!D:D,A443)))</f>
+        <f>IF(A443="","",IF(D443=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A443)))</f>
         <v/>
       </c>
       <c r="G443">
@@ -30920,7 +30920,7 @@
         <v/>
       </c>
       <c r="F444" s="3">
-        <f>IF(A444="","",IF(D444=0,"",MAXIFS(Sales!C:C,Sales!D:D,A444)))</f>
+        <f>IF(A444="","",IF(D444=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A444)))</f>
         <v/>
       </c>
       <c r="G444">
@@ -30954,7 +30954,7 @@
         <v/>
       </c>
       <c r="F445" s="3">
-        <f>IF(A445="","",IF(D445=0,"",MAXIFS(Sales!C:C,Sales!D:D,A445)))</f>
+        <f>IF(A445="","",IF(D445=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A445)))</f>
         <v/>
       </c>
       <c r="G445">
@@ -30988,7 +30988,7 @@
         <v/>
       </c>
       <c r="F446" s="3">
-        <f>IF(A446="","",IF(D446=0,"",MAXIFS(Sales!C:C,Sales!D:D,A446)))</f>
+        <f>IF(A446="","",IF(D446=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A446)))</f>
         <v/>
       </c>
       <c r="G446">
@@ -31022,7 +31022,7 @@
         <v/>
       </c>
       <c r="F447" s="3">
-        <f>IF(A447="","",IF(D447=0,"",MAXIFS(Sales!C:C,Sales!D:D,A447)))</f>
+        <f>IF(A447="","",IF(D447=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A447)))</f>
         <v/>
       </c>
       <c r="G447">
@@ -31056,7 +31056,7 @@
         <v/>
       </c>
       <c r="F448" s="3">
-        <f>IF(A448="","",IF(D448=0,"",MAXIFS(Sales!C:C,Sales!D:D,A448)))</f>
+        <f>IF(A448="","",IF(D448=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A448)))</f>
         <v/>
       </c>
       <c r="G448">
@@ -31090,7 +31090,7 @@
         <v/>
       </c>
       <c r="F449" s="3">
-        <f>IF(A449="","",IF(D449=0,"",MAXIFS(Sales!C:C,Sales!D:D,A449)))</f>
+        <f>IF(A449="","",IF(D449=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A449)))</f>
         <v/>
       </c>
       <c r="G449">
@@ -31124,7 +31124,7 @@
         <v/>
       </c>
       <c r="F450" s="3">
-        <f>IF(A450="","",IF(D450=0,"",MAXIFS(Sales!C:C,Sales!D:D,A450)))</f>
+        <f>IF(A450="","",IF(D450=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A450)))</f>
         <v/>
       </c>
       <c r="G450">
@@ -31158,7 +31158,7 @@
         <v/>
       </c>
       <c r="F451" s="3">
-        <f>IF(A451="","",IF(D451=0,"",MAXIFS(Sales!C:C,Sales!D:D,A451)))</f>
+        <f>IF(A451="","",IF(D451=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A451)))</f>
         <v/>
       </c>
       <c r="G451">
@@ -31192,7 +31192,7 @@
         <v/>
       </c>
       <c r="F452" s="3">
-        <f>IF(A452="","",IF(D452=0,"",MAXIFS(Sales!C:C,Sales!D:D,A452)))</f>
+        <f>IF(A452="","",IF(D452=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A452)))</f>
         <v/>
       </c>
       <c r="G452">
@@ -31226,7 +31226,7 @@
         <v/>
       </c>
       <c r="F453" s="3">
-        <f>IF(A453="","",IF(D453=0,"",MAXIFS(Sales!C:C,Sales!D:D,A453)))</f>
+        <f>IF(A453="","",IF(D453=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A453)))</f>
         <v/>
       </c>
       <c r="G453">
@@ -31260,7 +31260,7 @@
         <v/>
       </c>
       <c r="F454" s="3">
-        <f>IF(A454="","",IF(D454=0,"",MAXIFS(Sales!C:C,Sales!D:D,A454)))</f>
+        <f>IF(A454="","",IF(D454=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A454)))</f>
         <v/>
       </c>
       <c r="G454">
@@ -31294,7 +31294,7 @@
         <v/>
       </c>
       <c r="F455" s="3">
-        <f>IF(A455="","",IF(D455=0,"",MAXIFS(Sales!C:C,Sales!D:D,A455)))</f>
+        <f>IF(A455="","",IF(D455=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A455)))</f>
         <v/>
       </c>
       <c r="G455">
@@ -31328,7 +31328,7 @@
         <v/>
       </c>
       <c r="F456" s="3">
-        <f>IF(A456="","",IF(D456=0,"",MAXIFS(Sales!C:C,Sales!D:D,A456)))</f>
+        <f>IF(A456="","",IF(D456=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A456)))</f>
         <v/>
       </c>
       <c r="G456">
@@ -31362,7 +31362,7 @@
         <v/>
       </c>
       <c r="F457" s="3">
-        <f>IF(A457="","",IF(D457=0,"",MAXIFS(Sales!C:C,Sales!D:D,A457)))</f>
+        <f>IF(A457="","",IF(D457=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A457)))</f>
         <v/>
       </c>
       <c r="G457">
@@ -31396,7 +31396,7 @@
         <v/>
       </c>
       <c r="F458" s="3">
-        <f>IF(A458="","",IF(D458=0,"",MAXIFS(Sales!C:C,Sales!D:D,A458)))</f>
+        <f>IF(A458="","",IF(D458=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A458)))</f>
         <v/>
       </c>
       <c r="G458">
@@ -31430,7 +31430,7 @@
         <v/>
       </c>
       <c r="F459" s="3">
-        <f>IF(A459="","",IF(D459=0,"",MAXIFS(Sales!C:C,Sales!D:D,A459)))</f>
+        <f>IF(A459="","",IF(D459=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A459)))</f>
         <v/>
       </c>
       <c r="G459">
@@ -31464,7 +31464,7 @@
         <v/>
       </c>
       <c r="F460" s="3">
-        <f>IF(A460="","",IF(D460=0,"",MAXIFS(Sales!C:C,Sales!D:D,A460)))</f>
+        <f>IF(A460="","",IF(D460=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A460)))</f>
         <v/>
       </c>
       <c r="G460">
@@ -31498,7 +31498,7 @@
         <v/>
       </c>
       <c r="F461" s="3">
-        <f>IF(A461="","",IF(D461=0,"",MAXIFS(Sales!C:C,Sales!D:D,A461)))</f>
+        <f>IF(A461="","",IF(D461=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A461)))</f>
         <v/>
       </c>
       <c r="G461">
@@ -31532,7 +31532,7 @@
         <v/>
       </c>
       <c r="F462" s="3">
-        <f>IF(A462="","",IF(D462=0,"",MAXIFS(Sales!C:C,Sales!D:D,A462)))</f>
+        <f>IF(A462="","",IF(D462=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A462)))</f>
         <v/>
       </c>
       <c r="G462">
@@ -31566,7 +31566,7 @@
         <v/>
       </c>
       <c r="F463" s="3">
-        <f>IF(A463="","",IF(D463=0,"",MAXIFS(Sales!C:C,Sales!D:D,A463)))</f>
+        <f>IF(A463="","",IF(D463=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A463)))</f>
         <v/>
       </c>
       <c r="G463">
@@ -31600,7 +31600,7 @@
         <v/>
       </c>
       <c r="F464" s="3">
-        <f>IF(A464="","",IF(D464=0,"",MAXIFS(Sales!C:C,Sales!D:D,A464)))</f>
+        <f>IF(A464="","",IF(D464=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A464)))</f>
         <v/>
       </c>
       <c r="G464">
@@ -31634,7 +31634,7 @@
         <v/>
       </c>
       <c r="F465" s="3">
-        <f>IF(A465="","",IF(D465=0,"",MAXIFS(Sales!C:C,Sales!D:D,A465)))</f>
+        <f>IF(A465="","",IF(D465=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A465)))</f>
         <v/>
       </c>
       <c r="G465">
@@ -31668,7 +31668,7 @@
         <v/>
       </c>
       <c r="F466" s="3">
-        <f>IF(A466="","",IF(D466=0,"",MAXIFS(Sales!C:C,Sales!D:D,A466)))</f>
+        <f>IF(A466="","",IF(D466=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A466)))</f>
         <v/>
       </c>
       <c r="G466">
@@ -31702,7 +31702,7 @@
         <v/>
       </c>
       <c r="F467" s="3">
-        <f>IF(A467="","",IF(D467=0,"",MAXIFS(Sales!C:C,Sales!D:D,A467)))</f>
+        <f>IF(A467="","",IF(D467=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A467)))</f>
         <v/>
       </c>
       <c r="G467">
@@ -31736,7 +31736,7 @@
         <v/>
       </c>
       <c r="F468" s="3">
-        <f>IF(A468="","",IF(D468=0,"",MAXIFS(Sales!C:C,Sales!D:D,A468)))</f>
+        <f>IF(A468="","",IF(D468=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A468)))</f>
         <v/>
       </c>
       <c r="G468">
@@ -31770,7 +31770,7 @@
         <v/>
       </c>
       <c r="F469" s="3">
-        <f>IF(A469="","",IF(D469=0,"",MAXIFS(Sales!C:C,Sales!D:D,A469)))</f>
+        <f>IF(A469="","",IF(D469=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A469)))</f>
         <v/>
       </c>
       <c r="G469">
@@ -31804,7 +31804,7 @@
         <v/>
       </c>
       <c r="F470" s="3">
-        <f>IF(A470="","",IF(D470=0,"",MAXIFS(Sales!C:C,Sales!D:D,A470)))</f>
+        <f>IF(A470="","",IF(D470=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A470)))</f>
         <v/>
       </c>
       <c r="G470">
@@ -31838,7 +31838,7 @@
         <v/>
       </c>
       <c r="F471" s="3">
-        <f>IF(A471="","",IF(D471=0,"",MAXIFS(Sales!C:C,Sales!D:D,A471)))</f>
+        <f>IF(A471="","",IF(D471=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A471)))</f>
         <v/>
       </c>
       <c r="G471">
@@ -31872,7 +31872,7 @@
         <v/>
       </c>
       <c r="F472" s="3">
-        <f>IF(A472="","",IF(D472=0,"",MAXIFS(Sales!C:C,Sales!D:D,A472)))</f>
+        <f>IF(A472="","",IF(D472=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A472)))</f>
         <v/>
       </c>
       <c r="G472">
@@ -31906,7 +31906,7 @@
         <v/>
       </c>
       <c r="F473" s="3">
-        <f>IF(A473="","",IF(D473=0,"",MAXIFS(Sales!C:C,Sales!D:D,A473)))</f>
+        <f>IF(A473="","",IF(D473=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A473)))</f>
         <v/>
       </c>
       <c r="G473">
@@ -31940,7 +31940,7 @@
         <v/>
       </c>
       <c r="F474" s="3">
-        <f>IF(A474="","",IF(D474=0,"",MAXIFS(Sales!C:C,Sales!D:D,A474)))</f>
+        <f>IF(A474="","",IF(D474=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A474)))</f>
         <v/>
       </c>
       <c r="G474">
@@ -31974,7 +31974,7 @@
         <v/>
       </c>
       <c r="F475" s="3">
-        <f>IF(A475="","",IF(D475=0,"",MAXIFS(Sales!C:C,Sales!D:D,A475)))</f>
+        <f>IF(A475="","",IF(D475=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A475)))</f>
         <v/>
       </c>
       <c r="G475">
@@ -32008,7 +32008,7 @@
         <v/>
       </c>
       <c r="F476" s="3">
-        <f>IF(A476="","",IF(D476=0,"",MAXIFS(Sales!C:C,Sales!D:D,A476)))</f>
+        <f>IF(A476="","",IF(D476=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A476)))</f>
         <v/>
       </c>
       <c r="G476">
@@ -32042,7 +32042,7 @@
         <v/>
       </c>
       <c r="F477" s="3">
-        <f>IF(A477="","",IF(D477=0,"",MAXIFS(Sales!C:C,Sales!D:D,A477)))</f>
+        <f>IF(A477="","",IF(D477=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A477)))</f>
         <v/>
       </c>
       <c r="G477">
@@ -32076,7 +32076,7 @@
         <v/>
       </c>
       <c r="F478" s="3">
-        <f>IF(A478="","",IF(D478=0,"",MAXIFS(Sales!C:C,Sales!D:D,A478)))</f>
+        <f>IF(A478="","",IF(D478=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A478)))</f>
         <v/>
       </c>
       <c r="G478">
@@ -32110,7 +32110,7 @@
         <v/>
       </c>
       <c r="F479" s="3">
-        <f>IF(A479="","",IF(D479=0,"",MAXIFS(Sales!C:C,Sales!D:D,A479)))</f>
+        <f>IF(A479="","",IF(D479=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A479)))</f>
         <v/>
       </c>
       <c r="G479">
@@ -32144,7 +32144,7 @@
         <v/>
       </c>
       <c r="F480" s="3">
-        <f>IF(A480="","",IF(D480=0,"",MAXIFS(Sales!C:C,Sales!D:D,A480)))</f>
+        <f>IF(A480="","",IF(D480=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A480)))</f>
         <v/>
       </c>
       <c r="G480">
@@ -32178,7 +32178,7 @@
         <v/>
       </c>
       <c r="F481" s="3">
-        <f>IF(A481="","",IF(D481=0,"",MAXIFS(Sales!C:C,Sales!D:D,A481)))</f>
+        <f>IF(A481="","",IF(D481=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A481)))</f>
         <v/>
       </c>
       <c r="G481">
@@ -32212,7 +32212,7 @@
         <v/>
       </c>
       <c r="F482" s="3">
-        <f>IF(A482="","",IF(D482=0,"",MAXIFS(Sales!C:C,Sales!D:D,A482)))</f>
+        <f>IF(A482="","",IF(D482=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A482)))</f>
         <v/>
       </c>
       <c r="G482">
@@ -32246,7 +32246,7 @@
         <v/>
       </c>
       <c r="F483" s="3">
-        <f>IF(A483="","",IF(D483=0,"",MAXIFS(Sales!C:C,Sales!D:D,A483)))</f>
+        <f>IF(A483="","",IF(D483=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A483)))</f>
         <v/>
       </c>
       <c r="G483">
@@ -32280,7 +32280,7 @@
         <v/>
       </c>
       <c r="F484" s="3">
-        <f>IF(A484="","",IF(D484=0,"",MAXIFS(Sales!C:C,Sales!D:D,A484)))</f>
+        <f>IF(A484="","",IF(D484=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A484)))</f>
         <v/>
       </c>
       <c r="G484">
@@ -32314,7 +32314,7 @@
         <v/>
       </c>
       <c r="F485" s="3">
-        <f>IF(A485="","",IF(D485=0,"",MAXIFS(Sales!C:C,Sales!D:D,A485)))</f>
+        <f>IF(A485="","",IF(D485=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A485)))</f>
         <v/>
       </c>
       <c r="G485">
@@ -32348,7 +32348,7 @@
         <v/>
       </c>
       <c r="F486" s="3">
-        <f>IF(A486="","",IF(D486=0,"",MAXIFS(Sales!C:C,Sales!D:D,A486)))</f>
+        <f>IF(A486="","",IF(D486=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A486)))</f>
         <v/>
       </c>
       <c r="G486">
@@ -32382,7 +32382,7 @@
         <v/>
       </c>
       <c r="F487" s="3">
-        <f>IF(A487="","",IF(D487=0,"",MAXIFS(Sales!C:C,Sales!D:D,A487)))</f>
+        <f>IF(A487="","",IF(D487=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A487)))</f>
         <v/>
       </c>
       <c r="G487">
@@ -32416,7 +32416,7 @@
         <v/>
       </c>
       <c r="F488" s="3">
-        <f>IF(A488="","",IF(D488=0,"",MAXIFS(Sales!C:C,Sales!D:D,A488)))</f>
+        <f>IF(A488="","",IF(D488=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A488)))</f>
         <v/>
       </c>
       <c r="G488">
@@ -32450,7 +32450,7 @@
         <v/>
       </c>
       <c r="F489" s="3">
-        <f>IF(A489="","",IF(D489=0,"",MAXIFS(Sales!C:C,Sales!D:D,A489)))</f>
+        <f>IF(A489="","",IF(D489=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A489)))</f>
         <v/>
       </c>
       <c r="G489">
@@ -32484,7 +32484,7 @@
         <v/>
       </c>
       <c r="F490" s="3">
-        <f>IF(A490="","",IF(D490=0,"",MAXIFS(Sales!C:C,Sales!D:D,A490)))</f>
+        <f>IF(A490="","",IF(D490=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A490)))</f>
         <v/>
       </c>
       <c r="G490">
@@ -32518,7 +32518,7 @@
         <v/>
       </c>
       <c r="F491" s="3">
-        <f>IF(A491="","",IF(D491=0,"",MAXIFS(Sales!C:C,Sales!D:D,A491)))</f>
+        <f>IF(A491="","",IF(D491=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A491)))</f>
         <v/>
       </c>
       <c r="G491">
@@ -32552,7 +32552,7 @@
         <v/>
       </c>
       <c r="F492" s="3">
-        <f>IF(A492="","",IF(D492=0,"",MAXIFS(Sales!C:C,Sales!D:D,A492)))</f>
+        <f>IF(A492="","",IF(D492=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A492)))</f>
         <v/>
       </c>
       <c r="G492">
@@ -32586,7 +32586,7 @@
         <v/>
       </c>
       <c r="F493" s="3">
-        <f>IF(A493="","",IF(D493=0,"",MAXIFS(Sales!C:C,Sales!D:D,A493)))</f>
+        <f>IF(A493="","",IF(D493=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A493)))</f>
         <v/>
       </c>
       <c r="G493">
@@ -32620,7 +32620,7 @@
         <v/>
       </c>
       <c r="F494" s="3">
-        <f>IF(A494="","",IF(D494=0,"",MAXIFS(Sales!C:C,Sales!D:D,A494)))</f>
+        <f>IF(A494="","",IF(D494=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A494)))</f>
         <v/>
       </c>
       <c r="G494">
@@ -32654,7 +32654,7 @@
         <v/>
       </c>
       <c r="F495" s="3">
-        <f>IF(A495="","",IF(D495=0,"",MAXIFS(Sales!C:C,Sales!D:D,A495)))</f>
+        <f>IF(A495="","",IF(D495=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A495)))</f>
         <v/>
       </c>
       <c r="G495">
@@ -32688,7 +32688,7 @@
         <v/>
       </c>
       <c r="F496" s="3">
-        <f>IF(A496="","",IF(D496=0,"",MAXIFS(Sales!C:C,Sales!D:D,A496)))</f>
+        <f>IF(A496="","",IF(D496=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A496)))</f>
         <v/>
       </c>
       <c r="G496">
@@ -32722,7 +32722,7 @@
         <v/>
       </c>
       <c r="F497" s="3">
-        <f>IF(A497="","",IF(D497=0,"",MAXIFS(Sales!C:C,Sales!D:D,A497)))</f>
+        <f>IF(A497="","",IF(D497=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A497)))</f>
         <v/>
       </c>
       <c r="G497">
@@ -32756,7 +32756,7 @@
         <v/>
       </c>
       <c r="F498" s="3">
-        <f>IF(A498="","",IF(D498=0,"",MAXIFS(Sales!C:C,Sales!D:D,A498)))</f>
+        <f>IF(A498="","",IF(D498=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A498)))</f>
         <v/>
       </c>
       <c r="G498">
@@ -32790,7 +32790,7 @@
         <v/>
       </c>
       <c r="F499" s="3">
-        <f>IF(A499="","",IF(D499=0,"",MAXIFS(Sales!C:C,Sales!D:D,A499)))</f>
+        <f>IF(A499="","",IF(D499=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A499)))</f>
         <v/>
       </c>
       <c r="G499">
@@ -32824,7 +32824,7 @@
         <v/>
       </c>
       <c r="F500" s="3">
-        <f>IF(A500="","",IF(D500=0,"",MAXIFS(Sales!C:C,Sales!D:D,A500)))</f>
+        <f>IF(A500="","",IF(D500=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A500)))</f>
         <v/>
       </c>
       <c r="G500">
@@ -32858,7 +32858,7 @@
         <v/>
       </c>
       <c r="F501" s="3">
-        <f>IF(A501="","",IF(D501=0,"",MAXIFS(Sales!C:C,Sales!D:D,A501)))</f>
+        <f>IF(A501="","",IF(D501=0,"",_xlfn.MAXIFS(Sales!C:C,Sales!D:D,A501)))</f>
         <v/>
       </c>
       <c r="G501">

</xml_diff>

<commit_message>
Catalogue redesign: MRP-first cards, instant multilingual search with voice, units (pcs/kg/L...), buying price and opening stock on add product
</commit_message>
<xml_diff>
--- a/data/Ayyappa_Pooja_Store_Data.xlsx
+++ b/data/Ayyappa_Pooja_Store_Data.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -571,6 +571,11 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -624,6 +629,31 @@
           <t>Image_Folder</t>
         </is>
       </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>MRP</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Description_English</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Image_URL</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1426,9 +1456,12 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pooja Items,Idols,Incense,Kerala Snacks,Kerala Sweets,Kerala Products"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"piece,pack,dozen,g,kg,ml,l"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>